<commit_message>
chore: update CBAC demo form definitions
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/cbac.xlsx
+++ b/config/demo/forms/app/cbac.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.16015625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="27.94" customWidth="1" style="12" min="1" max="1"/>
@@ -940,100 +940,100 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>page_1a</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>Part A: Risk Assessment (1 of 2)</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16.4" customHeight="1" s="13">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>select_one age_range</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>age_range</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>1. What is your age? (in complete years)</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="30" ht="31.3" customHeight="1" s="13">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>select_one smoke_frequency</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>smoke_frequency</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>2. Do you smoke or consume smokeless products such as gutka or khaini?</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="31" ht="31.3" customHeight="1" s="13">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>select_one alcohol_frequency</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>alcohol_frequency</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>3. Do you consume alcohol daily</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="32" ht="46.25" customHeight="1" s="13">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>page_1a</t>
         </is>
@@ -1041,140 +1041,139 @@
     </row>
     <row r="33" ht="31.3" customHeight="1" s="13"/>
     <row r="34" ht="31.3" customHeight="1" s="13">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>page_1b</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="16" t="inlineStr">
         <is>
           <t>Part A: Risk Assessment (2 of 2)</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="35" ht="46.25" customHeight="1" s="13">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>select_one waist_size</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>waist_size</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="16" t="inlineStr">
         <is>
           <t>4. Measurement of waist (in cm)</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="16" t="inlineStr">
         <is>
           <t>filter = ${gender}</t>
         </is>
       </c>
     </row>
     <row r="36" ht="61.15" customHeight="1" s="13">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>select_one physical_activities_frequency</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>physical_activities_frequency</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="16" t="inlineStr">
         <is>
           <t>5. Do you undertake any physical activities for minimum of 150 minutes in a week?</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16.4" customHeight="1" s="13">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>select_one family_medical_history</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>family_medical_history</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="16" t="inlineStr">
         <is>
           <t>6. Do you have a family history (any one of your parents or siblings) of high blood pressure, diabetes and heart disease?</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>page_1b</t>
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="16" t="inlineStr">
         <is>
           <t>total_score</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="16" t="inlineStr">
         <is>
           <t>${age_range} + ${smoke_frequency} + ${alcohol_frequency} + ${waist_size} + ${physical_activities_frequency} + ${family_medical_history}</t>
         </is>
       </c>
     </row>
     <row r="41" ht="31.3" customHeight="1" s="13">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="16" t="inlineStr">
         <is>
           <t>risk_category</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="16" t="inlineStr">
         <is>
           <t>if(${total_score} &gt; 4, 'High Risk', 'Low Risk')</t>
         </is>
@@ -1182,112 +1181,112 @@
     </row>
     <row r="42" ht="16.4" customHeight="1" s="13"/>
     <row r="43" ht="31.3" customHeight="1" s="13">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="16" t="inlineStr">
         <is>
           <t>page_score</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="16" t="inlineStr">
         <is>
           <t>Part A: Score Summary</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16.4" customHeight="1" s="13">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t>score_display</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="16" t="inlineStr">
         <is>
           <t>CBAC Total Score: ${total_score}</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16.4" customHeight="1" s="13">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="16" t="inlineStr">
         <is>
           <t>risk_display</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="16" t="inlineStr">
         <is>
           <t>Risk Category: ${risk_category}</t>
         </is>
       </c>
     </row>
     <row r="46" ht="16.4" customHeight="1" s="13">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="16" t="inlineStr">
         <is>
           <t>score_high_note</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="16" t="inlineStr">
         <is>
           <t>Score is greater than 4. This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" s="16" t="inlineStr">
         <is>
           <t>${total_score} &gt; 4</t>
         </is>
       </c>
     </row>
     <row r="47" ht="16.4" customHeight="1" s="13">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>score_low_note</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="16" t="inlineStr">
         <is>
           <t>Score is 4 or below. This person appears to be at low risk for NCDs at this time.</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="16" t="inlineStr">
         <is>
           <t>${total_score} &lt;= 4</t>
         </is>
       </c>
     </row>
     <row r="48" ht="16.4" customHeight="1" s="13">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>page_score</t>
         </is>
@@ -1295,85 +1294,85 @@
     </row>
     <row r="49" ht="16.4" customHeight="1" s="13"/>
     <row r="50" ht="31.3" customHeight="1" s="13">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="16" t="inlineStr">
         <is>
           <t>page_2a</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B1: Women and Men (1 of 6)</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="51" ht="31.3" customHeight="1" s="13">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="16" t="inlineStr">
         <is>
           <t>shortness_of_breath</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="16" t="inlineStr">
         <is>
           <t>7. Shortness of breath</t>
         </is>
       </c>
     </row>
     <row r="52" ht="16.4" customHeight="1" s="13">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="16" t="inlineStr">
         <is>
           <t>cough_more_than_2_weeks</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="16" t="inlineStr">
         <is>
           <t>8. Coughing more than 2 weeks</t>
         </is>
       </c>
     </row>
     <row r="53" ht="16.4" customHeight="1" s="13">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="16" t="inlineStr">
         <is>
           <t>blood_in_sputum</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="16" t="inlineStr">
         <is>
           <t>9. Blood in sputum</t>
         </is>
       </c>
     </row>
     <row r="54" ht="16.4" customHeight="1" s="13">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t>page_2a</t>
         </is>
@@ -1381,171 +1380,170 @@
     </row>
     <row r="55" ht="31.3" customHeight="1" s="13"/>
     <row r="56" ht="31.3" customHeight="1" s="13">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="16" t="inlineStr">
         <is>
           <t>page_2b</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B1: Women and Men (2 of 6)</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="57" ht="16.4" customHeight="1" s="13">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="16" t="inlineStr">
         <is>
           <t>fever_more_than_2_weeks</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="16" t="inlineStr">
         <is>
           <t>10. Fever for more than 2 weeks</t>
         </is>
       </c>
     </row>
     <row r="58" ht="31.3" customFormat="1" customHeight="1" s="15">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="16" t="inlineStr">
         <is>
           <t>loss_of_weight</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="16" t="inlineStr">
         <is>
           <t>11. Loss of weight</t>
         </is>
       </c>
     </row>
     <row r="59" ht="31.3" customHeight="1" s="13">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="16" t="inlineStr">
         <is>
           <t>night_sweats</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="16" t="inlineStr">
         <is>
           <t>12. Night Sweats</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16.4" customHeight="1" s="13">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="16" t="inlineStr">
         <is>
           <t>page_2b</t>
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="16" t="inlineStr">
         <is>
           <t>page_2c</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B1: Women and Men (3 of 6)</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="63" ht="31.3" customHeight="1" s="13">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="16" t="inlineStr">
         <is>
           <t>current_anti_tb_drug</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="16" t="inlineStr">
         <is>
           <t>13. Are you currently taking anti-TB drugs</t>
         </is>
       </c>
     </row>
     <row r="64" ht="16.4" customHeight="1" s="13">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="16" t="inlineStr">
         <is>
           <t>family_tb</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="16" t="inlineStr">
         <is>
           <t>14. Anyone in family currently suffering from TB</t>
         </is>
       </c>
     </row>
     <row r="65" ht="31.3" customHeight="1" s="13">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="16" t="inlineStr">
         <is>
           <t>history_of_tb</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="16" t="inlineStr">
         <is>
           <t>15. History of TB</t>
         </is>
       </c>
     </row>
     <row r="66" ht="31.3" customHeight="1" s="13">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="16" t="inlineStr">
         <is>
           <t>page_2c</t>
         </is>
@@ -1553,85 +1551,85 @@
     </row>
     <row r="67" ht="31.3" customHeight="1" s="13"/>
     <row r="68" ht="31.3" customHeight="1" s="13">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="16" t="inlineStr">
         <is>
           <t>page_2d</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B1: Women and Men (4 of 6)</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E68" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="69" ht="31.3" customHeight="1" s="13">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="16" t="inlineStr">
         <is>
           <t>history_of_fits</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="16" t="inlineStr">
         <is>
           <t>16. History of fits</t>
         </is>
       </c>
     </row>
     <row r="70" ht="31.3" customHeight="1" s="13">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="16" t="inlineStr">
         <is>
           <t>difficulty_opening_mouth</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="16" t="inlineStr">
         <is>
           <t>17. Difficulty in opening mouth</t>
         </is>
       </c>
     </row>
     <row r="71" ht="31.3" customHeight="1" s="13">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="16" t="inlineStr">
         <is>
           <t>mouth_ulcers_or_growth</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
         <is>
           <t>18. Ulcers/patch/growth in mouth that has not healed in two weeks</t>
         </is>
       </c>
     </row>
     <row r="72" ht="31.3" customHeight="1" s="13">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="16" t="inlineStr">
         <is>
           <t>page_2d</t>
         </is>
@@ -1639,137 +1637,136 @@
     </row>
     <row r="73" ht="31.3" customHeight="1" s="13"/>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="16" t="inlineStr">
         <is>
           <t>page_2e</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B1: Women and Men (5 of 6)</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="75" ht="16.4" customHeight="1" s="13">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="16" t="inlineStr">
         <is>
           <t>voice_change</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="16" t="inlineStr">
         <is>
           <t>19. Any change in the tone of your voice</t>
         </is>
       </c>
     </row>
     <row r="76" ht="16.4" customHeight="1" s="13">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="16" t="inlineStr">
         <is>
           <t>skin_patch_discoloration</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="16" t="inlineStr">
         <is>
           <t>20. Any patch or discoloration on skin</t>
         </is>
       </c>
     </row>
     <row r="77" ht="31.3" customHeight="1" s="13">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="16" t="inlineStr">
         <is>
           <t>difficulty_holding_objects</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="16" t="inlineStr">
         <is>
           <t>21. Difficulty in holding objects with fingers</t>
         </is>
       </c>
     </row>
     <row r="78" ht="16.4" customHeight="1" s="13">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="16" t="inlineStr">
         <is>
           <t>page_2e</t>
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="16" t="inlineStr">
         <is>
           <t>page_2f</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B1: Women and Men (6 of 6)</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="81" ht="61.15" customHeight="1" s="13">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="16" t="inlineStr">
         <is>
           <t>loss_of_sensation</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="16" t="inlineStr">
         <is>
           <t>22. Loss of sensation for cold/hot objects in palm or sole</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="16" t="inlineStr">
         <is>
           <t>page_2f</t>
         </is>
@@ -1777,110 +1774,110 @@
     </row>
     <row r="83" ht="16.4" customHeight="1" s="13"/>
     <row r="84" ht="16.4" customHeight="1" s="13">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="16" t="inlineStr">
         <is>
           <t>page_3a</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B2: Women only (1 of 3)</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E84" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H84" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="85" ht="61.15" customHeight="1" s="13">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="16" t="inlineStr">
         <is>
           <t>breast_lump</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="16" t="inlineStr">
         <is>
           <t>23. Lump in the breast</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H85" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="86" ht="46.25" customHeight="1" s="13">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="16" t="inlineStr">
         <is>
           <t>nipple_discharge</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="16" t="inlineStr">
         <is>
           <t>24. Blood stained discharge from the nipple</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H86" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16.4" customHeight="1" s="13">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="16" t="inlineStr">
         <is>
           <t>breast_shape_size_change</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="16" t="inlineStr">
         <is>
           <t>25. Change in shape and size of breast</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="H87" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16.4" customHeight="1" s="13">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="16" t="inlineStr">
         <is>
           <t>page_3a</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="H88" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
@@ -1888,514 +1885,546 @@
     </row>
     <row r="89" ht="16.4" customHeight="1" s="13"/>
     <row r="90" ht="16.4" customHeight="1" s="13">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="16" t="inlineStr">
         <is>
           <t>page_3b</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B2: Women only (2 of 3)</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="E90" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="H90" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="91" ht="16.4" customHeight="1" s="13">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="16" t="inlineStr">
         <is>
           <t>bleeding_between_periods</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="16" t="inlineStr">
         <is>
           <t>26. Bleeding between periods</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="H91" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="92" ht="16.4" customHeight="1" s="13">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="16" t="inlineStr">
         <is>
           <t>post_menopause_bleeding</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="16" t="inlineStr">
         <is>
           <t>27. Bleeding after menopause</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
+      <c r="H92" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16.4" customHeight="1" s="13">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="16" t="inlineStr">
         <is>
           <t>post_intercourse_bleeding</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="16" t="inlineStr">
         <is>
           <t>28. Bleeding after intercourse</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="H93" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16.4" customHeight="1" s="13">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="16" t="inlineStr">
         <is>
           <t>page_3b</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr">
+      <c r="H94" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
-    <row r="95"/>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="16" t="inlineStr">
         <is>
           <t>page_3c</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="16" t="inlineStr">
         <is>
           <t>Part B: Early Detection – B2: Women only (3 of 3)</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="E96" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr">
+      <c r="H96" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="16" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="16" t="inlineStr">
         <is>
           <t>foul_smelling_vaginal_discharge</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="16" t="inlineStr">
         <is>
           <t>29. Foul smelling vaginal discharge</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr">
+      <c r="H97" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B98" s="16" t="inlineStr">
         <is>
           <t>page_3c</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr">
+      <c r="H98" s="16" t="inlineStr">
         <is>
           <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
-    <row r="99"/>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>page_4</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Part C: Circle all that Apply</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>field-list</t>
+      <c r="A100" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B100" s="16" t="inlineStr">
+        <is>
+          <t>part_c_start_q</t>
+        </is>
+      </c>
+      <c r="F100" s="16" t="inlineStr">
+        <is>
+          <t>if(${gender} = 'male', 23, 30)</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>part_c_q2</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>if(${gender} = 'male', 24, 31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B102" s="16" t="inlineStr">
+        <is>
+          <t>page_4</t>
+        </is>
+      </c>
+      <c r="C102" s="16" t="inlineStr">
+        <is>
+          <t>Part C: Circle all that Apply</t>
+        </is>
+      </c>
+      <c r="E102" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="inlineStr">
+        <is>
           <t>select_multiple fuel_type</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B103" s="16" t="inlineStr">
         <is>
           <t>fuel_type_for_cooking</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Type of Fuel used for cooking</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>${part_c_start_q}. Type of Fuel used for cooking</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="inlineStr">
         <is>
           <t>select_multiple occupational_exposure</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B104" s="16" t="inlineStr">
         <is>
           <t>occupational_exposure</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Occupational exposure</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>${part_c_q2}. Occupational exposure</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B105" s="16" t="inlineStr">
         <is>
           <t>page_4</t>
         </is>
       </c>
     </row>
-    <row r="104"/>
-    <row r="105">
-      <c r="A105" t="inlineStr">
+    <row r="106"/>
+    <row r="107">
+      <c r="A107" s="16" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B107" s="16" t="inlineStr">
         <is>
           <t>group_summary</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C107" s="16" t="inlineStr">
         <is>
           <t>Assessment Summary</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E107" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B108" s="16" t="inlineStr">
         <is>
           <t>summary_high_risk</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C108" s="16" t="inlineStr">
         <is>
           <t>Score is greater than 4. This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr">
+      <c r="H108" s="16" t="inlineStr">
         <is>
           <t>${total_score} &gt; 4</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B109" s="16" t="inlineStr">
         <is>
           <t>summary_low_risk</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C109" s="16" t="inlineStr">
         <is>
           <t>Score is 4 or below. This person appears to be at low risk for NCDs at this time.</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
+      <c r="H109" s="16" t="inlineStr">
         <is>
           <t>${total_score} &lt;= 4</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B110" s="16" t="inlineStr">
         <is>
           <t>lbl_filled_by</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C110" s="16" t="inlineStr">
         <is>
           <t>**Filled by:**</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E110" s="16" t="inlineStr">
         <is>
           <t>w5</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F110" s="16" t="inlineStr">
         <is>
           <t>${reporter_name}</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B111" s="16" t="inlineStr">
         <is>
           <t>lbl_patient_val</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C111" s="16" t="inlineStr">
         <is>
           <t>**Patient:**</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E111" s="16" t="inlineStr">
         <is>
           <t>w5</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
+      <c r="F111" s="16" t="inlineStr">
         <is>
           <t>${patient_name}</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B112" s="16" t="inlineStr">
         <is>
           <t>lbl_gender_val</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C112" s="16" t="inlineStr">
         <is>
           <t>**Gender:**</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E112" s="16" t="inlineStr">
         <is>
           <t>w5</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F112" s="16" t="inlineStr">
         <is>
           <t>${gender}</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B113" s="16" t="inlineStr">
         <is>
           <t>lbl_state_val</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C113" s="16" t="inlineStr">
         <is>
           <t>**State:**</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E113" s="16" t="inlineStr">
         <is>
           <t>w5</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
+      <c r="F113" s="16" t="inlineStr">
         <is>
           <t>${state}</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B114" s="16" t="inlineStr">
         <is>
           <t>lbl_district_val</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C114" s="16" t="inlineStr">
         <is>
           <t>**District:**</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E114" s="16" t="inlineStr">
         <is>
           <t>w5</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F114" s="16" t="inlineStr">
         <is>
           <t>${district}</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B115" s="16" t="inlineStr">
         <is>
           <t>lbl_score_val</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C115" s="16" t="inlineStr">
         <is>
           <t>**CBAC Total Score:**</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
+      <c r="E115" s="16" t="inlineStr">
         <is>
           <t>w5</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
+      <c r="F115" s="16" t="inlineStr">
         <is>
           <t>${total_score}</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="16" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B116" s="16" t="inlineStr">
         <is>
           <t>lbl_risk_val</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C116" s="16" t="inlineStr">
         <is>
           <t>**Risk Category:**</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E116" s="16" t="inlineStr">
         <is>
           <t>w5</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
+      <c r="F116" s="16" t="inlineStr">
         <is>
           <t>${risk_category}</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="16" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B117" s="16" t="inlineStr">
         <is>
           <t>group_summary</t>
         </is>

</xml_diff>

<commit_message>
feat: update person-edit roles, add form timestamps to follow-up and assessment forms, and remove versioning from person-edit metadata
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/cbac.xlsx
+++ b/config/demo/forms/app/cbac.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I117"/>
+  <dimension ref="A1:I178"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.16015625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="27.94" customWidth="1" style="12" min="1" max="1"/>
@@ -562,6 +562,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="31.3" customHeight="1" s="13">
       <c r="A7" s="12" t="inlineStr">
         <is>
@@ -602,60 +603,65 @@
       </c>
     </row>
     <row r="9" ht="16.4" customHeight="1" s="13">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>inputs</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Patient &amp; Reporter Info</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>field-list</t>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>form_start_timestamp</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>once(if(${_id} != '', now(), ''))</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16.4" customHeight="1" s="13">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>source</t>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>form_sync_timestamp</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16.4" customHeight="1" s="13">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>source_id</t>
+          <t>inputs</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Patient &amp; Reporter Info</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16.4" customHeight="1" s="13">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>source</t>
         </is>
       </c>
     </row>
@@ -667,114 +673,84 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>source_id</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16.4" customHeight="1" s="13">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>user</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16.4" customHeight="1" s="13">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>name</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16.4" customHeight="1" s="13">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>reporter_name_note</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>Filled by: ${reporter_name}</t>
+          <t>phone</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16.4" customHeight="1" s="13">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>user</t>
         </is>
       </c>
     </row>
     <row r="18" ht="31.3" customHeight="1" s="13">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>_id</t>
+          <t>reporter_name_note</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Patient's Name</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Select the patient from your area</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>select-contact type-person role-patient</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Filled by: ${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16.4" customHeight="1" s="13">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>patient_id</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>Medic ID</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>hidden</t>
+          <t>contact</t>
         </is>
       </c>
     </row>
@@ -786,73 +762,88 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>_id</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Patient Name</t>
+          <t>Patient's Name</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Select the patient from your area</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>select-contact type-person role-patient</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16.4" customHeight="1" s="13">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>select_one gender</t>
+          <t>string</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>patient_id</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Medic ID</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>hidden</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16.4" customHeight="1" s="13">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>string</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>hidden</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16.4" customHeight="1" s="13">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>select_one states</t>
+          <t>select_one gender</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>minimal</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="G23" s="12" t="inlineStr">
@@ -864,161 +855,156 @@
     <row r="24" ht="31.3" customHeight="1" s="13">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>select_one districts</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>District</t>
-        </is>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="G24" s="12" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I24" s="12" t="inlineStr">
-        <is>
-          <t>filter = ${state}</t>
+          <t>contact</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16.4" customHeight="1" s="13">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one states</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>inputs</t>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="26" ht="61.15" customHeight="1" s="13">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one districts</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>instructions</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>A score above 4 indicates that the person may be at risk for these NCDs and needs to be prioritized for attending the weekly NCD day</t>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>filter = ${state}</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16.4" customHeight="1" s="13">
       <c r="A27" s="12" t="inlineStr">
         <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>total_question</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>if(${gender} = ‘male’, '22', '29')</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>page_1a</t>
-        </is>
-      </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>Part A: Risk Assessment (1 of 2)</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>if(${gender} = 'male', '0', '7')</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16.4" customHeight="1" s="13">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>select_one age_range</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>age_range</t>
+          <t>instructions</t>
         </is>
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>1. What is your age? (in complete years)</t>
-        </is>
-      </c>
-      <c r="G29" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Part A consists of 6 questions. Each question carries a score. A total score above 4 indicates high risk for NCDs — such a person should be prioritised for further examination at the weekly NCD clinic.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="31.3" customHeight="1" s="13">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>select_one smoke_frequency</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>smoke_frequency</t>
+          <t>page_1a</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>2. Do you smoke or consume smokeless products such as gutka or khaini?</t>
-        </is>
-      </c>
-      <c r="G30" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Part A: Risk Assessment (1 of 2)</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="31" ht="31.3" customHeight="1" s="13">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>select_one alcohol_frequency</t>
+          <t>select_one age_range</t>
         </is>
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>alcohol_frequency</t>
+          <t>age_range</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>3. Do you consume alcohol daily</t>
+          <t>1. What is your age? (in complete years)</t>
         </is>
       </c>
       <c r="G31" s="16" t="inlineStr">
@@ -1030,209 +1016,220 @@
     <row r="32" ht="46.25" customHeight="1" s="13">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one smoke_frequency</t>
         </is>
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>page_1a</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="31.3" customHeight="1" s="13"/>
+          <t>smoke_frequency</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>2. Do you smoke or consume smokeless products such as gutka or khaini?</t>
+        </is>
+      </c>
+      <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="31.3" customHeight="1" s="13">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>select_one alcohol_frequency</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>alcohol_frequency</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>3. Do you consume alcohol daily</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
     <row r="34" ht="31.3" customHeight="1" s="13">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>page_1b</t>
-        </is>
-      </c>
-      <c r="C34" s="16" t="inlineStr">
-        <is>
-          <t>Part A: Risk Assessment (2 of 2)</t>
-        </is>
-      </c>
-      <c r="E34" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="46.25" customHeight="1" s="13">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>select_one waist_size</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="inlineStr">
-        <is>
-          <t>waist_size</t>
-        </is>
-      </c>
-      <c r="C35" s="16" t="inlineStr">
-        <is>
-          <t>4. Measurement of waist (in cm)</t>
-        </is>
-      </c>
-      <c r="G35" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I35" s="16" t="inlineStr">
-        <is>
-          <t>filter = ${gender}</t>
-        </is>
-      </c>
-    </row>
+          <t>page_1a</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="46.25" customHeight="1" s="13"/>
     <row r="36" ht="61.15" customHeight="1" s="13">
       <c r="A36" s="16" t="inlineStr">
         <is>
-          <t>select_one physical_activities_frequency</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>physical_activities_frequency</t>
+          <t>page_1b</t>
         </is>
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>5. Do you undertake any physical activities for minimum of 150 minutes in a week?</t>
-        </is>
-      </c>
-      <c r="G36" s="16" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Part A: Risk Assessment (2 of 2)</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16.4" customHeight="1" s="13">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t>select_one family_medical_history</t>
+          <t>select_one waist_size</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>family_medical_history</t>
+          <t>waist_size</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>6. Do you have a family history (any one of your parents or siblings) of high blood pressure, diabetes and heart disease?</t>
+          <t>4. Measurement of waist (in cm)</t>
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>filter = ${gender}</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one physical_activities_frequency</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>page_1b</t>
+          <t>physical_activities_frequency</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>5. Do you undertake any physical activities for minimum of 150 minutes in a week?</t>
+        </is>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>select_one family_medical_history</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>family_medical_history</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>6. Do you have a family history (any one of your parents or siblings) of high blood pressure, diabetes and heart disease?</t>
+        </is>
+      </c>
+      <c r="G39" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>page_1b</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="31.3" customHeight="1" s="13"/>
+    <row r="42" ht="16.4" customHeight="1" s="13">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B42" s="16" t="inlineStr">
         <is>
           <t>total_score</t>
         </is>
       </c>
-      <c r="F40" s="16" t="inlineStr">
+      <c r="F42" s="16" t="inlineStr">
         <is>
           <t>${age_range} + ${smoke_frequency} + ${alcohol_frequency} + ${waist_size} + ${physical_activities_frequency} + ${family_medical_history}</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="31.3" customHeight="1" s="13">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B41" s="16" t="inlineStr">
-        <is>
-          <t>risk_category</t>
-        </is>
-      </c>
-      <c r="F41" s="16" t="inlineStr">
-        <is>
-          <t>if(${total_score} &gt; 4, 'High Risk', 'Low Risk')</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16.4" customHeight="1" s="13"/>
     <row r="43" ht="31.3" customHeight="1" s="13">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>page_score</t>
-        </is>
-      </c>
-      <c r="C43" s="16" t="inlineStr">
-        <is>
-          <t>Part A: Score Summary</t>
-        </is>
-      </c>
-      <c r="E43" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16.4" customHeight="1" s="13">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B44" s="16" t="inlineStr">
-        <is>
-          <t>score_display</t>
-        </is>
-      </c>
-      <c r="C44" s="16" t="inlineStr">
-        <is>
-          <t>CBAC Total Score: ${total_score}</t>
-        </is>
-      </c>
-    </row>
+          <t>risk_category</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>if(${total_score} &gt; 4, 'High Risk', 'Low Risk')</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16.4" customHeight="1" s="13"/>
     <row r="45" ht="16.4" customHeight="1" s="13">
       <c r="A45" s="16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>risk_display</t>
+          <t>page_score</t>
         </is>
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Risk Category: ${risk_category}</t>
+          <t>Part A: Score Summary</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -1244,17 +1241,12 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>score_high_note</t>
+          <t>score_display</t>
         </is>
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
-          <t>Score is greater than 4. This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
-        </is>
-      </c>
-      <c r="H46" s="16" t="inlineStr">
-        <is>
-          <t>${total_score} &gt; 4</t>
+          <t>CBAC Total Score: ${total_score}</t>
         </is>
       </c>
     </row>
@@ -1266,86 +1258,96 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>score_low_note</t>
+          <t>risk_display</t>
         </is>
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>Score is 4 or below. This person appears to be at low risk for NCDs at this time.</t>
-        </is>
-      </c>
-      <c r="H47" s="16" t="inlineStr">
-        <is>
-          <t>${total_score} &lt;= 4</t>
+          <t>Risk Category: ${risk_category}</t>
         </is>
       </c>
     </row>
     <row r="48" ht="16.4" customHeight="1" s="13">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>page_score</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="16.4" customHeight="1" s="13"/>
+          <t>score_high_note</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Score is greater than 4. This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
+        </is>
+      </c>
+      <c r="H48" s="16" t="inlineStr">
+        <is>
+          <t>${total_score} &gt; 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16.4" customHeight="1" s="13">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>score_low_note</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Score is 4 or below. This person appears to be at low risk for NCDs at this time.</t>
+        </is>
+      </c>
+      <c r="H49" s="16" t="inlineStr">
+        <is>
+          <t>${total_score} &lt;= 4</t>
+        </is>
+      </c>
+    </row>
     <row r="50" ht="31.3" customHeight="1" s="13">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>page_2a</t>
-        </is>
-      </c>
-      <c r="C50" s="16" t="inlineStr">
-        <is>
-          <t>Part B: Early Detection – B1: Women and Men (1 of 6)</t>
-        </is>
-      </c>
-      <c r="E50" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="31.3" customHeight="1" s="13">
-      <c r="A51" s="16" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B51" s="16" t="inlineStr">
-        <is>
-          <t>shortness_of_breath</t>
-        </is>
-      </c>
-      <c r="C51" s="16" t="inlineStr">
-        <is>
-          <t>7. Shortness of breath</t>
-        </is>
-      </c>
-    </row>
+          <t>page_score</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="31.3" customHeight="1" s="13"/>
     <row r="52" ht="16.4" customHeight="1" s="13">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>cough_more_than_2_weeks</t>
+          <t>page_3a</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
         <is>
-          <t>8. Coughing more than 2 weeks</t>
+          <t>Part B: Early Detection – Women only (1 of 3)</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H52" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -1357,81 +1359,121 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>blood_in_sputum</t>
+          <t>breast_lump</t>
         </is>
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>9. Blood in sputum</t>
+          <t>7. Lump in the breast</t>
+        </is>
+      </c>
+      <c r="G53" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H53" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="54" ht="16.4" customHeight="1" s="13">
       <c r="A54" s="16" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>page_2a</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="31.3" customHeight="1" s="13"/>
+          <t>nipple_discharge</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>8. Blood stained discharge from the nipple</t>
+        </is>
+      </c>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H54" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="31.3" customHeight="1" s="13">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>select_one yes_no</t>
+        </is>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>breast_shape_size_change</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>9. Change in shape and size of breast</t>
+        </is>
+      </c>
+      <c r="G55" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H55" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
     <row r="56" ht="31.3" customHeight="1" s="13">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>page_2b</t>
-        </is>
-      </c>
-      <c r="C56" s="16" t="inlineStr">
-        <is>
-          <t>Part B: Early Detection – B1: Women and Men (2 of 6)</t>
-        </is>
-      </c>
-      <c r="E56" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="16.4" customHeight="1" s="13">
-      <c r="A57" s="16" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B57" s="16" t="inlineStr">
-        <is>
-          <t>fever_more_than_2_weeks</t>
-        </is>
-      </c>
-      <c r="C57" s="16" t="inlineStr">
-        <is>
-          <t>10. Fever for more than 2 weeks</t>
-        </is>
-      </c>
-    </row>
+          <t>page_3a</t>
+        </is>
+      </c>
+      <c r="H56" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="16.4" customHeight="1" s="13"/>
     <row r="58" ht="31.3" customFormat="1" customHeight="1" s="15">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>loss_of_weight</t>
+          <t>page_3b</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
         <is>
-          <t>11. Loss of weight</t>
+          <t>Part B: Early Detection – Women only (2 of 3)</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H58" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -1443,80 +1485,121 @@
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>night_sweats</t>
+          <t>bleeding_between_periods</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>12. Night Sweats</t>
+          <t>10. Bleeding between periods</t>
+        </is>
+      </c>
+      <c r="G59" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H59" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16.4" customHeight="1" s="13">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>page_2b</t>
+          <t>post_menopause_bleeding</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>11. Bleeding after menopause</t>
+        </is>
+      </c>
+      <c r="G60" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H60" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>select_one yes_no</t>
+        </is>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>post_intercourse_bleeding</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>12. Bleeding after intercourse</t>
+        </is>
+      </c>
+      <c r="G61" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H61" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>page_2c</t>
-        </is>
-      </c>
-      <c r="C62" s="16" t="inlineStr">
-        <is>
-          <t>Part B: Early Detection – B1: Women and Men (3 of 6)</t>
-        </is>
-      </c>
-      <c r="E62" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="31.3" customHeight="1" s="13">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B63" s="16" t="inlineStr">
-        <is>
-          <t>current_anti_tb_drug</t>
-        </is>
-      </c>
-      <c r="C63" s="16" t="inlineStr">
-        <is>
-          <t>13. Are you currently taking anti-TB drugs</t>
-        </is>
-      </c>
-    </row>
+          <t>page_3b</t>
+        </is>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="31.3" customHeight="1" s="13"/>
     <row r="64" ht="16.4" customHeight="1" s="13">
       <c r="A64" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>family_tb</t>
+          <t>page_3c</t>
         </is>
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
-          <t>14. Anyone in family currently suffering from TB</t>
+          <t>Part B: Early Detection – Women only (3 of 3)</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H64" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1611,22 @@
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>history_of_tb</t>
+          <t>foul_smelling_vaginal_discharge</t>
         </is>
       </c>
       <c r="C65" s="16" t="inlineStr">
         <is>
-          <t>15. History of TB</t>
+          <t>13. Foul smelling vaginal discharge</t>
+        </is>
+      </c>
+      <c r="G65" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H65" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1638,12 @@
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>page_2c</t>
+          <t>page_3c</t>
+        </is>
+      </c>
+      <c r="H66" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -1558,12 +1656,12 @@
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>page_2d</t>
+          <t>page_4_phq2</t>
         </is>
       </c>
       <c r="C68" s="16" t="inlineStr">
         <is>
-          <t>Part B: Early Detection – B1: Women and Men (4 of 6)</t>
+          <t>Part C: PHQ 2</t>
         </is>
       </c>
       <c r="E68" s="16" t="inlineStr">
@@ -1575,51 +1673,61 @@
     <row r="69" ht="31.3" customHeight="1" s="13">
       <c r="A69" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>history_of_fits</t>
+          <t>phq2_instructions</t>
         </is>
       </c>
       <c r="C69" s="16" t="inlineStr">
         <is>
-          <t>16. History of fits</t>
+          <t>Over the last 2 weeks, how often have you been bothered by the following problems?</t>
         </is>
       </c>
     </row>
     <row r="70" ht="31.3" customHeight="1" s="13">
       <c r="A70" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B70" s="16" t="inlineStr">
         <is>
-          <t>difficulty_opening_mouth</t>
+          <t>phq2_q1</t>
         </is>
       </c>
       <c r="C70" s="16" t="inlineStr">
         <is>
-          <t>17. Difficulty in opening mouth</t>
+          <t>1. Little interest or pleasure in doing things?</t>
+        </is>
+      </c>
+      <c r="G70" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="71" ht="31.3" customHeight="1" s="13">
       <c r="A71" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B71" s="16" t="inlineStr">
         <is>
-          <t>mouth_ulcers_or_growth</t>
+          <t>phq2_q2</t>
         </is>
       </c>
       <c r="C71" s="16" t="inlineStr">
         <is>
-          <t>18. Ulcers/patch/growth in mouth that has not healed in two weeks</t>
+          <t>2. Feeling down, depressed or hopeless?</t>
+        </is>
+      </c>
+      <c r="G71" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1631,11 +1739,27 @@
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>page_2d</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="31.3" customHeight="1" s="13"/>
+          <t>page_4_phq2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="31.3" customHeight="1" s="13">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>phq2_total</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>${phq2_q1} + ${phq2_q2}</t>
+        </is>
+      </c>
+    </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
         <is>
@@ -1644,12 +1768,12 @@
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>page_2e</t>
+          <t>page_4_phq2_score</t>
         </is>
       </c>
       <c r="C74" s="16" t="inlineStr">
         <is>
-          <t>Part B: Early Detection – B1: Women and Men (5 of 6)</t>
+          <t>Part C: PHQ 2 Score</t>
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr">
@@ -1661,63 +1785,76 @@
     <row r="75" ht="16.4" customHeight="1" s="13">
       <c r="A75" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B75" s="16" t="inlineStr">
         <is>
-          <t>voice_change</t>
+          <t>phq2_score_display</t>
         </is>
       </c>
       <c r="C75" s="16" t="inlineStr">
         <is>
-          <t>19. Any change in the tone of your voice</t>
+          <t>PHQ-2 Total Score: ${phq2_total}</t>
         </is>
       </c>
     </row>
     <row r="76" ht="16.4" customHeight="1" s="13">
       <c r="A76" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B76" s="16" t="inlineStr">
         <is>
-          <t>skin_patch_discoloration</t>
+          <t>phq2_referral_note</t>
         </is>
       </c>
       <c r="C76" s="16" t="inlineStr">
         <is>
-          <t>20. Any patch or discoloration on skin</t>
+          <t>Anyone with total score greater than 3 should be referred to CHO/MO (PHC/UPHC)</t>
+        </is>
+      </c>
+      <c r="H76" s="16" t="inlineStr">
+        <is>
+          <t>${phq2_total} &gt; 3</t>
         </is>
       </c>
     </row>
     <row r="77" ht="31.3" customHeight="1" s="13">
       <c r="A77" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B77" s="16" t="inlineStr">
         <is>
-          <t>difficulty_holding_objects</t>
-        </is>
-      </c>
-      <c r="C77" s="16" t="inlineStr">
-        <is>
-          <t>21. Difficulty in holding objects with fingers</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="16.4" customHeight="1" s="13">
-      <c r="A78" s="16" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B78" s="16" t="inlineStr">
-        <is>
-          <t>page_2e</t>
+          <t>page_4_phq2_score</t>
+        </is>
+      </c>
+      <c r="C77" s="16" t="n"/>
+      <c r="E77" s="16" t="n"/>
+    </row>
+    <row r="78" ht="16.4" customHeight="1" s="13"/>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B79" s="16" t="inlineStr">
+        <is>
+          <t>group_summary</t>
+        </is>
+      </c>
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>Assessment Summary</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1866,7 @@
       </c>
       <c r="B80" s="16" t="inlineStr">
         <is>
-          <t>page_2f</t>
-        </is>
-      </c>
-      <c r="C80" s="16" t="inlineStr">
-        <is>
-          <t>Part B: Early Detection – B1: Women and Men (6 of 6)</t>
+          <t>grp_filled_by</t>
         </is>
       </c>
       <c r="E80" s="16" t="inlineStr">
@@ -1746,33 +1878,49 @@
     <row r="81" ht="61.15" customHeight="1" s="13">
       <c r="A81" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B81" s="16" t="inlineStr">
         <is>
-          <t>loss_of_sensation</t>
+          <t>lbl_filled_by</t>
         </is>
       </c>
       <c r="C81" s="16" t="inlineStr">
         <is>
-          <t>22. Loss of sensation for cold/hot objects in palm or sole</t>
+          <t>**Filled by:** ${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>calc_reporter</t>
+        </is>
+      </c>
+      <c r="F82" s="16" t="inlineStr">
+        <is>
+          <t>${reporter_name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="16.4" customHeight="1" s="13">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B82" s="16" t="inlineStr">
-        <is>
-          <t>page_2f</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="16.4" customHeight="1" s="13"/>
+      <c r="B83" s="16" t="inlineStr">
+        <is>
+          <t>grp_filled_by</t>
+        </is>
+      </c>
+    </row>
     <row r="84" ht="16.4" customHeight="1" s="13">
       <c r="A84" s="16" t="inlineStr">
         <is>
@@ -1781,216 +1929,184 @@
       </c>
       <c r="B84" s="16" t="inlineStr">
         <is>
-          <t>page_3a</t>
-        </is>
-      </c>
-      <c r="C84" s="16" t="inlineStr">
-        <is>
-          <t>Part B: Early Detection – B2: Women only (1 of 3)</t>
+          <t>grp_patient</t>
         </is>
       </c>
       <c r="E84" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
-        </is>
-      </c>
-      <c r="H84" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="85" ht="61.15" customHeight="1" s="13">
       <c r="A85" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B85" s="16" t="inlineStr">
         <is>
-          <t>breast_lump</t>
+          <t>lbl_patient</t>
         </is>
       </c>
       <c r="C85" s="16" t="inlineStr">
         <is>
-          <t>23. Lump in the breast</t>
-        </is>
-      </c>
-      <c r="H85" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>**Patient:** ${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="86" ht="46.25" customHeight="1" s="13">
       <c r="A86" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B86" s="16" t="inlineStr">
         <is>
-          <t>nipple_discharge</t>
-        </is>
-      </c>
-      <c r="C86" s="16" t="inlineStr">
-        <is>
-          <t>24. Blood stained discharge from the nipple</t>
-        </is>
-      </c>
-      <c r="H86" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_patient</t>
+        </is>
+      </c>
+      <c r="F86" s="16" t="inlineStr">
+        <is>
+          <t>${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16.4" customHeight="1" s="13">
       <c r="A87" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B87" s="16" t="inlineStr">
         <is>
-          <t>breast_shape_size_change</t>
-        </is>
-      </c>
-      <c r="C87" s="16" t="inlineStr">
-        <is>
-          <t>25. Change in shape and size of breast</t>
-        </is>
-      </c>
-      <c r="H87" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>grp_patient</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16.4" customHeight="1" s="13">
       <c r="A88" s="16" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B88" s="16" t="inlineStr">
         <is>
-          <t>page_3a</t>
-        </is>
-      </c>
-      <c r="H88" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="16.4" customHeight="1" s="13"/>
+          <t>grp_gender</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="16.4" customHeight="1" s="13">
+      <c r="A89" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B89" s="16" t="inlineStr">
+        <is>
+          <t>lbl_gender</t>
+        </is>
+      </c>
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>**Gender:** ${gender}</t>
+        </is>
+      </c>
+    </row>
     <row r="90" ht="16.4" customHeight="1" s="13">
       <c r="A90" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B90" s="16" t="inlineStr">
         <is>
-          <t>page_3b</t>
-        </is>
-      </c>
-      <c r="C90" s="16" t="inlineStr">
-        <is>
-          <t>Part B: Early Detection – B2: Women only (2 of 3)</t>
-        </is>
-      </c>
-      <c r="E90" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-      <c r="H90" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_gender</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>${gender}</t>
         </is>
       </c>
     </row>
     <row r="91" ht="16.4" customHeight="1" s="13">
       <c r="A91" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
         <is>
-          <t>bleeding_between_periods</t>
-        </is>
-      </c>
-      <c r="C91" s="16" t="inlineStr">
-        <is>
-          <t>26. Bleeding between periods</t>
-        </is>
-      </c>
-      <c r="H91" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>grp_gender</t>
         </is>
       </c>
     </row>
     <row r="92" ht="16.4" customHeight="1" s="13">
       <c r="A92" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B92" s="16" t="inlineStr">
         <is>
-          <t>post_menopause_bleeding</t>
-        </is>
-      </c>
-      <c r="C92" s="16" t="inlineStr">
-        <is>
-          <t>27. Bleeding after menopause</t>
-        </is>
-      </c>
-      <c r="H92" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>grp_state</t>
+        </is>
+      </c>
+      <c r="E92" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16.4" customHeight="1" s="13">
       <c r="A93" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
         <is>
-          <t>post_intercourse_bleeding</t>
+          <t>lbl_state</t>
         </is>
       </c>
       <c r="C93" s="16" t="inlineStr">
         <is>
-          <t>28. Bleeding after intercourse</t>
-        </is>
-      </c>
-      <c r="H93" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>**State:** ${state}</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16.4" customHeight="1" s="13">
       <c r="A94" s="16" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B94" s="16" t="inlineStr">
+        <is>
+          <t>calc_state</t>
+        </is>
+      </c>
+      <c r="F94" s="16" t="inlineStr">
+        <is>
+          <t>${state}</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B94" s="16" t="inlineStr">
-        <is>
-          <t>page_3b</t>
-        </is>
-      </c>
-      <c r="H94" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+      <c r="B95" s="16" t="inlineStr">
+        <is>
+          <t>grp_state</t>
         </is>
       </c>
     </row>
@@ -2002,186 +2118,184 @@
       </c>
       <c r="B96" s="16" t="inlineStr">
         <is>
-          <t>page_3c</t>
-        </is>
-      </c>
-      <c r="C96" s="16" t="inlineStr">
-        <is>
-          <t>Part B: Early Detection – B2: Women only (3 of 3)</t>
+          <t>grp_district</t>
         </is>
       </c>
       <c r="E96" s="16" t="inlineStr">
         <is>
           <t>field-list</t>
-        </is>
-      </c>
-      <c r="H96" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
         <is>
-          <t>foul_smelling_vaginal_discharge</t>
+          <t>lbl_district</t>
         </is>
       </c>
       <c r="C97" s="16" t="inlineStr">
         <is>
-          <t>29. Foul smelling vaginal discharge</t>
-        </is>
-      </c>
-      <c r="H97" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>**District:** ${district}</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B98" s="16" t="inlineStr">
+        <is>
+          <t>calc_district</t>
+        </is>
+      </c>
+      <c r="F98" s="16" t="inlineStr">
+        <is>
+          <t>${district}</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B98" s="16" t="inlineStr">
-        <is>
-          <t>page_3c</t>
-        </is>
-      </c>
-      <c r="H98" s="16" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+      <c r="B99" s="16" t="inlineStr">
+        <is>
+          <t>grp_district</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B100" s="16" t="inlineStr">
         <is>
-          <t>part_c_start_q</t>
-        </is>
-      </c>
-      <c r="F100" s="16" t="inlineStr">
-        <is>
-          <t>if(${gender} = 'male', 23, 30)</t>
+          <t>grp_score</t>
+        </is>
+      </c>
+      <c r="E100" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>part_c_q2</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>if(${gender} = 'male', 24, 31)</t>
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B101" s="16" t="inlineStr">
+        <is>
+          <t>lbl_score</t>
+        </is>
+      </c>
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>**CBAC Total Score:** ${total_score}</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B102" s="16" t="inlineStr">
         <is>
-          <t>page_4</t>
-        </is>
-      </c>
-      <c r="C102" s="16" t="inlineStr">
-        <is>
-          <t>Part C: Circle all that Apply</t>
-        </is>
-      </c>
-      <c r="E102" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>calc_score</t>
+        </is>
+      </c>
+      <c r="F102" s="16" t="inlineStr">
+        <is>
+          <t>${total_score}</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
         <is>
-          <t>select_multiple fuel_type</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>fuel_type_for_cooking</t>
-        </is>
-      </c>
-      <c r="C103" s="16" t="inlineStr">
-        <is>
-          <t>${part_c_start_q}. Type of Fuel used for cooking</t>
+          <t>grp_score</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
         <is>
-          <t>select_multiple occupational_exposure</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B104" s="16" t="inlineStr">
         <is>
-          <t>occupational_exposure</t>
-        </is>
-      </c>
-      <c r="C104" s="16" t="inlineStr">
-        <is>
-          <t>${part_c_q2}. Occupational exposure</t>
+          <t>grp_risk</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>page_4</t>
-        </is>
-      </c>
-    </row>
-    <row r="106"/>
+          <t>lbl_risk</t>
+        </is>
+      </c>
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>**Risk Category:** ${risk_category}</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B106" s="16" t="inlineStr">
+        <is>
+          <t>calc_risk</t>
+        </is>
+      </c>
+      <c r="F106" s="16" t="inlineStr">
+        <is>
+          <t>${risk_category}</t>
+        </is>
+      </c>
+    </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>group_summary</t>
-        </is>
-      </c>
-      <c r="C107" s="16" t="inlineStr">
-        <is>
-          <t>Assessment Summary</t>
-        </is>
-      </c>
-      <c r="E107" s="16" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_risk</t>
         </is>
       </c>
     </row>
@@ -2193,39 +2307,29 @@
       </c>
       <c r="B108" s="16" t="inlineStr">
         <is>
-          <t>summary_high_risk</t>
+          <t>sum_hdr_a</t>
         </is>
       </c>
       <c r="C108" s="16" t="inlineStr">
         <is>
-          <t>Score is greater than 4. This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
-        </is>
-      </c>
-      <c r="H108" s="16" t="inlineStr">
-        <is>
-          <t>${total_score} &gt; 4</t>
+          <t>**Part A: Risk Assessment**</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>summary_low_risk</t>
-        </is>
-      </c>
-      <c r="C109" s="16" t="inlineStr">
-        <is>
-          <t>Score is 4 or below. This person appears to be at low risk for NCDs at this time.</t>
-        </is>
-      </c>
-      <c r="H109" s="16" t="inlineStr">
-        <is>
-          <t>${total_score} &lt;= 4</t>
+          <t>grp_q_age</t>
+        </is>
+      </c>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -2237,103 +2341,58 @@
       </c>
       <c r="B110" s="16" t="inlineStr">
         <is>
-          <t>lbl_filled_by</t>
+          <t>q_age</t>
         </is>
       </c>
       <c r="C110" s="16" t="inlineStr">
         <is>
-          <t>**Filled by:**</t>
-        </is>
-      </c>
-      <c r="E110" s="16" t="inlineStr">
-        <is>
-          <t>w5</t>
-        </is>
-      </c>
-      <c r="F110" s="16" t="inlineStr">
-        <is>
-          <t>${reporter_name}</t>
+          <t>1. Age: ${age_range}</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
         <is>
-          <t>lbl_patient_val</t>
-        </is>
-      </c>
-      <c r="C111" s="16" t="inlineStr">
-        <is>
-          <t>**Patient:**</t>
-        </is>
-      </c>
-      <c r="E111" s="16" t="inlineStr">
-        <is>
-          <t>w5</t>
+          <t>calc_q_age</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>${patient_name}</t>
+          <t>${age_range}</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B112" s="16" t="inlineStr">
         <is>
-          <t>lbl_gender_val</t>
-        </is>
-      </c>
-      <c r="C112" s="16" t="inlineStr">
-        <is>
-          <t>**Gender:**</t>
-        </is>
-      </c>
-      <c r="E112" s="16" t="inlineStr">
-        <is>
-          <t>w5</t>
-        </is>
-      </c>
-      <c r="F112" s="16" t="inlineStr">
-        <is>
-          <t>${gender}</t>
+          <t>grp_q_age</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
         <is>
-          <t>lbl_state_val</t>
-        </is>
-      </c>
-      <c r="C113" s="16" t="inlineStr">
-        <is>
-          <t>**State:**</t>
+          <t>grp_q_smoke</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>w5</t>
-        </is>
-      </c>
-      <c r="F113" s="16" t="inlineStr">
-        <is>
-          <t>${state}</t>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -2345,88 +2404,1140 @@
       </c>
       <c r="B114" s="16" t="inlineStr">
         <is>
-          <t>lbl_district_val</t>
+          <t>q_smoke</t>
         </is>
       </c>
       <c r="C114" s="16" t="inlineStr">
         <is>
-          <t>**District:**</t>
-        </is>
-      </c>
-      <c r="E114" s="16" t="inlineStr">
-        <is>
-          <t>w5</t>
-        </is>
-      </c>
-      <c r="F114" s="16" t="inlineStr">
-        <is>
-          <t>${district}</t>
+          <t>2. Smoke/Smokeless products: ${smoke_frequency}</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>lbl_score_val</t>
-        </is>
-      </c>
-      <c r="C115" s="16" t="inlineStr">
-        <is>
-          <t>**CBAC Total Score:**</t>
-        </is>
-      </c>
-      <c r="E115" s="16" t="inlineStr">
-        <is>
-          <t>w5</t>
+          <t>calc_q_smoke</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>${total_score}</t>
+          <t>${smoke_frequency}</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B116" s="16" t="inlineStr">
         <is>
-          <t>lbl_risk_val</t>
-        </is>
-      </c>
-      <c r="C116" s="16" t="inlineStr">
-        <is>
-          <t>**Risk Category:**</t>
-        </is>
-      </c>
-      <c r="E116" s="16" t="inlineStr">
-        <is>
-          <t>w5</t>
-        </is>
-      </c>
-      <c r="F116" s="16" t="inlineStr">
-        <is>
-          <t>${risk_category}</t>
+          <t>grp_q_smoke</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="16" t="inlineStr">
         <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B117" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_alcohol</t>
+        </is>
+      </c>
+      <c r="E117" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B118" s="16" t="inlineStr">
+        <is>
+          <t>q_alcohol</t>
+        </is>
+      </c>
+      <c r="C118" s="16" t="inlineStr">
+        <is>
+          <t>3. Alcohol daily: ${alcohol_frequency}</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B119" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_alcohol</t>
+        </is>
+      </c>
+      <c r="F119" s="16" t="inlineStr">
+        <is>
+          <t>${alcohol_frequency}</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="16" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B117" s="16" t="inlineStr">
+      <c r="B120" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_alcohol</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B121" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_waist</t>
+        </is>
+      </c>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B122" s="16" t="inlineStr">
+        <is>
+          <t>q_waist</t>
+        </is>
+      </c>
+      <c r="C122" s="16" t="inlineStr">
+        <is>
+          <t>4. Waist measurement: ${waist_size}</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B123" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_waist</t>
+        </is>
+      </c>
+      <c r="F123" s="16" t="inlineStr">
+        <is>
+          <t>${waist_size}</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B124" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_waist</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B125" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_physical</t>
+        </is>
+      </c>
+      <c r="E125" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B126" s="16" t="inlineStr">
+        <is>
+          <t>q_physical</t>
+        </is>
+      </c>
+      <c r="C126" s="16" t="inlineStr">
+        <is>
+          <t>5. Physical activity (150 min/week): ${physical_activities_frequency}</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B127" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_physical</t>
+        </is>
+      </c>
+      <c r="F127" s="16" t="inlineStr">
+        <is>
+          <t>${physical_activities_frequency}</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B128" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_physical</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B129" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_family</t>
+        </is>
+      </c>
+      <c r="E129" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B130" s="16" t="inlineStr">
+        <is>
+          <t>q_family</t>
+        </is>
+      </c>
+      <c r="C130" s="16" t="inlineStr">
+        <is>
+          <t>6. Family history of BP/Diabetes/Heart disease: ${family_medical_history}</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B131" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_family</t>
+        </is>
+      </c>
+      <c r="F131" s="16" t="inlineStr">
+        <is>
+          <t>${family_medical_history}</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B132" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_family</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B133" s="16" t="inlineStr">
+        <is>
+          <t>sum_hdr_b</t>
+        </is>
+      </c>
+      <c r="C133" s="16" t="inlineStr">
+        <is>
+          <t>**Part B: Early Detection**</t>
+        </is>
+      </c>
+      <c r="H133" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B134" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_breast_lump</t>
+        </is>
+      </c>
+      <c r="E134" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H134" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B135" s="16" t="inlineStr">
+        <is>
+          <t>q_breast_lump</t>
+        </is>
+      </c>
+      <c r="C135" s="16" t="inlineStr">
+        <is>
+          <t>7. Lump in the breast: ${breast_lump}</t>
+        </is>
+      </c>
+      <c r="H135" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B136" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_breast_lump</t>
+        </is>
+      </c>
+      <c r="F136" s="16" t="inlineStr">
+        <is>
+          <t>${breast_lump}</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B137" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_breast_lump</t>
+        </is>
+      </c>
+      <c r="H137" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B138" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_nipple</t>
+        </is>
+      </c>
+      <c r="E138" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H138" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B139" s="16" t="inlineStr">
+        <is>
+          <t>q_nipple</t>
+        </is>
+      </c>
+      <c r="C139" s="16" t="inlineStr">
+        <is>
+          <t>8. Blood stained nipple discharge: ${nipple_discharge}</t>
+        </is>
+      </c>
+      <c r="H139" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B140" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_nipple</t>
+        </is>
+      </c>
+      <c r="F140" s="16" t="inlineStr">
+        <is>
+          <t>${nipple_discharge}</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B141" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_nipple</t>
+        </is>
+      </c>
+      <c r="H141" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B142" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_breast_shape</t>
+        </is>
+      </c>
+      <c r="E142" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H142" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B143" s="16" t="inlineStr">
+        <is>
+          <t>q_breast_shape</t>
+        </is>
+      </c>
+      <c r="C143" s="16" t="inlineStr">
+        <is>
+          <t>9. Change in breast shape/size: ${breast_shape_size_change}</t>
+        </is>
+      </c>
+      <c r="H143" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B144" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_breast_shape</t>
+        </is>
+      </c>
+      <c r="F144" s="16" t="inlineStr">
+        <is>
+          <t>${breast_shape_size_change}</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B145" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_breast_shape</t>
+        </is>
+      </c>
+      <c r="H145" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B146" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="E146" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H146" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B147" s="16" t="inlineStr">
+        <is>
+          <t>q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="C147" s="16" t="inlineStr">
+        <is>
+          <t>10. Bleeding between periods: ${bleeding_between_periods}</t>
+        </is>
+      </c>
+      <c r="H147" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B148" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="F148" s="16" t="inlineStr">
+        <is>
+          <t>${bleeding_between_periods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B149" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="H149" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B150" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_menopause</t>
+        </is>
+      </c>
+      <c r="E150" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H150" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B151" s="16" t="inlineStr">
+        <is>
+          <t>q_menopause</t>
+        </is>
+      </c>
+      <c r="C151" s="16" t="inlineStr">
+        <is>
+          <t>11. Bleeding after menopause: ${post_menopause_bleeding}</t>
+        </is>
+      </c>
+      <c r="H151" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B152" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_menopause</t>
+        </is>
+      </c>
+      <c r="F152" s="16" t="inlineStr">
+        <is>
+          <t>${post_menopause_bleeding}</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B153" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_menopause</t>
+        </is>
+      </c>
+      <c r="H153" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B154" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_intercourse</t>
+        </is>
+      </c>
+      <c r="E154" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H154" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B155" s="16" t="inlineStr">
+        <is>
+          <t>q_intercourse</t>
+        </is>
+      </c>
+      <c r="C155" s="16" t="inlineStr">
+        <is>
+          <t>12. Bleeding after intercourse: ${post_intercourse_bleeding}</t>
+        </is>
+      </c>
+      <c r="H155" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B156" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_intercourse</t>
+        </is>
+      </c>
+      <c r="F156" s="16" t="inlineStr">
+        <is>
+          <t>${post_intercourse_bleeding}</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B157" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_intercourse</t>
+        </is>
+      </c>
+      <c r="H157" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B158" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_discharge</t>
+        </is>
+      </c>
+      <c r="E158" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H158" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B159" s="16" t="inlineStr">
+        <is>
+          <t>q_discharge</t>
+        </is>
+      </c>
+      <c r="C159" s="16" t="inlineStr">
+        <is>
+          <t>13. Foul smelling vaginal discharge: ${foul_smelling_vaginal_discharge}</t>
+        </is>
+      </c>
+      <c r="H159" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B160" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_discharge</t>
+        </is>
+      </c>
+      <c r="F160" s="16" t="inlineStr">
+        <is>
+          <t>${foul_smelling_vaginal_discharge}</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B161" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_discharge</t>
+        </is>
+      </c>
+      <c r="H161" s="16" t="inlineStr">
+        <is>
+          <t>${gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B162" s="16" t="inlineStr">
+        <is>
+          <t>sum_hdr_d</t>
+        </is>
+      </c>
+      <c r="C162" s="16" t="inlineStr">
+        <is>
+          <t>**Part C: PHQ-2**</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B163" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_phq1</t>
+        </is>
+      </c>
+      <c r="E163" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B164" s="16" t="inlineStr">
+        <is>
+          <t>q_phq1</t>
+        </is>
+      </c>
+      <c r="C164" s="16" t="inlineStr">
+        <is>
+          <t>1. Little interest or pleasure in doing things: ${phq2_q1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B165" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_phq1</t>
+        </is>
+      </c>
+      <c r="F165" s="16" t="inlineStr">
+        <is>
+          <t>${phq2_q1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B166" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_phq1</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B167" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_phq2</t>
+        </is>
+      </c>
+      <c r="E167" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B168" s="16" t="inlineStr">
+        <is>
+          <t>q_phq2</t>
+        </is>
+      </c>
+      <c r="C168" s="16" t="inlineStr">
+        <is>
+          <t>2. Feeling down, depressed or hopeless: ${phq2_q2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B169" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_phq2</t>
+        </is>
+      </c>
+      <c r="F169" s="16" t="inlineStr">
+        <is>
+          <t>${phq2_q2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B170" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_phq2</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="16" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B171" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_phq_tot</t>
+        </is>
+      </c>
+      <c r="E171" s="16" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B172" s="16" t="inlineStr">
+        <is>
+          <t>q_phq_tot</t>
+        </is>
+      </c>
+      <c r="C172" s="16" t="inlineStr">
+        <is>
+          <t>PHQ-2 Total Score: ${phq2_total}</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B173" s="16" t="inlineStr">
+        <is>
+          <t>calc_q_phq_tot</t>
+        </is>
+      </c>
+      <c r="F173" s="16" t="inlineStr">
+        <is>
+          <t>${phq2_total}</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B174" s="16" t="inlineStr">
+        <is>
+          <t>grp_q_phq_tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B175" s="16" t="inlineStr">
+        <is>
+          <t>summary_high_risk</t>
+        </is>
+      </c>
+      <c r="C175" s="16" t="inlineStr">
+        <is>
+          <t>**Score is greater than 4.** This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
+        </is>
+      </c>
+      <c r="H175" s="16" t="inlineStr">
+        <is>
+          <t>${total_score} &gt; 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="16" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B176" s="16" t="inlineStr">
+        <is>
+          <t>summary_low_risk</t>
+        </is>
+      </c>
+      <c r="C176" s="16" t="inlineStr">
+        <is>
+          <t>**Score is 4 or below.** This person appears to be at low risk for NCDs at this time.</t>
+        </is>
+      </c>
+      <c r="H176" s="16" t="inlineStr">
+        <is>
+          <t>${total_score} &lt;= 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="16" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B177" s="16" t="inlineStr">
         <is>
           <t>group_summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B178" s="16" t="inlineStr">
+        <is>
+          <t>form_submit_timestamp</t>
+        </is>
+      </c>
+      <c r="F178" s="16" t="inlineStr">
+        <is>
+          <t>now()</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: use jr:choice-name to display human-readable labels in form summary calculations
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/cbac.xlsx
+++ b/config/demo/forms/app/cbac.xlsx
@@ -1893,17 +1893,17 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="16" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B82" s="16" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>calc_reporter</t>
         </is>
       </c>
-      <c r="F82" s="16" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>${reporter_name}</t>
         </is>
@@ -1956,17 +1956,17 @@
       </c>
     </row>
     <row r="86" ht="46.25" customHeight="1" s="13">
-      <c r="A86" s="16" t="inlineStr">
+      <c r="A86" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B86" s="16" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>calc_patient</t>
         </is>
       </c>
-      <c r="F86" s="16" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>${patient_name}</t>
         </is>
@@ -2019,17 +2019,17 @@
       </c>
     </row>
     <row r="90" ht="16.4" customHeight="1" s="13">
-      <c r="A90" s="16" t="inlineStr">
+      <c r="A90" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B90" s="16" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>calc_gender</t>
         </is>
       </c>
-      <c r="F90" s="16" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>${gender}</t>
         </is>
@@ -2082,17 +2082,17 @@
       </c>
     </row>
     <row r="94" ht="16.4" customHeight="1" s="13">
-      <c r="A94" s="16" t="inlineStr">
+      <c r="A94" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B94" s="16" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>calc_state</t>
         </is>
       </c>
-      <c r="F94" s="16" t="inlineStr">
+      <c r="F94" t="inlineStr">
         <is>
           <t>${state}</t>
         </is>
@@ -2145,17 +2145,17 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="16" t="inlineStr">
+      <c r="A98" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B98" s="16" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>calc_district</t>
         </is>
       </c>
-      <c r="F98" s="16" t="inlineStr">
+      <c r="F98" t="inlineStr">
         <is>
           <t>${district}</t>
         </is>
@@ -2208,17 +2208,17 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="16" t="inlineStr">
+      <c r="A102" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B102" s="16" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>calc_score</t>
         </is>
       </c>
-      <c r="F102" s="16" t="inlineStr">
+      <c r="F102" t="inlineStr">
         <is>
           <t>${total_score}</t>
         </is>
@@ -2271,17 +2271,17 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="16" t="inlineStr">
+      <c r="A106" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B106" s="16" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>calc_risk</t>
         </is>
       </c>
-      <c r="F106" s="16" t="inlineStr">
+      <c r="F106" t="inlineStr">
         <is>
           <t>${risk_category}</t>
         </is>
@@ -2346,24 +2346,24 @@
       </c>
       <c r="C110" s="16" t="inlineStr">
         <is>
-          <t>1. Age: ${age_range}</t>
+          <t>1. Age: ${calc_q_age}</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="16" t="inlineStr">
+      <c r="A111" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B111" s="16" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>calc_q_age</t>
         </is>
       </c>
-      <c r="F111" s="16" t="inlineStr">
-        <is>
-          <t>${age_range}</t>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${age_range}, '${age_range}')</t>
         </is>
       </c>
     </row>
@@ -2409,24 +2409,24 @@
       </c>
       <c r="C114" s="16" t="inlineStr">
         <is>
-          <t>2. Smoke/Smokeless products: ${smoke_frequency}</t>
+          <t>2. Smoke/Smokeless products: ${calc_q_smoke}</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="16" t="inlineStr">
+      <c r="A115" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B115" s="16" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>calc_q_smoke</t>
         </is>
       </c>
-      <c r="F115" s="16" t="inlineStr">
-        <is>
-          <t>${smoke_frequency}</t>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${smoke_frequency}, '${smoke_frequency}')</t>
         </is>
       </c>
     </row>
@@ -2472,24 +2472,24 @@
       </c>
       <c r="C118" s="16" t="inlineStr">
         <is>
-          <t>3. Alcohol daily: ${alcohol_frequency}</t>
+          <t>3. Alcohol daily: ${calc_q_alcohol}</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="16" t="inlineStr">
+      <c r="A119" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B119" s="16" t="inlineStr">
+      <c r="B119" t="inlineStr">
         <is>
           <t>calc_q_alcohol</t>
         </is>
       </c>
-      <c r="F119" s="16" t="inlineStr">
-        <is>
-          <t>${alcohol_frequency}</t>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${alcohol_frequency}, '${alcohol_frequency}')</t>
         </is>
       </c>
     </row>
@@ -2535,24 +2535,24 @@
       </c>
       <c r="C122" s="16" t="inlineStr">
         <is>
-          <t>4. Waist measurement: ${waist_size}</t>
+          <t>4. Waist measurement: ${calc_q_waist}</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="16" t="inlineStr">
+      <c r="A123" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B123" s="16" t="inlineStr">
+      <c r="B123" t="inlineStr">
         <is>
           <t>calc_q_waist</t>
         </is>
       </c>
-      <c r="F123" s="16" t="inlineStr">
-        <is>
-          <t>${waist_size}</t>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${waist_size}, '${waist_size}')</t>
         </is>
       </c>
     </row>
@@ -2598,24 +2598,24 @@
       </c>
       <c r="C126" s="16" t="inlineStr">
         <is>
-          <t>5. Physical activity (150 min/week): ${physical_activities_frequency}</t>
+          <t>5. Physical activity (150 min/week): ${calc_q_physical}</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="16" t="inlineStr">
+      <c r="A127" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B127" s="16" t="inlineStr">
+      <c r="B127" t="inlineStr">
         <is>
           <t>calc_q_physical</t>
         </is>
       </c>
-      <c r="F127" s="16" t="inlineStr">
-        <is>
-          <t>${physical_activities_frequency}</t>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${physical_activities_frequency}, '${physical_activities_frequency}')</t>
         </is>
       </c>
     </row>
@@ -2661,24 +2661,24 @@
       </c>
       <c r="C130" s="16" t="inlineStr">
         <is>
-          <t>6. Family history of BP/Diabetes/Heart disease: ${family_medical_history}</t>
+          <t>6. Family history of BP/Diabetes/Heart disease: ${calc_q_family}</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="16" t="inlineStr">
+      <c r="A131" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B131" s="16" t="inlineStr">
+      <c r="B131" t="inlineStr">
         <is>
           <t>calc_q_family</t>
         </is>
       </c>
-      <c r="F131" s="16" t="inlineStr">
-        <is>
-          <t>${family_medical_history}</t>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${family_medical_history}, '${family_medical_history}')</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C135" s="16" t="inlineStr">
         <is>
-          <t>7. Lump in the breast: ${breast_lump}</t>
+          <t>7. Lump in the breast: ${calc_q_breast_lump}</t>
         </is>
       </c>
       <c r="H135" s="16" t="inlineStr">
@@ -2761,19 +2761,19 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="16" t="inlineStr">
+      <c r="A136" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B136" s="16" t="inlineStr">
+      <c r="B136" t="inlineStr">
         <is>
           <t>calc_q_breast_lump</t>
         </is>
       </c>
-      <c r="F136" s="16" t="inlineStr">
-        <is>
-          <t>${breast_lump}</t>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="C139" s="16" t="inlineStr">
         <is>
-          <t>8. Blood stained nipple discharge: ${nipple_discharge}</t>
+          <t>8. Blood stained nipple discharge: ${calc_q_nipple}</t>
         </is>
       </c>
       <c r="H139" s="16" t="inlineStr">
@@ -2839,19 +2839,19 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="16" t="inlineStr">
+      <c r="A140" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B140" s="16" t="inlineStr">
+      <c r="B140" t="inlineStr">
         <is>
           <t>calc_q_nipple</t>
         </is>
       </c>
-      <c r="F140" s="16" t="inlineStr">
-        <is>
-          <t>${nipple_discharge}</t>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2907,7 @@
       </c>
       <c r="C143" s="16" t="inlineStr">
         <is>
-          <t>9. Change in breast shape/size: ${breast_shape_size_change}</t>
+          <t>9. Change in breast shape/size: ${calc_q_breast_shape}</t>
         </is>
       </c>
       <c r="H143" s="16" t="inlineStr">
@@ -2917,19 +2917,19 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="16" t="inlineStr">
+      <c r="A144" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B144" s="16" t="inlineStr">
+      <c r="B144" t="inlineStr">
         <is>
           <t>calc_q_breast_shape</t>
         </is>
       </c>
-      <c r="F144" s="16" t="inlineStr">
-        <is>
-          <t>${breast_shape_size_change}</t>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="C147" s="16" t="inlineStr">
         <is>
-          <t>10. Bleeding between periods: ${bleeding_between_periods}</t>
+          <t>10. Bleeding between periods: ${calc_q_bleeding_periods}</t>
         </is>
       </c>
       <c r="H147" s="16" t="inlineStr">
@@ -2995,19 +2995,19 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="16" t="inlineStr">
+      <c r="A148" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B148" s="16" t="inlineStr">
+      <c r="B148" t="inlineStr">
         <is>
           <t>calc_q_bleeding_periods</t>
         </is>
       </c>
-      <c r="F148" s="16" t="inlineStr">
-        <is>
-          <t>${bleeding_between_periods}</t>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="C151" s="16" t="inlineStr">
         <is>
-          <t>11. Bleeding after menopause: ${post_menopause_bleeding}</t>
+          <t>11. Bleeding after menopause: ${calc_q_menopause}</t>
         </is>
       </c>
       <c r="H151" s="16" t="inlineStr">
@@ -3073,19 +3073,19 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="16" t="inlineStr">
+      <c r="A152" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B152" s="16" t="inlineStr">
+      <c r="B152" t="inlineStr">
         <is>
           <t>calc_q_menopause</t>
         </is>
       </c>
-      <c r="F152" s="16" t="inlineStr">
-        <is>
-          <t>${post_menopause_bleeding}</t>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="C155" s="16" t="inlineStr">
         <is>
-          <t>12. Bleeding after intercourse: ${post_intercourse_bleeding}</t>
+          <t>12. Bleeding after intercourse: ${calc_q_intercourse}</t>
         </is>
       </c>
       <c r="H155" s="16" t="inlineStr">
@@ -3151,19 +3151,19 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="16" t="inlineStr">
+      <c r="A156" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B156" s="16" t="inlineStr">
+      <c r="B156" t="inlineStr">
         <is>
           <t>calc_q_intercourse</t>
         </is>
       </c>
-      <c r="F156" s="16" t="inlineStr">
-        <is>
-          <t>${post_intercourse_bleeding}</t>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="C159" s="16" t="inlineStr">
         <is>
-          <t>13. Foul smelling vaginal discharge: ${foul_smelling_vaginal_discharge}</t>
+          <t>13. Foul smelling vaginal discharge: ${calc_q_discharge}</t>
         </is>
       </c>
       <c r="H159" s="16" t="inlineStr">
@@ -3229,19 +3229,19 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="16" t="inlineStr">
+      <c r="A160" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B160" s="16" t="inlineStr">
+      <c r="B160" t="inlineStr">
         <is>
           <t>calc_q_discharge</t>
         </is>
       </c>
-      <c r="F160" s="16" t="inlineStr">
-        <is>
-          <t>${foul_smelling_vaginal_discharge}</t>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
         </is>
       </c>
     </row>
@@ -3309,24 +3309,24 @@
       </c>
       <c r="C164" s="16" t="inlineStr">
         <is>
-          <t>1. Little interest or pleasure in doing things: ${phq2_q1}</t>
+          <t>1. Little interest or pleasure in doing things: ${calc_q_phq1}</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="16" t="inlineStr">
+      <c r="A165" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B165" s="16" t="inlineStr">
+      <c r="B165" t="inlineStr">
         <is>
           <t>calc_q_phq1</t>
         </is>
       </c>
-      <c r="F165" s="16" t="inlineStr">
-        <is>
-          <t>${phq2_q1}</t>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
         </is>
       </c>
     </row>
@@ -3372,24 +3372,24 @@
       </c>
       <c r="C168" s="16" t="inlineStr">
         <is>
-          <t>2. Feeling down, depressed or hopeless: ${phq2_q2}</t>
+          <t>2. Feeling down, depressed or hopeless: ${calc_q_phq2}</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="16" t="inlineStr">
+      <c r="A169" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B169" s="16" t="inlineStr">
+      <c r="B169" t="inlineStr">
         <is>
           <t>calc_q_phq2</t>
         </is>
       </c>
-      <c r="F169" s="16" t="inlineStr">
-        <is>
-          <t>${phq2_q2}</t>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
         </is>
       </c>
     </row>
@@ -3440,17 +3440,17 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="16" t="inlineStr">
+      <c r="A173" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B173" s="16" t="inlineStr">
+      <c r="B173" t="inlineStr">
         <is>
           <t>calc_q_phq_tot</t>
         </is>
       </c>
-      <c r="F173" s="16" t="inlineStr">
+      <c r="F173" t="inlineStr">
         <is>
           <t>${phq2_total}</t>
         </is>

</xml_diff>

<commit_message>
refactor: replace manual age and gender inputs with profile data in NCD forms and update patient contact labels.
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/cbac.xlsx
+++ b/config/demo/forms/app/cbac.xlsx
@@ -422,21 +422,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I207"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="10.16015625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:I208"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="29.53515625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="27.94" customWidth="1" style="10" min="1" max="1"/>
-    <col width="24.51" customWidth="1" style="10" min="2" max="2"/>
-    <col width="33.09" customWidth="1" style="10" min="3" max="3"/>
-    <col width="17.03" customWidth="1" style="10" min="4" max="4"/>
-    <col width="21.32" customWidth="1" style="10" min="5" max="5"/>
-    <col width="37.54" customWidth="1" style="10" min="6" max="6"/>
-    <col width="10.16" customWidth="1" style="10" min="7" max="7"/>
-    <col width="17.44" customWidth="1" style="10" min="8" max="8"/>
-    <col width="10.16" customWidth="1" style="10" min="9" max="16384"/>
+    <col width="29.53" customWidth="1" style="10" min="1" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30.75" customHeight="1" s="11">
+    <row r="1" ht="16.4" customHeight="1" s="11">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>type</t>
@@ -483,7 +475,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="11">
+    <row r="2" ht="16.4" customHeight="1" s="11">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>calculate</t>
@@ -500,7 +492,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" s="11">
+    <row r="3" ht="16.4" customHeight="1" s="11">
       <c r="A3" s="10" t="inlineStr">
         <is>
           <t>calculate</t>
@@ -517,7 +509,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" s="11">
+    <row r="4" ht="16.4" customHeight="1" s="11">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>calculate</t>
@@ -534,1587 +526,1577 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" s="11">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="5" ht="16.4" customHeight="1" s="11">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>patient_gender</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>../inputs/contact/sex</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>reporter_name</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Reporter Name</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>../inputs/user/name</t>
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7" ht="30.75" customHeight="1" s="11">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="7" ht="31.3" customHeight="1" s="11"/>
+    <row r="8" ht="16.4" customHeight="1" s="11">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>reporter_place</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Reporter Place</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>instance('user-contact-summary')/context/facility_name</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1" s="11">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="11">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>${patient_name}</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="11">
-      <c r="A9" s="13" t="inlineStr">
+    <row r="10" ht="16.4" customHeight="1" s="11">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>form_start_timestamp</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>once(if(${_id} != '', now(), ''))</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" s="11">
-      <c r="A10" s="10" t="inlineStr">
+    <row r="11" ht="16.4" customHeight="1" s="11">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>inputs</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Patient &amp; Reporter Info</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1" s="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12" ht="16.4" customHeight="1" s="11">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1" s="11">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="13" ht="16.4" customHeight="1" s="11">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>source_id</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1" s="11">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14" ht="16.4" customHeight="1" s="11">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1" s="11">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="15" ht="16.4" customHeight="1" s="11">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15.75" customHeight="1" s="11">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="16" ht="16.4" customHeight="1" s="11">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1" s="11">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="17" ht="16.4" customHeight="1" s="11">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="11">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18" ht="16.4" customHeight="1" s="11">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>reporter_name_note</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Filled by: ${reporter_name}</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30.75" customHeight="1" s="11">
-      <c r="A18" s="10" t="inlineStr">
+    <row r="19" ht="16.4" customHeight="1" s="11">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>contact</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="11">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="20" ht="16.4" customHeight="1" s="11">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>_id</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Patient's Name</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Select the patient from your area</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>select-contact type-patient</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" s="11">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="21" ht="16.4" customHeight="1" s="11">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>patient_id</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Medic ID</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="11">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="11">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>Patient Name</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1" s="11">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>select_one gender</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>gender</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="G22" s="10" t="inlineStr">
+    <row r="23" ht="16.4" customHeight="1" s="11">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16.4" customHeight="1" s="11">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16.4" customHeight="1" s="11">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>select_one states</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1" s="11">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="26" ht="16.4" customHeight="1" s="11">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>select_one districts</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>filter = ${state}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16.4" customHeight="1" s="11">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>contact</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30.75" customHeight="1" s="11">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>select_one states</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16.4" customHeight="1" s="11">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>total_question</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>if(${patient_gender} = 'male', '0', '7')</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="11">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>instructions</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Part A consists of 6 questions. Each question carries a score. A total score above 4 indicates high risk for NCDs — such a person should be prioritised for further examination at the weekly NCD clinic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="11">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>page_1a</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Part A: Risk Assessment (1 of 2)</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="11">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>select_one age_range</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>age_range</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>1. What is your age? (in complete years)</t>
+        </is>
+      </c>
+      <c r="G31" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" s="11">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>select_one districts</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>District</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="G25" s="10" t="inlineStr">
+    <row r="32" ht="15" customHeight="1" s="11">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>age_range_label</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${age_range}, '${age_range}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="11">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>select_one smoke_frequency</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>smoke_frequency</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>2. Do you smoke or consume smokeless products such as gutka or khaini?</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>filter = ${state}</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="60.75" customHeight="1" s="11">
-      <c r="A26" s="10" t="inlineStr">
+    </row>
+    <row r="34" ht="15" customHeight="1" s="11">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>smoke_frequency_label</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${smoke_frequency}, '${smoke_frequency}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="11">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>select_one alcohol_frequency</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>alcohol_frequency</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>3. Do you consume alcohol daily</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="11">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>alcohol_frequency_label</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${alcohol_frequency}, '${alcohol_frequency}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="11">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>inputs</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="11">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>total_question</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>if(${gender} = 'male', '0', '7')</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="11">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>instructions</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>Part A consists of 6 questions. Each question carries a score. A total score above 4 indicates high risk for NCDs — such a person should be prioritised for further examination at the weekly NCD clinic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1" s="11">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>page_1a</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>Part A: Risk Assessment (1 of 2)</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30.75" customHeight="1" s="11">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>select_one age_range</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>age_range</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>1. What is your age? (in complete years)</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30.75" customHeight="1" s="11">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>age_range_label</t>
-        </is>
-      </c>
-      <c r="F31" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${age_range}, '${age_range}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="45.75" customHeight="1" s="11">
-      <c r="A32" s="13" t="inlineStr">
-        <is>
-          <t>select_one smoke_frequency</t>
-        </is>
-      </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>smoke_frequency</t>
-        </is>
-      </c>
-      <c r="C32" s="13" t="inlineStr">
-        <is>
-          <t>2. Do you smoke or consume smokeless products such as gutka or khaini?</t>
-        </is>
-      </c>
-      <c r="G32" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30.75" customHeight="1" s="11">
-      <c r="A33" s="13" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>smoke_frequency_label</t>
-        </is>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${smoke_frequency}, '${smoke_frequency}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30.75" customHeight="1" s="11">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>select_one alcohol_frequency</t>
-        </is>
-      </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>alcohol_frequency</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="inlineStr">
-        <is>
-          <t>3. Do you consume alcohol daily</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="45.75" customHeight="1" s="11">
-      <c r="A35" s="13" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>alcohol_frequency_label</t>
-        </is>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${alcohol_frequency}, '${alcohol_frequency}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="60.75" customHeight="1" s="11">
-      <c r="A36" s="13" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>page_1a</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" s="11"/>
-    <row r="38" ht="15" customHeight="1" s="11">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>page_1b</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>Part A: Risk Assessment (2 of 2)</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
+    </row>
+    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="11">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>select_one waist_size</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>waist_size</t>
+          <t>page_1b</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>4. Measurement of waist (in cm)</t>
-        </is>
-      </c>
-      <c r="G39" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I39" s="13" t="inlineStr">
-        <is>
-          <t>filter = ${gender}</t>
+          <t>Part A: Risk Assessment (2 of 2)</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="11">
       <c r="A40" s="13" t="inlineStr">
         <is>
+          <t>select_one waist_size</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>waist_size</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>4. Measurement of waist (in cm)</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>filter = ${patient_gender}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="11">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>waist_size_label</t>
         </is>
       </c>
-      <c r="F40" s="13" t="inlineStr">
+      <c r="F41" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${waist_size}, '${waist_size}')</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30.75" customHeight="1" s="11">
-      <c r="A41" s="13" t="inlineStr">
+    <row r="42" ht="15" customHeight="1" s="11">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>select_one physical_activities_frequency</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>physical_activities_frequency</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
+      <c r="C42" s="13" t="inlineStr">
         <is>
           <t>5. Do you undertake any physical activities for minimum of 150 minutes in a week?</t>
         </is>
       </c>
-      <c r="G41" s="13" t="inlineStr">
+      <c r="G42" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="15.75" customHeight="1" s="11">
-      <c r="A42" s="13" t="inlineStr">
+    <row r="43" ht="15" customHeight="1" s="11">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>physical_activities_frequency_label</t>
         </is>
       </c>
-      <c r="F42" s="13" t="inlineStr">
+      <c r="F43" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${physical_activities_frequency}, '${physical_activities_frequency}')</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="30.75" customHeight="1" s="11">
-      <c r="A43" s="13" t="inlineStr">
+    <row r="44" ht="15" customHeight="1" s="11">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>select_one family_medical_history</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>family_medical_history</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
         <is>
           <t>6. Do you have a family history (any one of your parents or siblings) of high blood pressure, diabetes and heart disease?</t>
         </is>
       </c>
-      <c r="G43" s="13" t="inlineStr">
+      <c r="G44" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1" s="11">
-      <c r="A44" s="13" t="inlineStr">
+    <row r="45" ht="15" customHeight="1" s="11">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>family_medical_history_label</t>
         </is>
       </c>
-      <c r="F44" s="13" t="inlineStr">
+      <c r="F45" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${family_medical_history}, '${family_medical_history}')</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1" s="11">
-      <c r="A45" s="13" t="inlineStr">
+    <row r="46" ht="15" customHeight="1" s="11">
+      <c r="A46" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B46" s="13" t="inlineStr">
         <is>
           <t>page_1b</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1" s="11"/>
-    <row r="47" ht="15.75" customHeight="1" s="11">
-      <c r="A47" s="13" t="inlineStr">
+    <row r="47"/>
+    <row r="48" ht="15" customHeight="1" s="11">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>total_score</t>
         </is>
       </c>
-      <c r="F47" s="13" t="inlineStr">
+      <c r="F48" s="13" t="inlineStr">
         <is>
           <t>${age_range} + ${smoke_frequency} + ${alcohol_frequency} + ${waist_size} + ${physical_activities_frequency} + ${family_medical_history}</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1" s="11">
-      <c r="A48" s="13" t="inlineStr">
+    <row r="49" ht="15" customHeight="1" s="11">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
+      <c r="B49" s="13" t="inlineStr">
         <is>
           <t>risk_category</t>
         </is>
       </c>
-      <c r="F48" s="13" t="inlineStr">
+      <c r="F49" s="13" t="inlineStr">
         <is>
           <t>if(${total_score} &gt; 4, 'High Risk', 'Low Risk')</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="15.75" customHeight="1" s="11"/>
-    <row r="50" ht="30.75" customHeight="1" s="11">
-      <c r="A50" s="13" t="inlineStr">
+    <row r="50"/>
+    <row r="51" ht="15" customHeight="1" s="11">
+      <c r="A51" s="13" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B51" s="13" t="inlineStr">
         <is>
           <t>page_score</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>Part A: Risk Assessment Score Summary</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E51" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="30.75" customHeight="1" s="11">
-      <c r="A51" s="13" t="inlineStr">
+    <row r="52" ht="15" customHeight="1" s="11">
+      <c r="A52" s="13" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>score_display</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C52" s="13" t="inlineStr">
         <is>
           <t>CBAC Total Score: ${total_score}</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="15.75" customHeight="1" s="11">
-      <c r="A52" s="13" t="inlineStr">
+    <row r="53" ht="15" customHeight="1" s="11">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B53" s="13" t="inlineStr">
         <is>
           <t>risk_display</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>Risk Category: ${risk_category}</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1" s="11">
-      <c r="A53" s="13" t="inlineStr">
+    <row r="54" ht="15" customHeight="1" s="11">
+      <c r="A54" s="13" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B53" s="13" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
         <is>
           <t>score_high_note</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C54" s="13" t="inlineStr">
         <is>
           <t>Score is greater than 4. This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
         </is>
       </c>
-      <c r="H53" s="13" t="inlineStr">
+      <c r="H54" s="13" t="inlineStr">
         <is>
           <t>${total_score} &gt; 4</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="15.75" customHeight="1" s="11">
-      <c r="A54" s="13" t="inlineStr">
+    <row r="55" ht="15" customHeight="1" s="11">
+      <c r="A55" s="13" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
+      <c r="B55" s="13" t="inlineStr">
         <is>
           <t>score_low_note</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>Score is 4 or below. This person appears to be at low risk for NCDs at this time.</t>
         </is>
       </c>
-      <c r="H54" s="13" t="inlineStr">
+      <c r="H55" s="13" t="inlineStr">
         <is>
           <t>${total_score} &lt;= 4</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="30.75" customHeight="1" s="11">
-      <c r="A55" s="13" t="inlineStr">
+    <row r="56" ht="15" customHeight="1" s="11">
+      <c r="A56" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B55" s="13" t="inlineStr">
+      <c r="B56" s="13" t="inlineStr">
         <is>
           <t>page_score</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="30.75" customHeight="1" s="11"/>
-    <row r="57" ht="15.75" customHeight="1" s="11">
-      <c r="A57" s="13" t="inlineStr">
+    <row r="57"/>
+    <row r="58" ht="15" customFormat="1" customHeight="1" s="14">
+      <c r="A58" s="13" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B57" s="13" t="inlineStr">
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>page_3a</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
         <is>
           <t>Part B: Early Detection – Women only (1 of 3)</t>
         </is>
       </c>
-      <c r="E57" s="13" t="inlineStr">
+      <c r="E58" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="H57" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="30.75" customFormat="1" customHeight="1" s="14">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="H58" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1" s="11">
+      <c r="A59" s="13" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
+      <c r="B59" s="13" t="inlineStr">
         <is>
           <t>breast_lump</t>
         </is>
       </c>
-      <c r="C58" s="13" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>7. Lump in the breast</t>
         </is>
       </c>
-      <c r="G58" s="13" t="inlineStr">
+      <c r="G59" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H58" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="30.75" customHeight="1" s="11">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="H59" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15" customHeight="1" s="11">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>breast_lump_label</t>
         </is>
       </c>
-      <c r="F59" s="13" t="inlineStr">
+      <c r="F60" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="15.75" customHeight="1" s="11">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>nipple_discharge</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>8. Blood stained discharge from the nipple</t>
-        </is>
-      </c>
-      <c r="G60" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H60" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="11">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B61" s="13" t="inlineStr">
         <is>
-          <t>nipple_discharge_label</t>
-        </is>
-      </c>
-      <c r="F61" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
+          <t>nipple_discharge</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>8. Blood stained discharge from the nipple</t>
+        </is>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H61" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="11">
       <c r="A62" s="13" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>nipple_discharge_label</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15" customHeight="1" s="11">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B62" s="13" t="inlineStr">
+      <c r="B63" s="13" t="inlineStr">
         <is>
           <t>breast_shape_size_change</t>
         </is>
       </c>
-      <c r="C62" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>9. Change in shape and size of breast</t>
         </is>
       </c>
-      <c r="G62" s="13" t="inlineStr">
+      <c r="G63" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H62" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="30.75" customHeight="1" s="11">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15" customHeight="1" s="11">
+      <c r="A64" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B63" s="13" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>breast_shape_size_change_label</t>
         </is>
       </c>
-      <c r="F63" s="13" t="inlineStr">
+      <c r="F64" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="15.75" customHeight="1" s="11">
-      <c r="A64" s="13" t="inlineStr">
+    <row r="65" ht="15" customHeight="1" s="11">
+      <c r="A65" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
+      <c r="B65" s="13" t="inlineStr">
         <is>
           <t>page_3a</t>
         </is>
       </c>
-      <c r="H64" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="30.75" customHeight="1" s="11"/>
-    <row r="66" ht="30.75" customHeight="1" s="11">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="H65" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="66"/>
+    <row r="67" ht="15" customHeight="1" s="11">
+      <c r="A67" s="13" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
+      <c r="B67" s="13" t="inlineStr">
         <is>
           <t>page_3b</t>
         </is>
       </c>
-      <c r="C66" s="13" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>Part B: Early Detection – Women only (2 of 3)</t>
         </is>
       </c>
-      <c r="E66" s="13" t="inlineStr">
+      <c r="E67" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="H66" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="30.75" customHeight="1" s="11">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="H67" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="15" customHeight="1" s="11">
+      <c r="A68" s="13" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
         <is>
           <t>bleeding_between_periods</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C68" s="13" t="inlineStr">
         <is>
           <t>10. Bleeding between periods</t>
         </is>
       </c>
-      <c r="G67" s="13" t="inlineStr">
+      <c r="G68" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H67" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="30.75" customHeight="1" s="11">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="H68" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15" customHeight="1" s="11">
+      <c r="A69" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr">
+      <c r="B69" s="13" t="inlineStr">
         <is>
           <t>bleeding_between_periods_label</t>
         </is>
       </c>
-      <c r="F68" s="13" t="inlineStr">
+      <c r="F69" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="30.75" customHeight="1" s="11">
-      <c r="A69" s="13" t="inlineStr">
+    <row r="70" ht="15" customHeight="1" s="11">
+      <c r="A70" s="13" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B69" s="13" t="inlineStr">
+      <c r="B70" s="13" t="inlineStr">
         <is>
           <t>post_menopause_bleeding</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
+      <c r="C70" s="13" t="inlineStr">
         <is>
           <t>11. Bleeding after menopause</t>
         </is>
       </c>
-      <c r="G69" s="13" t="inlineStr">
+      <c r="G70" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H69" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="30.75" customHeight="1" s="11">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="15" customHeight="1" s="11">
+      <c r="A71" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B70" s="13" t="inlineStr">
+      <c r="B71" s="13" t="inlineStr">
         <is>
           <t>post_menopause_bleeding_label</t>
         </is>
       </c>
-      <c r="F70" s="13" t="inlineStr">
+      <c r="F71" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="30.75" customHeight="1" s="11">
-      <c r="A71" s="13" t="inlineStr">
+    <row r="72" ht="15" customHeight="1" s="11">
+      <c r="A72" s="13" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B71" s="13" t="inlineStr">
+      <c r="B72" s="13" t="inlineStr">
         <is>
           <t>post_intercourse_bleeding</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
+      <c r="C72" s="13" t="inlineStr">
         <is>
           <t>12. Bleeding after intercourse</t>
         </is>
       </c>
-      <c r="G71" s="13" t="inlineStr">
+      <c r="G72" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H71" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="30.75" customHeight="1" s="11">
-      <c r="A72" s="13" t="inlineStr">
+      <c r="H72" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="15" customHeight="1" s="11">
+      <c r="A73" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B72" s="13" t="inlineStr">
+      <c r="B73" s="13" t="inlineStr">
         <is>
           <t>post_intercourse_bleeding_label</t>
         </is>
       </c>
-      <c r="F72" s="13" t="inlineStr">
+      <c r="F73" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="30.75" customHeight="1" s="11">
-      <c r="A73" s="13" t="inlineStr">
+    <row r="74" ht="15" customHeight="1" s="11">
+      <c r="A74" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B73" s="13" t="inlineStr">
+      <c r="B74" s="13" t="inlineStr">
         <is>
           <t>page_3b</t>
         </is>
       </c>
-      <c r="H73" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="74"/>
-    <row r="75" ht="15.75" customHeight="1" s="11">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="H74" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="75"/>
+    <row r="76" ht="15" customHeight="1" s="11">
+      <c r="A76" s="13" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B75" s="13" t="inlineStr">
+      <c r="B76" s="13" t="inlineStr">
         <is>
           <t>page_3c</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
+      <c r="C76" s="13" t="inlineStr">
         <is>
           <t>Part B: Early Detection – Women only (3 of 3)</t>
         </is>
       </c>
-      <c r="E75" s="13" t="inlineStr">
+      <c r="E76" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="H75" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="15.75" customHeight="1" s="11">
-      <c r="A76" s="13" t="inlineStr">
+      <c r="H76" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="15" customHeight="1" s="11">
+      <c r="A77" s="13" t="inlineStr">
         <is>
           <t>select_one yes_no</t>
         </is>
       </c>
-      <c r="B76" s="13" t="inlineStr">
+      <c r="B77" s="13" t="inlineStr">
         <is>
           <t>foul_smelling_vaginal_discharge</t>
         </is>
       </c>
-      <c r="C76" s="13" t="inlineStr">
+      <c r="C77" s="13" t="inlineStr">
         <is>
           <t>13. Foul smelling vaginal discharge</t>
         </is>
       </c>
-      <c r="G76" s="13" t="inlineStr">
+      <c r="G77" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H76" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="30.75" customHeight="1" s="11">
-      <c r="A77" s="13" t="inlineStr">
+      <c r="H77" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="15" customHeight="1" s="11">
+      <c r="A78" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B77" s="13" t="inlineStr">
+      <c r="B78" s="13" t="inlineStr">
         <is>
           <t>foul_smelling_vaginal_discharge_label</t>
         </is>
       </c>
-      <c r="F77" s="13" t="inlineStr">
+      <c r="F78" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="15.75" customHeight="1" s="11">
-      <c r="A78" s="13" t="inlineStr">
+    <row r="79" ht="15" customHeight="1" s="11">
+      <c r="A79" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B78" s="13" t="inlineStr">
+      <c r="B79" s="13" t="inlineStr">
         <is>
           <t>page_3c</t>
         </is>
       </c>
-      <c r="H78" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="79"/>
-    <row r="80" ht="15" customHeight="1" s="11">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="H79" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="80"/>
+    <row r="81" ht="15" customHeight="1" s="11">
+      <c r="A81" s="13" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B80" s="13" t="inlineStr">
+      <c r="B81" s="13" t="inlineStr">
         <is>
           <t>page_4</t>
         </is>
       </c>
-      <c r="C80" s="13" t="inlineStr">
+      <c r="C81" s="13" t="inlineStr">
         <is>
           <t>Part C: Environmental &amp; Occupational Risk Factors</t>
         </is>
       </c>
-      <c r="E80" s="13" t="inlineStr">
+      <c r="E81" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="60.75" customHeight="1" s="11">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>select_multiple fuel_type</t>
-        </is>
-      </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>fuel_type_for_cooking</t>
-        </is>
-      </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>Type of Fuel used for cooking</t>
-        </is>
-      </c>
-      <c r="G81" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="11">
       <c r="A82" s="13" t="inlineStr">
         <is>
+          <t>select_multiple fuel_type</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>fuel_type_for_cooking</t>
+        </is>
+      </c>
+      <c r="C82" s="13" t="inlineStr">
+        <is>
+          <t>Type of Fuel used for cooking</t>
+        </is>
+      </c>
+      <c r="G82" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1" s="11">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
           <t>select_multiple occupational_exposure</t>
         </is>
       </c>
-      <c r="B82" s="13" t="inlineStr">
+      <c r="B83" s="13" t="inlineStr">
         <is>
           <t>occupational_exposure</t>
         </is>
       </c>
-      <c r="C82" s="13" t="inlineStr">
+      <c r="C83" s="13" t="inlineStr">
         <is>
           <t>Occupational exposure</t>
         </is>
       </c>
-      <c r="G82" s="13" t="inlineStr">
+      <c r="G83" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="15.75" customHeight="1" s="11">
-      <c r="A83" s="13" t="inlineStr">
+    <row r="84" ht="15" customHeight="1" s="11">
+      <c r="A84" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B83" s="13" t="inlineStr">
+      <c r="B84" s="13" t="inlineStr">
         <is>
           <t>page_4</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="15.75" customHeight="1" s="11"/>
-    <row r="85" ht="60.75" customHeight="1" s="11">
-      <c r="A85" s="13" t="inlineStr">
+    <row r="85"/>
+    <row r="86" ht="15" customHeight="1" s="11">
+      <c r="A86" s="13" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B85" s="13" t="inlineStr">
+      <c r="B86" s="13" t="inlineStr">
         <is>
           <t>page_5</t>
         </is>
       </c>
-      <c r="C85" s="13" t="inlineStr">
+      <c r="C86" s="13" t="inlineStr">
         <is>
           <t>Part D: PHQ 2</t>
         </is>
       </c>
-      <c r="E85" s="13" t="inlineStr">
+      <c r="E86" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="45.75" customHeight="1" s="11">
-      <c r="A86" s="13" t="inlineStr">
+    <row r="87" ht="15" customHeight="1" s="11">
+      <c r="A87" s="13" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B86" s="13" t="inlineStr">
+      <c r="B87" s="13" t="inlineStr">
         <is>
           <t>phq2_instructions</t>
         </is>
       </c>
-      <c r="C86" s="13" t="inlineStr">
+      <c r="C87" s="13" t="inlineStr">
         <is>
           <t>Over the last 2 weeks, how often have you been bothered by the following problems?</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="15.75" customHeight="1" s="11">
-      <c r="A87" s="13" t="inlineStr">
+    <row r="88" ht="15" customHeight="1" s="11">
+      <c r="A88" s="13" t="inlineStr">
         <is>
           <t>select_one frequency</t>
         </is>
       </c>
-      <c r="B87" s="13" t="inlineStr">
+      <c r="B88" s="13" t="inlineStr">
         <is>
           <t>phq2_q1</t>
         </is>
       </c>
-      <c r="C87" s="13" t="inlineStr">
+      <c r="C88" s="13" t="inlineStr">
         <is>
           <t>1. Little interest or pleasure in doing things?</t>
         </is>
       </c>
-      <c r="G87" s="13" t="inlineStr">
+      <c r="G88" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="15.75" customHeight="1" s="11">
-      <c r="A88" s="13" t="inlineStr">
+    <row r="89" ht="15" customHeight="1" s="11">
+      <c r="A89" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B88" s="13" t="inlineStr">
+      <c r="B89" s="13" t="inlineStr">
         <is>
           <t>phq2_q1_label</t>
         </is>
       </c>
-      <c r="C88" s="13" t="n"/>
-      <c r="F88" s="13" t="inlineStr">
+      <c r="C89" s="13" t="n"/>
+      <c r="F89" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
         </is>
       </c>
-      <c r="G88" s="13" t="n"/>
-    </row>
-    <row r="89" ht="15.75" customHeight="1" s="11">
-      <c r="A89" s="13" t="inlineStr">
+      <c r="G89" s="13" t="n"/>
+    </row>
+    <row r="90" ht="15" customHeight="1" s="11">
+      <c r="A90" s="13" t="inlineStr">
         <is>
           <t>select_one frequency</t>
         </is>
       </c>
-      <c r="B89" s="13" t="inlineStr">
+      <c r="B90" s="13" t="inlineStr">
         <is>
           <t>phq2_q2</t>
         </is>
       </c>
-      <c r="C89" s="13" t="inlineStr">
+      <c r="C90" s="13" t="inlineStr">
         <is>
           <t>2. Feeling down, depressed or hopeless?</t>
         </is>
       </c>
-      <c r="F89" s="13" t="n"/>
-      <c r="G89" s="13" t="inlineStr">
+      <c r="F90" s="13" t="n"/>
+      <c r="G90" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="15.75" customHeight="1" s="11">
-      <c r="A90" s="13" t="inlineStr">
+    <row r="91" ht="15" customHeight="1" s="11">
+      <c r="A91" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B90" s="13" t="inlineStr">
+      <c r="B91" s="13" t="inlineStr">
         <is>
           <t>phq2_q2_label</t>
         </is>
       </c>
-      <c r="F90" s="13" t="inlineStr">
+      <c r="F91" s="13" t="inlineStr">
         <is>
           <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="15.75" customHeight="1" s="11">
-      <c r="A91" s="13" t="inlineStr">
+    <row r="92" ht="15" customHeight="1" s="11">
+      <c r="A92" s="13" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B91" s="13" t="inlineStr">
+      <c r="B92" s="13" t="inlineStr">
         <is>
           <t>page_5</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="15.75" customHeight="1" s="11">
-      <c r="A92" s="13" t="inlineStr">
+    <row r="93" ht="15" customHeight="1" s="11">
+      <c r="A93" s="13" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B92" s="13" t="inlineStr">
+      <c r="B93" s="13" t="inlineStr">
         <is>
           <t>phq2_total</t>
         </is>
       </c>
-      <c r="F92" s="13" t="inlineStr">
+      <c r="F93" s="13" t="inlineStr">
         <is>
           <t>${phq2_q1} + ${phq2_q2}</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="15.75" customHeight="1" s="11">
-      <c r="A93" s="13" t="inlineStr">
+    <row r="94" ht="15" customHeight="1" s="11">
+      <c r="A94" s="13" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B93" s="13" t="inlineStr">
+      <c r="B94" s="13" t="inlineStr">
         <is>
           <t>page_5_score</t>
         </is>
       </c>
-      <c r="C93" s="13" t="inlineStr">
+      <c r="C94" s="13" t="inlineStr">
         <is>
           <t>Part D: PHQ-2 Score Summary</t>
         </is>
       </c>
-      <c r="E93" s="13" t="inlineStr">
+      <c r="E94" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="15.75" customHeight="1" s="11">
-      <c r="A94" s="13" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B94" s="13" t="inlineStr">
-        <is>
-          <t>phq2_score_display</t>
-        </is>
-      </c>
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>PHQ-2 Total Score: ${phq2_total}</t>
         </is>
       </c>
     </row>
@@ -2126,57 +2108,52 @@
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>phq2_referral_note</t>
+          <t>phq2_score_display</t>
         </is>
       </c>
       <c r="C95" s="13" t="inlineStr">
         <is>
-          <t>Anyone with total score greater than 3 should be referred to CHO/MO (PHC/UPHC)</t>
-        </is>
-      </c>
-      <c r="H95" s="13" t="inlineStr">
-        <is>
-          <t>${phq2_total} &gt; 3</t>
+          <t>PHQ-2 Total Score: ${phq2_total}</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="11">
       <c r="A96" s="13" t="inlineStr">
         <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B96" s="13" t="inlineStr">
+        <is>
+          <t>phq2_referral_note</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>Anyone with total score greater than 3 should be referred to CHO/MO (PHC/UPHC)</t>
+        </is>
+      </c>
+      <c r="H96" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total} &gt; 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15" customHeight="1" s="11">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B96" s="13" t="inlineStr">
+      <c r="B97" s="13" t="inlineStr">
         <is>
           <t>page_5_score</t>
         </is>
       </c>
-      <c r="C96" s="13" t="n"/>
-      <c r="E96" s="13" t="n"/>
-    </row>
-    <row r="97"/>
-    <row r="98" ht="15" customHeight="1" s="11">
-      <c r="A98" s="13" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B98" s="13" t="inlineStr">
-        <is>
-          <t>group_summary</t>
-        </is>
-      </c>
-      <c r="C98" s="13" t="inlineStr">
-        <is>
-          <t>Assessment Summary for CBAC Screening</t>
-        </is>
-      </c>
-      <c r="E98" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
+      <c r="C97" s="13" t="n"/>
+      <c r="E97" s="13" t="n"/>
+    </row>
+    <row r="98"/>
     <row r="99" ht="15" customHeight="1" s="11">
       <c r="A99" s="13" t="inlineStr">
         <is>
@@ -2185,7 +2162,12 @@
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>grp_filled_by</t>
+          <t>group_summary</t>
+        </is>
+      </c>
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>Assessment Summary for CBAC Screening</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
@@ -2197,1758 +2179,1753 @@
     <row r="100" ht="15" customHeight="1" s="11">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>lbl_filled_by</t>
-        </is>
-      </c>
-      <c r="C100" s="13" t="inlineStr">
-        <is>
-          <t>**Filled by:** ${reporter_name}</t>
+          <t>grp_filled_by</t>
+        </is>
+      </c>
+      <c r="E100" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="11">
       <c r="A101" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>calc_reporter</t>
-        </is>
-      </c>
-      <c r="F101" s="13" t="inlineStr">
-        <is>
-          <t>${reporter_name}</t>
+          <t>lbl_filled_by</t>
+        </is>
+      </c>
+      <c r="C101" s="13" t="inlineStr">
+        <is>
+          <t>**Filled by:** ${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="11">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>grp_filled_by</t>
+          <t>calc_reporter</t>
+        </is>
+      </c>
+      <c r="F102" s="13" t="inlineStr">
+        <is>
+          <t>${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="11">
       <c r="A103" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>grp_patient</t>
-        </is>
-      </c>
-      <c r="E103" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_filled_by</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="11">
       <c r="A104" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
-          <t>lbl_patient</t>
-        </is>
-      </c>
-      <c r="C104" s="13" t="inlineStr">
-        <is>
-          <t>**Patient:** ${patient_name}</t>
+          <t>grp_patient</t>
+        </is>
+      </c>
+      <c r="E104" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="11">
       <c r="A105" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>calc_patient</t>
-        </is>
-      </c>
-      <c r="F105" s="13" t="inlineStr">
-        <is>
-          <t>${patient_name}</t>
+          <t>lbl_patient</t>
+        </is>
+      </c>
+      <c r="C105" s="13" t="inlineStr">
+        <is>
+          <t>**Patient:** ${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="11">
       <c r="A106" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>grp_patient</t>
+          <t>calc_patient</t>
+        </is>
+      </c>
+      <c r="F106" s="13" t="inlineStr">
+        <is>
+          <t>${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="11">
       <c r="A107" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>grp_gender</t>
-        </is>
-      </c>
-      <c r="E107" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_patient</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="11">
       <c r="A108" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
-          <t>lbl_gender</t>
-        </is>
-      </c>
-      <c r="C108" s="13" t="inlineStr">
-        <is>
-          <t>**Gender:** ${gender}</t>
+          <t>grp_gender</t>
+        </is>
+      </c>
+      <c r="E108" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="11">
       <c r="A109" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>calc_gender</t>
-        </is>
-      </c>
-      <c r="F109" s="13" t="inlineStr">
-        <is>
-          <t>${gender}</t>
+          <t>lbl_gender</t>
+        </is>
+      </c>
+      <c r="C109" s="13" t="inlineStr">
+        <is>
+          <t>**Gender:** ${calc_gender}</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="11">
       <c r="A110" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>grp_gender</t>
+          <t>calc_gender</t>
+        </is>
+      </c>
+      <c r="F110" s="13" t="inlineStr">
+        <is>
+          <t>if(${patient_gender} = 'male', 'Male', 'Female')</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="11">
       <c r="A111" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>grp_state</t>
-        </is>
-      </c>
-      <c r="E111" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_gender</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="11">
       <c r="A112" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>lbl_state</t>
-        </is>
-      </c>
-      <c r="C112" s="13" t="inlineStr">
-        <is>
-          <t>**State:** ${state}</t>
+          <t>grp_state</t>
+        </is>
+      </c>
+      <c r="E112" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="11">
       <c r="A113" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>calc_state</t>
-        </is>
-      </c>
-      <c r="F113" s="13" t="inlineStr">
-        <is>
-          <t>${state}</t>
+          <t>lbl_state</t>
+        </is>
+      </c>
+      <c r="C113" s="13" t="inlineStr">
+        <is>
+          <t>**State:** ${state}</t>
         </is>
       </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="11">
       <c r="A114" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>grp_state</t>
+          <t>calc_state</t>
+        </is>
+      </c>
+      <c r="F114" s="13" t="inlineStr">
+        <is>
+          <t>${state}</t>
         </is>
       </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="11">
       <c r="A115" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>grp_district</t>
-        </is>
-      </c>
-      <c r="E115" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_state</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="11">
       <c r="A116" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>lbl_district</t>
-        </is>
-      </c>
-      <c r="C116" s="13" t="inlineStr">
-        <is>
-          <t>**District:** ${district}</t>
+          <t>grp_district</t>
+        </is>
+      </c>
+      <c r="E116" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="11">
       <c r="A117" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>calc_district</t>
-        </is>
-      </c>
-      <c r="F117" s="13" t="inlineStr">
-        <is>
-          <t>${district}</t>
+          <t>lbl_district</t>
+        </is>
+      </c>
+      <c r="C117" s="13" t="inlineStr">
+        <is>
+          <t>**District:** ${district}</t>
         </is>
       </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="11">
       <c r="A118" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>grp_district</t>
+          <t>calc_district</t>
+        </is>
+      </c>
+      <c r="F118" s="13" t="inlineStr">
+        <is>
+          <t>${district}</t>
         </is>
       </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="11">
       <c r="A119" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>grp_score</t>
-        </is>
-      </c>
-      <c r="E119" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_district</t>
         </is>
       </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="11">
       <c r="A120" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>lbl_score</t>
-        </is>
-      </c>
-      <c r="C120" s="13" t="inlineStr">
-        <is>
-          <t>**CBAC Total Score:** ${total_score}</t>
+          <t>grp_score</t>
+        </is>
+      </c>
+      <c r="E120" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="11">
       <c r="A121" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>calc_score</t>
-        </is>
-      </c>
-      <c r="F121" s="13" t="inlineStr">
-        <is>
-          <t>${total_score}</t>
+          <t>lbl_score</t>
+        </is>
+      </c>
+      <c r="C121" s="13" t="inlineStr">
+        <is>
+          <t>**CBAC Total Score:** ${total_score}</t>
         </is>
       </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="11">
       <c r="A122" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>grp_score</t>
+          <t>calc_score</t>
+        </is>
+      </c>
+      <c r="F122" s="13" t="inlineStr">
+        <is>
+          <t>${total_score}</t>
         </is>
       </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="11">
       <c r="A123" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>grp_risk</t>
-        </is>
-      </c>
-      <c r="E123" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_score</t>
         </is>
       </c>
     </row>
     <row r="124" ht="15" customHeight="1" s="11">
       <c r="A124" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>lbl_risk</t>
-        </is>
-      </c>
-      <c r="C124" s="13" t="inlineStr">
-        <is>
-          <t>**Risk Category:** ${risk_category}</t>
+          <t>grp_risk</t>
+        </is>
+      </c>
+      <c r="E124" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="11">
       <c r="A125" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
-          <t>calc_risk</t>
-        </is>
-      </c>
-      <c r="F125" s="13" t="inlineStr">
-        <is>
-          <t>${risk_category}</t>
+          <t>lbl_risk</t>
+        </is>
+      </c>
+      <c r="C125" s="13" t="inlineStr">
+        <is>
+          <t>**Risk Category:** ${risk_category}</t>
         </is>
       </c>
     </row>
     <row r="126" ht="15" customHeight="1" s="11">
       <c r="A126" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
-          <t>grp_risk</t>
+          <t>calc_risk</t>
+        </is>
+      </c>
+      <c r="F126" s="13" t="inlineStr">
+        <is>
+          <t>${risk_category}</t>
         </is>
       </c>
     </row>
     <row r="127" ht="15" customHeight="1" s="11">
       <c r="A127" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B127" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_a</t>
-        </is>
-      </c>
-      <c r="C127" s="13" t="inlineStr">
-        <is>
-          <t>**Part A: Risk Assessment**</t>
+          <t>grp_risk</t>
         </is>
       </c>
     </row>
     <row r="128" ht="15" customHeight="1" s="11">
       <c r="A128" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B128" s="13" t="inlineStr">
         <is>
-          <t>grp_q_age</t>
-        </is>
-      </c>
-      <c r="E128" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>sum_hdr_a</t>
+        </is>
+      </c>
+      <c r="C128" s="13" t="inlineStr">
+        <is>
+          <t>**Part A: Risk Assessment**</t>
         </is>
       </c>
     </row>
     <row r="129" ht="15" customHeight="1" s="11">
       <c r="A129" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B129" s="13" t="inlineStr">
         <is>
-          <t>q_age</t>
-        </is>
-      </c>
-      <c r="C129" s="13" t="inlineStr">
-        <is>
-          <t>1. Age: ${calc_q_age}</t>
+          <t>grp_q_age</t>
+        </is>
+      </c>
+      <c r="E129" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="130" ht="15" customHeight="1" s="11">
       <c r="A130" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B130" s="13" t="inlineStr">
         <is>
-          <t>calc_q_age</t>
-        </is>
-      </c>
-      <c r="F130" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${age_range}, '${age_range}')</t>
+          <t>q_age</t>
+        </is>
+      </c>
+      <c r="C130" s="13" t="inlineStr">
+        <is>
+          <t>1. Age: ${calc_q_age}</t>
         </is>
       </c>
     </row>
     <row r="131" ht="15" customHeight="1" s="11">
       <c r="A131" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B131" s="13" t="inlineStr">
         <is>
-          <t>grp_q_age</t>
+          <t>calc_q_age</t>
+        </is>
+      </c>
+      <c r="F131" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${age_range}, '${age_range}')</t>
         </is>
       </c>
     </row>
     <row r="132" ht="15" customHeight="1" s="11">
       <c r="A132" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B132" s="13" t="inlineStr">
         <is>
-          <t>grp_q_smoke</t>
-        </is>
-      </c>
-      <c r="E132" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_age</t>
         </is>
       </c>
     </row>
     <row r="133" ht="15" customHeight="1" s="11">
       <c r="A133" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B133" s="13" t="inlineStr">
         <is>
-          <t>q_smoke</t>
-        </is>
-      </c>
-      <c r="C133" s="13" t="inlineStr">
-        <is>
-          <t>2. Smoke/Smokeless products: ${calc_q_smoke}</t>
+          <t>grp_q_smoke</t>
+        </is>
+      </c>
+      <c r="E133" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="134" ht="15" customHeight="1" s="11">
       <c r="A134" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B134" s="13" t="inlineStr">
         <is>
-          <t>calc_q_smoke</t>
-        </is>
-      </c>
-      <c r="F134" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${smoke_frequency}, '${smoke_frequency}')</t>
+          <t>q_smoke</t>
+        </is>
+      </c>
+      <c r="C134" s="13" t="inlineStr">
+        <is>
+          <t>2. Smoke/Smokeless products: ${calc_q_smoke}</t>
         </is>
       </c>
     </row>
     <row r="135" ht="15" customHeight="1" s="11">
       <c r="A135" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B135" s="13" t="inlineStr">
         <is>
-          <t>grp_q_smoke</t>
+          <t>calc_q_smoke</t>
+        </is>
+      </c>
+      <c r="F135" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${smoke_frequency}, '${smoke_frequency}')</t>
         </is>
       </c>
     </row>
     <row r="136" ht="15" customHeight="1" s="11">
       <c r="A136" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B136" s="13" t="inlineStr">
         <is>
-          <t>grp_q_alcohol</t>
-        </is>
-      </c>
-      <c r="E136" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_smoke</t>
         </is>
       </c>
     </row>
     <row r="137" ht="15" customHeight="1" s="11">
       <c r="A137" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B137" s="13" t="inlineStr">
         <is>
-          <t>q_alcohol</t>
-        </is>
-      </c>
-      <c r="C137" s="13" t="inlineStr">
-        <is>
-          <t>3. Alcohol daily: ${calc_q_alcohol}</t>
+          <t>grp_q_alcohol</t>
+        </is>
+      </c>
+      <c r="E137" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="138" ht="15" customHeight="1" s="11">
       <c r="A138" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B138" s="13" t="inlineStr">
         <is>
-          <t>calc_q_alcohol</t>
-        </is>
-      </c>
-      <c r="F138" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${alcohol_frequency}, '${alcohol_frequency}')</t>
+          <t>q_alcohol</t>
+        </is>
+      </c>
+      <c r="C138" s="13" t="inlineStr">
+        <is>
+          <t>3. Alcohol daily: ${calc_q_alcohol}</t>
         </is>
       </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="11">
       <c r="A139" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B139" s="13" t="inlineStr">
         <is>
-          <t>grp_q_alcohol</t>
+          <t>calc_q_alcohol</t>
+        </is>
+      </c>
+      <c r="F139" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${alcohol_frequency}, '${alcohol_frequency}')</t>
         </is>
       </c>
     </row>
     <row r="140" ht="15" customHeight="1" s="11">
       <c r="A140" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B140" s="13" t="inlineStr">
         <is>
-          <t>grp_q_waist</t>
-        </is>
-      </c>
-      <c r="E140" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_alcohol</t>
         </is>
       </c>
     </row>
     <row r="141" ht="15" customHeight="1" s="11">
       <c r="A141" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B141" s="13" t="inlineStr">
         <is>
-          <t>q_waist</t>
-        </is>
-      </c>
-      <c r="C141" s="13" t="inlineStr">
-        <is>
-          <t>4. Waist measurement: ${calc_q_waist}</t>
+          <t>grp_q_waist</t>
+        </is>
+      </c>
+      <c r="E141" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="142" ht="15" customHeight="1" s="11">
       <c r="A142" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B142" s="13" t="inlineStr">
         <is>
-          <t>calc_q_waist</t>
-        </is>
-      </c>
-      <c r="F142" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${waist_size}, '${waist_size}')</t>
+          <t>q_waist</t>
+        </is>
+      </c>
+      <c r="C142" s="13" t="inlineStr">
+        <is>
+          <t>4. Waist measurement: ${calc_q_waist}</t>
         </is>
       </c>
     </row>
     <row r="143" ht="15" customHeight="1" s="11">
       <c r="A143" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B143" s="13" t="inlineStr">
         <is>
-          <t>grp_q_waist</t>
+          <t>calc_q_waist</t>
+        </is>
+      </c>
+      <c r="F143" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${waist_size}, '${waist_size}')</t>
         </is>
       </c>
     </row>
     <row r="144" ht="15" customHeight="1" s="11">
       <c r="A144" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B144" s="13" t="inlineStr">
         <is>
-          <t>grp_q_physical</t>
-        </is>
-      </c>
-      <c r="E144" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_waist</t>
         </is>
       </c>
     </row>
     <row r="145" ht="15" customHeight="1" s="11">
       <c r="A145" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B145" s="13" t="inlineStr">
         <is>
-          <t>q_physical</t>
-        </is>
-      </c>
-      <c r="C145" s="13" t="inlineStr">
-        <is>
-          <t>5. Physical activity (150 min/week): ${calc_q_physical}</t>
+          <t>grp_q_physical</t>
+        </is>
+      </c>
+      <c r="E145" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="146" ht="15" customHeight="1" s="11">
       <c r="A146" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B146" s="13" t="inlineStr">
         <is>
-          <t>calc_q_physical</t>
-        </is>
-      </c>
-      <c r="F146" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${physical_activities_frequency}, '${physical_activities_frequency}')</t>
+          <t>q_physical</t>
+        </is>
+      </c>
+      <c r="C146" s="13" t="inlineStr">
+        <is>
+          <t>5. Physical activity (150 min/week): ${calc_q_physical}</t>
         </is>
       </c>
     </row>
     <row r="147" ht="15" customHeight="1" s="11">
       <c r="A147" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B147" s="13" t="inlineStr">
         <is>
-          <t>grp_q_physical</t>
+          <t>calc_q_physical</t>
+        </is>
+      </c>
+      <c r="F147" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${physical_activities_frequency}, '${physical_activities_frequency}')</t>
         </is>
       </c>
     </row>
     <row r="148" ht="15" customHeight="1" s="11">
       <c r="A148" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B148" s="13" t="inlineStr">
         <is>
-          <t>grp_q_family</t>
-        </is>
-      </c>
-      <c r="E148" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_physical</t>
         </is>
       </c>
     </row>
     <row r="149" ht="15" customHeight="1" s="11">
       <c r="A149" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B149" s="13" t="inlineStr">
         <is>
-          <t>q_family</t>
-        </is>
-      </c>
-      <c r="C149" s="13" t="inlineStr">
-        <is>
-          <t>6. Family history of BP/Diabetes/Heart disease: ${calc_q_family}</t>
+          <t>grp_q_family</t>
+        </is>
+      </c>
+      <c r="E149" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="150" ht="15" customHeight="1" s="11">
       <c r="A150" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B150" s="13" t="inlineStr">
         <is>
-          <t>calc_q_family</t>
-        </is>
-      </c>
-      <c r="F150" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${family_medical_history}, '${family_medical_history}')</t>
+          <t>q_family</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="inlineStr">
+        <is>
+          <t>6. Family history of BP/Diabetes/Heart disease: ${calc_q_family}</t>
         </is>
       </c>
     </row>
     <row r="151" ht="15" customHeight="1" s="11">
       <c r="A151" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B151" s="13" t="inlineStr">
         <is>
-          <t>grp_q_family</t>
+          <t>calc_q_family</t>
+        </is>
+      </c>
+      <c r="F151" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${family_medical_history}, '${family_medical_history}')</t>
         </is>
       </c>
     </row>
     <row r="152" ht="15" customHeight="1" s="11">
       <c r="A152" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B152" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_b</t>
-        </is>
-      </c>
-      <c r="C152" s="13" t="inlineStr">
-        <is>
-          <t>**Part B: Early Detection**</t>
-        </is>
-      </c>
-      <c r="H152" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>grp_q_family</t>
         </is>
       </c>
     </row>
     <row r="153" ht="15" customHeight="1" s="11">
       <c r="A153" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B153" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_lump</t>
-        </is>
-      </c>
-      <c r="E153" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>sum_hdr_b</t>
+        </is>
+      </c>
+      <c r="C153" s="13" t="inlineStr">
+        <is>
+          <t>**Part B: Early Detection**</t>
         </is>
       </c>
       <c r="H153" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="154" ht="15" customHeight="1" s="11">
       <c r="A154" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B154" s="13" t="inlineStr">
         <is>
-          <t>q_breast_lump</t>
-        </is>
-      </c>
-      <c r="C154" s="13" t="inlineStr">
-        <is>
-          <t>7. Lump in the breast: ${calc_q_breast_lump}</t>
+          <t>grp_q_breast_lump</t>
+        </is>
+      </c>
+      <c r="E154" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H154" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="155" ht="15" customHeight="1" s="11">
       <c r="A155" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B155" s="13" t="inlineStr">
         <is>
-          <t>calc_q_breast_lump</t>
-        </is>
-      </c>
-      <c r="F155" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
+          <t>q_breast_lump</t>
+        </is>
+      </c>
+      <c r="C155" s="13" t="inlineStr">
+        <is>
+          <t>7. Lump in the breast: ${calc_q_breast_lump}</t>
+        </is>
+      </c>
+      <c r="H155" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="156" ht="15" customHeight="1" s="11">
       <c r="A156" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B156" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_lump</t>
-        </is>
-      </c>
-      <c r="H156" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_q_breast_lump</t>
+        </is>
+      </c>
+      <c r="F156" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
         </is>
       </c>
     </row>
     <row r="157" ht="15" customHeight="1" s="11">
       <c r="A157" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B157" s="13" t="inlineStr">
         <is>
-          <t>grp_q_nipple</t>
-        </is>
-      </c>
-      <c r="E157" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_breast_lump</t>
         </is>
       </c>
       <c r="H157" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="11">
       <c r="A158" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B158" s="13" t="inlineStr">
         <is>
-          <t>q_nipple</t>
-        </is>
-      </c>
-      <c r="C158" s="13" t="inlineStr">
-        <is>
-          <t>8. Blood stained nipple discharge: ${calc_q_nipple}</t>
+          <t>grp_q_nipple</t>
+        </is>
+      </c>
+      <c r="E158" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H158" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="159" ht="15" customHeight="1" s="11">
       <c r="A159" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B159" s="13" t="inlineStr">
         <is>
-          <t>calc_q_nipple</t>
-        </is>
-      </c>
-      <c r="F159" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
+          <t>q_nipple</t>
+        </is>
+      </c>
+      <c r="C159" s="13" t="inlineStr">
+        <is>
+          <t>8. Blood stained nipple discharge: ${calc_q_nipple}</t>
+        </is>
+      </c>
+      <c r="H159" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="160" ht="15" customHeight="1" s="11">
       <c r="A160" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B160" s="13" t="inlineStr">
         <is>
-          <t>grp_q_nipple</t>
-        </is>
-      </c>
-      <c r="H160" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_q_nipple</t>
+        </is>
+      </c>
+      <c r="F160" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
         </is>
       </c>
     </row>
     <row r="161" ht="15" customHeight="1" s="11">
       <c r="A161" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B161" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_shape</t>
-        </is>
-      </c>
-      <c r="E161" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_nipple</t>
         </is>
       </c>
       <c r="H161" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="162" ht="15" customHeight="1" s="11">
       <c r="A162" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B162" s="13" t="inlineStr">
         <is>
-          <t>q_breast_shape</t>
-        </is>
-      </c>
-      <c r="C162" s="13" t="inlineStr">
-        <is>
-          <t>9. Change in breast shape/size: ${calc_q_breast_shape}</t>
+          <t>grp_q_breast_shape</t>
+        </is>
+      </c>
+      <c r="E162" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H162" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="163" ht="15" customHeight="1" s="11">
       <c r="A163" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B163" s="13" t="inlineStr">
         <is>
-          <t>calc_q_breast_shape</t>
-        </is>
-      </c>
-      <c r="F163" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
+          <t>q_breast_shape</t>
+        </is>
+      </c>
+      <c r="C163" s="13" t="inlineStr">
+        <is>
+          <t>9. Change in breast shape/size: ${calc_q_breast_shape}</t>
+        </is>
+      </c>
+      <c r="H163" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="164" ht="15" customHeight="1" s="11">
       <c r="A164" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B164" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_shape</t>
-        </is>
-      </c>
-      <c r="H164" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_q_breast_shape</t>
+        </is>
+      </c>
+      <c r="F164" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
         </is>
       </c>
     </row>
     <row r="165" ht="15" customHeight="1" s="11">
       <c r="A165" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B165" s="13" t="inlineStr">
         <is>
-          <t>grp_q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="E165" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_breast_shape</t>
         </is>
       </c>
       <c r="H165" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="166" ht="15" customHeight="1" s="11">
       <c r="A166" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B166" s="13" t="inlineStr">
         <is>
-          <t>q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="C166" s="13" t="inlineStr">
-        <is>
-          <t>10. Bleeding between periods: ${calc_q_bleeding_periods}</t>
+          <t>grp_q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="E166" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H166" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="167" ht="15" customHeight="1" s="11">
       <c r="A167" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B167" s="13" t="inlineStr">
         <is>
-          <t>calc_q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="F167" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
+          <t>q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="C167" s="13" t="inlineStr">
+        <is>
+          <t>10. Bleeding between periods: ${calc_q_bleeding_periods}</t>
+        </is>
+      </c>
+      <c r="H167" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="168" ht="15" customHeight="1" s="11">
       <c r="A168" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B168" s="13" t="inlineStr">
         <is>
-          <t>grp_q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="H168" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="F168" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
         </is>
       </c>
     </row>
     <row r="169" ht="15" customHeight="1" s="11">
       <c r="A169" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B169" s="13" t="inlineStr">
         <is>
-          <t>grp_q_menopause</t>
-        </is>
-      </c>
-      <c r="E169" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_bleeding_periods</t>
         </is>
       </c>
       <c r="H169" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="170" ht="15" customHeight="1" s="11">
       <c r="A170" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B170" s="13" t="inlineStr">
         <is>
-          <t>q_menopause</t>
-        </is>
-      </c>
-      <c r="C170" s="13" t="inlineStr">
-        <is>
-          <t>11. Bleeding after menopause: ${calc_q_menopause}</t>
+          <t>grp_q_menopause</t>
+        </is>
+      </c>
+      <c r="E170" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H170" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="171" ht="15" customHeight="1" s="11">
       <c r="A171" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B171" s="13" t="inlineStr">
         <is>
-          <t>calc_q_menopause</t>
-        </is>
-      </c>
-      <c r="F171" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
+          <t>q_menopause</t>
+        </is>
+      </c>
+      <c r="C171" s="13" t="inlineStr">
+        <is>
+          <t>11. Bleeding after menopause: ${calc_q_menopause}</t>
+        </is>
+      </c>
+      <c r="H171" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="172" ht="15" customHeight="1" s="11">
       <c r="A172" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B172" s="13" t="inlineStr">
         <is>
-          <t>grp_q_menopause</t>
-        </is>
-      </c>
-      <c r="H172" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_q_menopause</t>
+        </is>
+      </c>
+      <c r="F172" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
         </is>
       </c>
     </row>
     <row r="173" ht="15" customHeight="1" s="11">
       <c r="A173" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B173" s="13" t="inlineStr">
         <is>
-          <t>grp_q_intercourse</t>
-        </is>
-      </c>
-      <c r="E173" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_menopause</t>
         </is>
       </c>
       <c r="H173" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="174" ht="15" customHeight="1" s="11">
       <c r="A174" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B174" s="13" t="inlineStr">
         <is>
-          <t>q_intercourse</t>
-        </is>
-      </c>
-      <c r="C174" s="13" t="inlineStr">
-        <is>
-          <t>12. Bleeding after intercourse: ${calc_q_intercourse}</t>
+          <t>grp_q_intercourse</t>
+        </is>
+      </c>
+      <c r="E174" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H174" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="175" ht="15" customHeight="1" s="11">
       <c r="A175" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B175" s="13" t="inlineStr">
         <is>
-          <t>calc_q_intercourse</t>
-        </is>
-      </c>
-      <c r="F175" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
+          <t>q_intercourse</t>
+        </is>
+      </c>
+      <c r="C175" s="13" t="inlineStr">
+        <is>
+          <t>12. Bleeding after intercourse: ${calc_q_intercourse}</t>
+        </is>
+      </c>
+      <c r="H175" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="176" ht="15" customHeight="1" s="11">
       <c r="A176" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B176" s="13" t="inlineStr">
         <is>
-          <t>grp_q_intercourse</t>
-        </is>
-      </c>
-      <c r="H176" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_q_intercourse</t>
+        </is>
+      </c>
+      <c r="F176" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
         </is>
       </c>
     </row>
     <row r="177" ht="15" customHeight="1" s="11">
       <c r="A177" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B177" s="13" t="inlineStr">
         <is>
-          <t>grp_q_discharge</t>
-        </is>
-      </c>
-      <c r="E177" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_intercourse</t>
         </is>
       </c>
       <c r="H177" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="178" ht="15" customHeight="1" s="11">
       <c r="A178" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B178" s="13" t="inlineStr">
         <is>
-          <t>q_discharge</t>
-        </is>
-      </c>
-      <c r="C178" s="13" t="inlineStr">
-        <is>
-          <t>13. Foul smelling vaginal discharge: ${calc_q_discharge}</t>
+          <t>grp_q_discharge</t>
+        </is>
+      </c>
+      <c r="E178" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H178" s="13" t="inlineStr">
         <is>
-          <t>${gender} = 'female'</t>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="179" ht="15" customHeight="1" s="11">
       <c r="A179" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B179" s="13" t="inlineStr">
         <is>
-          <t>calc_q_discharge</t>
-        </is>
-      </c>
-      <c r="F179" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
+          <t>q_discharge</t>
+        </is>
+      </c>
+      <c r="C179" s="13" t="inlineStr">
+        <is>
+          <t>13. Foul smelling vaginal discharge: ${calc_q_discharge}</t>
+        </is>
+      </c>
+      <c r="H179" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="180" ht="15" customHeight="1" s="11">
       <c r="A180" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B180" s="13" t="inlineStr">
         <is>
-          <t>grp_q_discharge</t>
-        </is>
-      </c>
-      <c r="H180" s="13" t="inlineStr">
-        <is>
-          <t>${gender} = 'female'</t>
+          <t>calc_q_discharge</t>
+        </is>
+      </c>
+      <c r="F180" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
         </is>
       </c>
     </row>
     <row r="181" ht="15" customHeight="1" s="11">
       <c r="A181" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B181" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_c</t>
-        </is>
-      </c>
-      <c r="C181" s="13" t="inlineStr">
-        <is>
-          <t>**Part C: Environmental &amp; Occupational Risk Factors**</t>
+          <t>grp_q_discharge</t>
+        </is>
+      </c>
+      <c r="H181" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="182" ht="15" customHeight="1" s="11">
       <c r="A182" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B182" s="13" t="inlineStr">
         <is>
-          <t>grp_q_fuel</t>
-        </is>
-      </c>
-      <c r="E182" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>sum_hdr_c</t>
+        </is>
+      </c>
+      <c r="C182" s="13" t="inlineStr">
+        <is>
+          <t>**Part C: Environmental &amp; Occupational Risk Factors**</t>
         </is>
       </c>
     </row>
     <row r="183" ht="15" customHeight="1" s="11">
       <c r="A183" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B183" s="13" t="inlineStr">
         <is>
-          <t>q_fuel</t>
-        </is>
-      </c>
-      <c r="C183" s="13" t="inlineStr">
-        <is>
-          <t>Fuel used for cooking: ${calc_q_fuel}</t>
+          <t>grp_q_fuel</t>
+        </is>
+      </c>
+      <c r="E183" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="184" ht="15" customHeight="1" s="11">
       <c r="A184" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B184" s="13" t="inlineStr">
         <is>
-          <t>calc_q_fuel</t>
-        </is>
-      </c>
-      <c r="F184" s="13" t="inlineStr">
-        <is>
-          <t>concat(if(selected(${fuel_type_for_cooking}, 'firewood'), 'Firewood', ''), if(selected(${fuel_type_for_cooking}, 'firewood') and string-length(${fuel_type_for_cooking}) &gt; 9, ' / ', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue'), 'Crop Residue', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue') and (selected(${fuel_type_for_cooking}, 'cow_dung_cake') or selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake'), 'Cow dung cake', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake') and (selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'coal'), 'Coal', ''), if(selected(${fuel_type_for_cooking}, 'coal') and (selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'kerosene'), 'Kerosene', ''), if(selected(${fuel_type_for_cooking}, 'kerosene') and selected(${fuel_type_for_cooking}, 'lpg'), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'lpg'), 'LPG', ''))</t>
+          <t>q_fuel</t>
+        </is>
+      </c>
+      <c r="C184" s="13" t="inlineStr">
+        <is>
+          <t>Fuel used for cooking: ${calc_q_fuel}</t>
         </is>
       </c>
     </row>
     <row r="185" ht="15" customHeight="1" s="11">
       <c r="A185" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B185" s="13" t="inlineStr">
         <is>
-          <t>grp_q_fuel</t>
+          <t>calc_q_fuel</t>
+        </is>
+      </c>
+      <c r="F185" s="13" t="inlineStr">
+        <is>
+          <t>concat(if(selected(${fuel_type_for_cooking}, 'firewood'), 'Firewood', ''), if(selected(${fuel_type_for_cooking}, 'firewood') and string-length(${fuel_type_for_cooking}) &gt; 9, ' / ', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue'), 'Crop Residue', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue') and (selected(${fuel_type_for_cooking}, 'cow_dung_cake') or selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake'), 'Cow dung cake', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake') and (selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'coal'), 'Coal', ''), if(selected(${fuel_type_for_cooking}, 'coal') and (selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'kerosene'), 'Kerosene', ''), if(selected(${fuel_type_for_cooking}, 'kerosene') and selected(${fuel_type_for_cooking}, 'lpg'), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'lpg'), 'LPG', ''))</t>
         </is>
       </c>
     </row>
     <row r="186" ht="15" customHeight="1" s="11">
       <c r="A186" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B186" s="13" t="inlineStr">
         <is>
-          <t>grp_q_occupation</t>
-        </is>
-      </c>
-      <c r="E186" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_fuel</t>
         </is>
       </c>
     </row>
     <row r="187" ht="15" customHeight="1" s="11">
       <c r="A187" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B187" s="13" t="inlineStr">
         <is>
-          <t>q_occupation</t>
-        </is>
-      </c>
-      <c r="C187" s="13" t="inlineStr">
-        <is>
-          <t>Occupational exposure: ${calc_q_occupation}</t>
+          <t>grp_q_occupation</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="188" ht="15" customHeight="1" s="11">
       <c r="A188" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B188" s="13" t="inlineStr">
         <is>
-          <t>calc_q_occupation</t>
-        </is>
-      </c>
-      <c r="F188" s="13" t="inlineStr">
-        <is>
-          <t>concat(if(selected(${occupational_exposure}, 'crop_residue_burning'), 'Crop residue burning', ''), if(selected(${occupational_exposure}, 'crop_residue_burning') and (selected(${occupational_exposure}, 'working_in_industries') or selected(${occupational_exposure}, 'none')), ' / ', ''), if(selected(${occupational_exposure}, 'working_in_industries'), 'Working in industries', ''), if(selected(${occupational_exposure}, 'working_in_industries') and selected(${occupational_exposure}, 'none'), ' / ', ''), if(selected(${occupational_exposure}, 'none'), 'None of the above', ''))</t>
+          <t>q_occupation</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="inlineStr">
+        <is>
+          <t>Occupational exposure: ${calc_q_occupation}</t>
         </is>
       </c>
     </row>
     <row r="189" ht="15" customHeight="1" s="11">
       <c r="A189" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B189" s="13" t="inlineStr">
         <is>
-          <t>grp_q_occupation</t>
+          <t>calc_q_occupation</t>
+        </is>
+      </c>
+      <c r="F189" s="13" t="inlineStr">
+        <is>
+          <t>concat(if(selected(${occupational_exposure}, 'crop_residue_burning'), 'Crop residue burning', ''), if(selected(${occupational_exposure}, 'crop_residue_burning') and (selected(${occupational_exposure}, 'working_in_industries') or selected(${occupational_exposure}, 'none')), ' / ', ''), if(selected(${occupational_exposure}, 'working_in_industries'), 'Working in industries', ''), if(selected(${occupational_exposure}, 'working_in_industries') and selected(${occupational_exposure}, 'none'), ' / ', ''), if(selected(${occupational_exposure}, 'none'), 'None of the above', ''))</t>
         </is>
       </c>
     </row>
     <row r="190" ht="15" customHeight="1" s="11">
       <c r="A190" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B190" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_d</t>
-        </is>
-      </c>
-      <c r="C190" s="13" t="inlineStr">
-        <is>
-          <t>**Part D: PHQ-2**</t>
+          <t>grp_q_occupation</t>
         </is>
       </c>
     </row>
     <row r="191" ht="15" customHeight="1" s="11">
       <c r="A191" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B191" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq1</t>
-        </is>
-      </c>
-      <c r="E191" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>sum_hdr_d</t>
+        </is>
+      </c>
+      <c r="C191" s="13" t="inlineStr">
+        <is>
+          <t>**Part D: PHQ-2**</t>
         </is>
       </c>
     </row>
     <row r="192" ht="15" customHeight="1" s="11">
       <c r="A192" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B192" s="13" t="inlineStr">
         <is>
-          <t>q_phq1</t>
-        </is>
-      </c>
-      <c r="C192" s="13" t="inlineStr">
-        <is>
-          <t>1. Little interest or pleasure in doing things: ${calc_q_phq1}</t>
+          <t>grp_q_phq1</t>
+        </is>
+      </c>
+      <c r="E192" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="193" ht="15" customHeight="1" s="11">
       <c r="A193" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B193" s="13" t="inlineStr">
         <is>
-          <t>calc_q_phq1</t>
-        </is>
-      </c>
-      <c r="F193" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
+          <t>q_phq1</t>
+        </is>
+      </c>
+      <c r="C193" s="13" t="inlineStr">
+        <is>
+          <t>1. Little interest or pleasure in doing things: ${calc_q_phq1}</t>
         </is>
       </c>
     </row>
     <row r="194" ht="15" customHeight="1" s="11">
       <c r="A194" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B194" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq1</t>
+          <t>calc_q_phq1</t>
+        </is>
+      </c>
+      <c r="F194" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
         </is>
       </c>
     </row>
     <row r="195" ht="15" customHeight="1" s="11">
       <c r="A195" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B195" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq2</t>
-        </is>
-      </c>
-      <c r="E195" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_phq1</t>
         </is>
       </c>
     </row>
     <row r="196" ht="15" customHeight="1" s="11">
       <c r="A196" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B196" s="13" t="inlineStr">
         <is>
-          <t>q_phq2</t>
-        </is>
-      </c>
-      <c r="C196" s="13" t="inlineStr">
-        <is>
-          <t>2. Feeling down, depressed or hopeless: ${calc_q_phq2}</t>
+          <t>grp_q_phq2</t>
+        </is>
+      </c>
+      <c r="E196" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="197" ht="15" customHeight="1" s="11">
       <c r="A197" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B197" s="13" t="inlineStr">
         <is>
-          <t>calc_q_phq2</t>
-        </is>
-      </c>
-      <c r="F197" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
+          <t>q_phq2</t>
+        </is>
+      </c>
+      <c r="C197" s="13" t="inlineStr">
+        <is>
+          <t>2. Feeling down, depressed or hopeless: ${calc_q_phq2}</t>
         </is>
       </c>
     </row>
     <row r="198" ht="15" customHeight="1" s="11">
       <c r="A198" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B198" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq2</t>
+          <t>calc_q_phq2</t>
+        </is>
+      </c>
+      <c r="F198" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
         </is>
       </c>
     </row>
     <row r="199" ht="15" customHeight="1" s="11">
       <c r="A199" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B199" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq_tot</t>
-        </is>
-      </c>
-      <c r="E199" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_phq2</t>
         </is>
       </c>
     </row>
     <row r="200" ht="15" customHeight="1" s="11">
       <c r="A200" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B200" s="13" t="inlineStr">
         <is>
-          <t>q_phq_tot</t>
-        </is>
-      </c>
-      <c r="C200" s="13" t="inlineStr">
-        <is>
-          <t>PHQ-2 Total Score: ${phq2_total}</t>
+          <t>grp_q_phq_tot</t>
+        </is>
+      </c>
+      <c r="E200" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="201" ht="15" customHeight="1" s="11">
       <c r="A201" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B201" s="13" t="inlineStr">
         <is>
-          <t>calc_q_phq_tot</t>
-        </is>
-      </c>
-      <c r="F201" s="13" t="inlineStr">
-        <is>
-          <t>${phq2_total}</t>
+          <t>q_phq_tot</t>
+        </is>
+      </c>
+      <c r="C201" s="13" t="inlineStr">
+        <is>
+          <t>PHQ-2 Total Score: ${phq2_total}</t>
         </is>
       </c>
     </row>
     <row r="202" ht="15" customHeight="1" s="11">
       <c r="A202" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B202" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq_tot</t>
+          <t>calc_q_phq_tot</t>
+        </is>
+      </c>
+      <c r="F202" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total}</t>
         </is>
       </c>
     </row>
     <row r="203" ht="15" customHeight="1" s="11">
       <c r="A203" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B203" s="13" t="inlineStr">
         <is>
-          <t>summary_high_risk</t>
-        </is>
-      </c>
-      <c r="C203" s="13" t="inlineStr">
-        <is>
-          <t>**Score is greater than 4.** This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
-        </is>
-      </c>
-      <c r="H203" s="13" t="inlineStr">
-        <is>
-          <t>${total_score} &gt; 4</t>
+          <t>grp_q_phq_tot</t>
         </is>
       </c>
     </row>
@@ -3960,46 +3937,51 @@
       </c>
       <c r="B204" s="13" t="inlineStr">
         <is>
-          <t>summary_low_risk</t>
+          <t>summary_high_risk</t>
         </is>
       </c>
       <c r="C204" s="13" t="inlineStr">
         <is>
-          <t>**Score is 4 or below.** This person appears to be at low risk for NCDs at this time.</t>
+          <t>**Score is greater than 4.** This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
         </is>
       </c>
       <c r="H204" s="13" t="inlineStr">
         <is>
-          <t>${total_score} &lt;= 4</t>
+          <t>${total_score} &gt; 4</t>
         </is>
       </c>
     </row>
     <row r="205" ht="15" customHeight="1" s="11">
       <c r="A205" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B205" s="13" t="inlineStr">
         <is>
-          <t>group_summary</t>
+          <t>summary_low_risk</t>
+        </is>
+      </c>
+      <c r="C205" s="13" t="inlineStr">
+        <is>
+          <t>**Score is 4 or below.** This person appears to be at low risk for NCDs at this time.</t>
+        </is>
+      </c>
+      <c r="H205" s="13" t="inlineStr">
+        <is>
+          <t>${total_score} &lt;= 4</t>
         </is>
       </c>
     </row>
     <row r="206" ht="15" customHeight="1" s="11">
       <c r="A206" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B206" s="13" t="inlineStr">
         <is>
-          <t>form_submit_timestamp_iso</t>
-        </is>
-      </c>
-      <c r="F206" s="13" t="inlineStr">
-        <is>
-          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+          <t>group_summary</t>
         </is>
       </c>
     </row>
@@ -4011,10 +3993,27 @@
       </c>
       <c r="B207" s="13" t="inlineStr">
         <is>
+          <t>form_submit_timestamp_iso</t>
+        </is>
+      </c>
+      <c r="F207" s="13" t="inlineStr">
+        <is>
+          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="15" customHeight="1" s="11">
+      <c r="A208" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B208" s="13" t="inlineStr">
+        <is>
           <t>form_submit_timestamp_display</t>
         </is>
       </c>
-      <c r="F207" s="13" t="inlineStr">
+      <c r="F208" s="13" t="inlineStr">
         <is>
           <t>format-date-time(now(), '%e-%b-%Y %H:%M:%S')</t>
         </is>

</xml_diff>

<commit_message>
feat: update CBAC and NCD forms to include referral facility selections and notes
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/cbac.xlsx
+++ b/config/demo/forms/app/cbac.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I208"/>
+  <dimension ref="A1:I224"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="29.53515625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="29.53" customWidth="1" style="10" min="1" max="16384"/>
@@ -822,12 +822,12 @@
       </c>
     </row>
     <row r="23" ht="16.4" customHeight="1" s="11">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>sex</t>
         </is>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="B58" s="13" t="inlineStr">
         <is>
-          <t>page_3a</t>
+          <t>page_referral</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Part B: Early Detection – Women only (1 of 3)</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
@@ -1430,151 +1430,95 @@
       </c>
       <c r="H58" s="13" t="inlineStr">
         <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>${total_score} &gt; 4</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="11">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B59" s="13" t="inlineStr">
         <is>
-          <t>breast_lump</t>
+          <t>referral_note</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>7. Lump in the breast</t>
-        </is>
-      </c>
-      <c r="G59" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>Refer this patient to **Health and Wellness Center (HWC)**</t>
+        </is>
+      </c>
+      <c r="E59" s="13" t="n"/>
+      <c r="G59" s="13" t="n"/>
       <c r="H59" s="13" t="inlineStr">
         <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>${total_score} &gt; 4</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="11">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
         <is>
-          <t>breast_lump_label</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="15" customHeight="1" s="11">
-      <c r="A61" s="13" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>nipple_discharge</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>8. Blood stained discharge from the nipple</t>
-        </is>
-      </c>
-      <c r="G61" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H61" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="15" customHeight="1" s="11">
-      <c r="A62" s="13" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>nipple_discharge_label</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="15" customHeight="1" s="11">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>breast_shape_size_change</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>9. Change in shape and size of breast</t>
-        </is>
-      </c>
-      <c r="G63" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H63" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
-        </is>
-      </c>
-    </row>
+          <t>page_referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15" customHeight="1" s="11"/>
+    <row r="62" ht="15" customHeight="1" s="11"/>
+    <row r="63" ht="15" customHeight="1" s="11"/>
     <row r="64" ht="15" customHeight="1" s="11">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
         <is>
-          <t>breast_shape_size_change_label</t>
-        </is>
-      </c>
-      <c r="F64" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
+          <t>page_3a</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>Part B: Early Detection – Women only (1 of 3)</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H64" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="11">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B65" s="13" t="inlineStr">
         <is>
-          <t>page_3a</t>
+          <t>breast_lump</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>7. Lump in the breast</t>
+        </is>
+      </c>
+      <c r="G65" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="H65" s="13" t="inlineStr">
@@ -1583,26 +1527,42 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>breast_lump_label</t>
+        </is>
+      </c>
+      <c r="F66" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
+        </is>
+      </c>
+    </row>
     <row r="67" ht="15" customHeight="1" s="11">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>page_3b</t>
+          <t>nipple_discharge</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>Part B: Early Detection – Women only (2 of 3)</t>
-        </is>
-      </c>
-      <c r="E67" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>8. Blood stained discharge from the nipple</t>
+        </is>
+      </c>
+      <c r="G67" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="H67" s="13" t="inlineStr">
@@ -1614,144 +1574,128 @@
     <row r="68" ht="15" customHeight="1" s="11">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
         <is>
-          <t>bleeding_between_periods</t>
-        </is>
-      </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>10. Bleeding between periods</t>
-        </is>
-      </c>
-      <c r="G68" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H68" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>nipple_discharge_label</t>
+        </is>
+      </c>
+      <c r="F68" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="11">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B69" s="13" t="inlineStr">
         <is>
-          <t>bleeding_between_periods_label</t>
-        </is>
-      </c>
-      <c r="F69" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
+          <t>breast_shape_size_change</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>9. Change in shape and size of breast</t>
+        </is>
+      </c>
+      <c r="G69" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="11">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
         <is>
-          <t>post_menopause_bleeding</t>
-        </is>
-      </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>11. Bleeding after menopause</t>
-        </is>
-      </c>
-      <c r="G70" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H70" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>breast_shape_size_change_label</t>
+        </is>
+      </c>
+      <c r="F70" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="11">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>post_menopause_bleeding_label</t>
-        </is>
-      </c>
-      <c r="F71" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="15" customHeight="1" s="11">
-      <c r="A72" s="13" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B72" s="13" t="inlineStr">
-        <is>
-          <t>post_intercourse_bleeding</t>
-        </is>
-      </c>
-      <c r="C72" s="13" t="inlineStr">
-        <is>
-          <t>12. Bleeding after intercourse</t>
-        </is>
-      </c>
-      <c r="G72" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H72" s="13" t="inlineStr">
+          <t>page_3a</t>
+        </is>
+      </c>
+      <c r="H71" s="13" t="inlineStr">
         <is>
           <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
+    <row r="72" ht="15" customHeight="1" s="11"/>
     <row r="73" ht="15" customHeight="1" s="11">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>post_intercourse_bleeding_label</t>
-        </is>
-      </c>
-      <c r="F73" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
+          <t>page_3b</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Part B: Early Detection – Women only (2 of 3)</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H73" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="11">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
         <is>
-          <t>page_3b</t>
+          <t>bleeding_between_periods</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>10. Bleeding between periods</t>
+        </is>
+      </c>
+      <c r="G74" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
@@ -1760,26 +1704,42 @@
         </is>
       </c>
     </row>
-    <row r="75"/>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>bleeding_between_periods_label</t>
+        </is>
+      </c>
+      <c r="F75" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
+        </is>
+      </c>
+    </row>
     <row r="76" ht="15" customHeight="1" s="11">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>page_3c</t>
+          <t>post_menopause_bleeding</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Part B: Early Detection – Women only (3 of 3)</t>
-        </is>
-      </c>
-      <c r="E76" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>11. Bleeding after menopause</t>
+        </is>
+      </c>
+      <c r="G76" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr">
@@ -1791,197 +1751,207 @@
     <row r="77" ht="15" customHeight="1" s="11">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>foul_smelling_vaginal_discharge</t>
-        </is>
-      </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>13. Foul smelling vaginal discharge</t>
-        </is>
-      </c>
-      <c r="G77" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H77" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>post_menopause_bleeding_label</t>
+        </is>
+      </c>
+      <c r="F77" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="11">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
         <is>
-          <t>foul_smelling_vaginal_discharge_label</t>
-        </is>
-      </c>
-      <c r="F78" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
+          <t>post_intercourse_bleeding</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>12. Bleeding after intercourse</t>
+        </is>
+      </c>
+      <c r="G78" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H78" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="11">
       <c r="A79" s="13" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>post_intercourse_bleeding_label</t>
+        </is>
+      </c>
+      <c r="F79" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>page_3c</t>
-        </is>
-      </c>
-      <c r="H79" s="13" t="inlineStr">
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>page_3b</t>
+        </is>
+      </c>
+      <c r="H80" s="13" t="inlineStr">
         <is>
           <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
-    <row r="80"/>
-    <row r="81" ht="15" customHeight="1" s="11">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>page_4</t>
-        </is>
-      </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>Part C: Environmental &amp; Occupational Risk Factors</t>
-        </is>
-      </c>
-      <c r="E81" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
+    <row r="81" ht="15" customHeight="1" s="11"/>
     <row r="82" ht="15" customHeight="1" s="11">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>select_multiple fuel_type</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
-          <t>fuel_type_for_cooking</t>
+          <t>page_3c</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Type of Fuel used for cooking</t>
-        </is>
-      </c>
-      <c r="G82" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Part B: Early Detection – Women only (3 of 3)</t>
+        </is>
+      </c>
+      <c r="E82" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H82" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="11">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>select_multiple occupational_exposure</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>occupational_exposure</t>
+          <t>foul_smelling_vaginal_discharge</t>
         </is>
       </c>
       <c r="C83" s="13" t="inlineStr">
         <is>
-          <t>Occupational exposure</t>
+          <t>13. Foul smelling vaginal discharge</t>
         </is>
       </c>
       <c r="G83" s="13" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="H83" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="11">
       <c r="A84" s="13" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>foul_smelling_vaginal_discharge_label</t>
+        </is>
+      </c>
+      <c r="F84" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B84" s="13" t="inlineStr">
-        <is>
-          <t>page_4</t>
-        </is>
-      </c>
-    </row>
-    <row r="85"/>
-    <row r="86" ht="15" customHeight="1" s="11">
-      <c r="A86" s="13" t="inlineStr">
-        <is>
-          <t>begin group</t>
-        </is>
-      </c>
-      <c r="B86" s="13" t="inlineStr">
-        <is>
-          <t>page_5</t>
-        </is>
-      </c>
-      <c r="C86" s="13" t="inlineStr">
-        <is>
-          <t>Part D: PHQ 2</t>
-        </is>
-      </c>
-      <c r="E86" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-    </row>
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>page_3c</t>
+        </is>
+      </c>
+      <c r="H85" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1" s="11"/>
     <row r="87" ht="15" customHeight="1" s="11">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B87" s="13" t="inlineStr">
         <is>
-          <t>phq2_instructions</t>
+          <t>page_4</t>
         </is>
       </c>
       <c r="C87" s="13" t="inlineStr">
         <is>
-          <t>Over the last 2 weeks, how often have you been bothered by the following problems?</t>
+          <t>Part C: Environmental &amp; Occupational Risk Factors</t>
+        </is>
+      </c>
+      <c r="E87" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="11">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>select_one frequency</t>
+          <t>select_multiple fuel_type</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>phq2_q1</t>
+          <t>fuel_type_for_cooking</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>1. Little interest or pleasure in doing things?</t>
+          <t>Type of Fuel used for cooking</t>
         </is>
       </c>
       <c r="G88" s="13" t="inlineStr">
@@ -1993,186 +1963,184 @@
     <row r="89" ht="15" customHeight="1" s="11">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>select_multiple occupational_exposure</t>
         </is>
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>phq2_q1_label</t>
-        </is>
-      </c>
-      <c r="C89" s="13" t="n"/>
-      <c r="F89" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
-        </is>
-      </c>
-      <c r="G89" s="13" t="n"/>
+          <t>occupational_exposure</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>Occupational exposure</t>
+        </is>
+      </c>
+      <c r="G89" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="11">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>select_one frequency</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>phq2_q2</t>
-        </is>
-      </c>
-      <c r="C90" s="13" t="inlineStr">
-        <is>
-          <t>2. Feeling down, depressed or hopeless?</t>
-        </is>
-      </c>
-      <c r="F90" s="13" t="n"/>
-      <c r="G90" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="15" customHeight="1" s="11">
-      <c r="A91" s="13" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B91" s="13" t="inlineStr">
-        <is>
-          <t>phq2_q2_label</t>
-        </is>
-      </c>
-      <c r="F91" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
-        </is>
-      </c>
-    </row>
+          <t>page_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15" customHeight="1" s="11"/>
     <row r="92" ht="15" customHeight="1" s="11">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
           <t>page_5</t>
+        </is>
+      </c>
+      <c r="C92" s="13" t="inlineStr">
+        <is>
+          <t>Part D: PHQ 2</t>
+        </is>
+      </c>
+      <c r="E92" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="11">
       <c r="A93" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B93" s="13" t="inlineStr">
         <is>
-          <t>phq2_total</t>
-        </is>
-      </c>
-      <c r="F93" s="13" t="inlineStr">
-        <is>
-          <t>${phq2_q1} + ${phq2_q2}</t>
+          <t>phq2_instructions</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>Over the last 2 weeks, how often have you been bothered by the following problems?</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="11">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B94" s="13" t="inlineStr">
         <is>
-          <t>page_5_score</t>
+          <t>phq2_q1</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Part D: PHQ-2 Score Summary</t>
-        </is>
-      </c>
-      <c r="E94" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>1. Little interest or pleasure in doing things?</t>
+        </is>
+      </c>
+      <c r="G94" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="11">
       <c r="A95" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>phq2_score_display</t>
-        </is>
-      </c>
-      <c r="C95" s="13" t="inlineStr">
-        <is>
-          <t>PHQ-2 Total Score: ${phq2_total}</t>
-        </is>
-      </c>
+          <t>phq2_q1_label</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="n"/>
+      <c r="F95" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
+        </is>
+      </c>
+      <c r="G95" s="13" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1" s="11">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>phq2_referral_note</t>
+          <t>phq2_q2</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Anyone with total score greater than 3 should be referred to CHO/MO (PHC/UPHC)</t>
-        </is>
-      </c>
-      <c r="H96" s="13" t="inlineStr">
-        <is>
-          <t>${phq2_total} &gt; 3</t>
+          <t>2. Feeling down, depressed or hopeless?</t>
+        </is>
+      </c>
+      <c r="F96" s="13" t="n"/>
+      <c r="G96" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="11">
       <c r="A97" s="13" t="inlineStr">
         <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B97" s="13" t="inlineStr">
+        <is>
+          <t>phq2_q2_label</t>
+        </is>
+      </c>
+      <c r="F97" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>page_5_score</t>
-        </is>
-      </c>
-      <c r="C97" s="13" t="n"/>
-      <c r="E97" s="13" t="n"/>
-    </row>
-    <row r="98"/>
+      <c r="B98" s="13" t="inlineStr">
+        <is>
+          <t>page_5</t>
+        </is>
+      </c>
+    </row>
     <row r="99" ht="15" customHeight="1" s="11">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>group_summary</t>
-        </is>
-      </c>
-      <c r="C99" s="13" t="inlineStr">
-        <is>
-          <t>Assessment Summary for CBAC Screening</t>
-        </is>
-      </c>
-      <c r="E99" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>phq2_total</t>
+        </is>
+      </c>
+      <c r="F99" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_q1} + ${phq2_q2}</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2152,12 @@
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>grp_filled_by</t>
+          <t>page_5_score</t>
+        </is>
+      </c>
+      <c r="C100" s="13" t="inlineStr">
+        <is>
+          <t>Part D: PHQ-2 Score Summary</t>
         </is>
       </c>
       <c r="E100" s="13" t="inlineStr">
@@ -2201,29 +2174,34 @@
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>lbl_filled_by</t>
+          <t>phq2_score_display</t>
         </is>
       </c>
       <c r="C101" s="13" t="inlineStr">
         <is>
-          <t>**Filled by:** ${reporter_name}</t>
+          <t>PHQ-2 Total Score: ${phq2_total}</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="11">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>calc_reporter</t>
-        </is>
-      </c>
-      <c r="F102" s="13" t="inlineStr">
-        <is>
-          <t>${reporter_name}</t>
+          <t>phq2_referral_note</t>
+        </is>
+      </c>
+      <c r="C102" s="13" t="inlineStr">
+        <is>
+          <t>Anyone with total score greater than 3 should be referred to Health and Wellness Center (HWC)</t>
+        </is>
+      </c>
+      <c r="H102" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total} &gt; 3</t>
         </is>
       </c>
     </row>
@@ -2235,9 +2213,11 @@
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>grp_filled_by</t>
-        </is>
-      </c>
+          <t>page_5_score</t>
+        </is>
+      </c>
+      <c r="C103" s="13" t="n"/>
+      <c r="E103" s="13" t="n"/>
     </row>
     <row r="104" ht="15" customHeight="1" s="11">
       <c r="A104" s="13" t="inlineStr">
@@ -2247,12 +2227,22 @@
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
-          <t>grp_patient</t>
+          <t>page_phq2_referral</t>
+        </is>
+      </c>
+      <c r="C104" s="13" t="inlineStr">
+        <is>
+          <t>PHQ-2 Referral</t>
         </is>
       </c>
       <c r="E104" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
+        </is>
+      </c>
+      <c r="H104" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total} &gt; 3</t>
         </is>
       </c>
     </row>
@@ -2264,44 +2254,33 @@
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>lbl_patient</t>
+          <t>phq2_referral_note_page</t>
         </is>
       </c>
       <c r="C105" s="13" t="inlineStr">
         <is>
-          <t>**Patient:** ${patient_name}</t>
+          <t>PHQ-2 score is greater than 3. Refer this patient to **Health and Wellness Center (HWC)**.</t>
+        </is>
+      </c>
+      <c r="H105" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total} &gt; 3</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="11">
       <c r="A106" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>calc_patient</t>
-        </is>
-      </c>
-      <c r="F106" s="13" t="inlineStr">
-        <is>
-          <t>${patient_name}</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="15" customHeight="1" s="11">
-      <c r="A107" s="13" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B107" s="13" t="inlineStr">
-        <is>
-          <t>grp_patient</t>
-        </is>
-      </c>
-    </row>
+          <t>page_phq2_referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1" s="11"/>
     <row r="108" ht="15" customHeight="1" s="11">
       <c r="A108" s="13" t="inlineStr">
         <is>
@@ -2310,7 +2289,12 @@
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
-          <t>grp_gender</t>
+          <t>group_summary</t>
+        </is>
+      </c>
+      <c r="C108" s="13" t="inlineStr">
+        <is>
+          <t>Assessment Summary for CBAC Screening</t>
         </is>
       </c>
       <c r="E108" s="13" t="inlineStr">
@@ -2322,315 +2306,315 @@
     <row r="109" ht="15" customHeight="1" s="11">
       <c r="A109" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>lbl_gender</t>
-        </is>
-      </c>
-      <c r="C109" s="13" t="inlineStr">
-        <is>
-          <t>**Gender:** ${calc_gender}</t>
+          <t>grp_filled_by</t>
+        </is>
+      </c>
+      <c r="E109" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="11">
       <c r="A110" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>calc_gender</t>
-        </is>
-      </c>
-      <c r="F110" s="13" t="inlineStr">
-        <is>
-          <t>if(${patient_gender} = 'male', 'Male', 'Female')</t>
+          <t>lbl_filled_by</t>
+        </is>
+      </c>
+      <c r="C110" s="13" t="inlineStr">
+        <is>
+          <t>**Filled by:** ${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="11">
       <c r="A111" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>grp_gender</t>
+          <t>calc_reporter</t>
+        </is>
+      </c>
+      <c r="F111" s="13" t="inlineStr">
+        <is>
+          <t>${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="11">
       <c r="A112" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>grp_state</t>
-        </is>
-      </c>
-      <c r="E112" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_filled_by</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="11">
       <c r="A113" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>lbl_state</t>
-        </is>
-      </c>
-      <c r="C113" s="13" t="inlineStr">
-        <is>
-          <t>**State:** ${state}</t>
+          <t>grp_patient</t>
+        </is>
+      </c>
+      <c r="E113" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="11">
       <c r="A114" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>calc_state</t>
-        </is>
-      </c>
-      <c r="F114" s="13" t="inlineStr">
-        <is>
-          <t>${state}</t>
+          <t>lbl_patient</t>
+        </is>
+      </c>
+      <c r="C114" s="13" t="inlineStr">
+        <is>
+          <t>**Patient:** ${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="11">
       <c r="A115" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>grp_state</t>
+          <t>calc_patient</t>
+        </is>
+      </c>
+      <c r="F115" s="13" t="inlineStr">
+        <is>
+          <t>${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="11">
       <c r="A116" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>grp_district</t>
-        </is>
-      </c>
-      <c r="E116" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_patient</t>
         </is>
       </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="11">
       <c r="A117" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>lbl_district</t>
-        </is>
-      </c>
-      <c r="C117" s="13" t="inlineStr">
-        <is>
-          <t>**District:** ${district}</t>
+          <t>grp_gender</t>
+        </is>
+      </c>
+      <c r="E117" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="11">
       <c r="A118" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>calc_district</t>
-        </is>
-      </c>
-      <c r="F118" s="13" t="inlineStr">
-        <is>
-          <t>${district}</t>
+          <t>lbl_gender</t>
+        </is>
+      </c>
+      <c r="C118" s="13" t="inlineStr">
+        <is>
+          <t>**Gender:** ${calc_gender}</t>
         </is>
       </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="11">
       <c r="A119" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>grp_district</t>
+          <t>calc_gender</t>
+        </is>
+      </c>
+      <c r="F119" s="13" t="inlineStr">
+        <is>
+          <t>if(${patient_gender} = 'male', 'Male', 'Female')</t>
         </is>
       </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="11">
       <c r="A120" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>grp_score</t>
-        </is>
-      </c>
-      <c r="E120" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_gender</t>
         </is>
       </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="11">
       <c r="A121" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>lbl_score</t>
-        </is>
-      </c>
-      <c r="C121" s="13" t="inlineStr">
-        <is>
-          <t>**CBAC Total Score:** ${total_score}</t>
+          <t>grp_state</t>
+        </is>
+      </c>
+      <c r="E121" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="11">
       <c r="A122" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>calc_score</t>
-        </is>
-      </c>
-      <c r="F122" s="13" t="inlineStr">
-        <is>
-          <t>${total_score}</t>
+          <t>lbl_state</t>
+        </is>
+      </c>
+      <c r="C122" s="13" t="inlineStr">
+        <is>
+          <t>**State:** ${state}</t>
         </is>
       </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="11">
       <c r="A123" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>grp_score</t>
+          <t>calc_state</t>
+        </is>
+      </c>
+      <c r="F123" s="13" t="inlineStr">
+        <is>
+          <t>${state}</t>
         </is>
       </c>
     </row>
     <row r="124" ht="15" customHeight="1" s="11">
       <c r="A124" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>grp_risk</t>
-        </is>
-      </c>
-      <c r="E124" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_state</t>
         </is>
       </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="11">
       <c r="A125" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
-          <t>lbl_risk</t>
-        </is>
-      </c>
-      <c r="C125" s="13" t="inlineStr">
-        <is>
-          <t>**Risk Category:** ${risk_category}</t>
+          <t>grp_district</t>
+        </is>
+      </c>
+      <c r="E125" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="126" ht="15" customHeight="1" s="11">
       <c r="A126" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
-          <t>calc_risk</t>
-        </is>
-      </c>
-      <c r="F126" s="13" t="inlineStr">
-        <is>
-          <t>${risk_category}</t>
+          <t>lbl_district</t>
+        </is>
+      </c>
+      <c r="C126" s="13" t="inlineStr">
+        <is>
+          <t>**District:** ${district}</t>
         </is>
       </c>
     </row>
     <row r="127" ht="15" customHeight="1" s="11">
       <c r="A127" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B127" s="13" t="inlineStr">
         <is>
-          <t>grp_risk</t>
+          <t>calc_district</t>
+        </is>
+      </c>
+      <c r="F127" s="13" t="inlineStr">
+        <is>
+          <t>${district}</t>
         </is>
       </c>
     </row>
     <row r="128" ht="15" customHeight="1" s="11">
       <c r="A128" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B128" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_a</t>
-        </is>
-      </c>
-      <c r="C128" s="13" t="inlineStr">
-        <is>
-          <t>**Part A: Risk Assessment**</t>
+          <t>grp_district</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2626,7 @@
       </c>
       <c r="B129" s="13" t="inlineStr">
         <is>
-          <t>grp_q_age</t>
+          <t>grp_score</t>
         </is>
       </c>
       <c r="E129" s="13" t="inlineStr">
@@ -2659,12 +2643,12 @@
       </c>
       <c r="B130" s="13" t="inlineStr">
         <is>
-          <t>q_age</t>
+          <t>lbl_score</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>1. Age: ${calc_q_age}</t>
+          <t>**CBAC Total Score:** ${total_score}</t>
         </is>
       </c>
     </row>
@@ -2676,12 +2660,12 @@
       </c>
       <c r="B131" s="13" t="inlineStr">
         <is>
-          <t>calc_q_age</t>
+          <t>calc_score</t>
         </is>
       </c>
       <c r="F131" s="13" t="inlineStr">
         <is>
-          <t>jr:choice-name(${age_range}, '${age_range}')</t>
+          <t>${total_score}</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2677,7 @@
       </c>
       <c r="B132" s="13" t="inlineStr">
         <is>
-          <t>grp_q_age</t>
+          <t>grp_score</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2689,7 @@
       </c>
       <c r="B133" s="13" t="inlineStr">
         <is>
-          <t>grp_q_smoke</t>
+          <t>grp_risk</t>
         </is>
       </c>
       <c r="E133" s="13" t="inlineStr">
@@ -2722,12 +2706,12 @@
       </c>
       <c r="B134" s="13" t="inlineStr">
         <is>
-          <t>q_smoke</t>
+          <t>lbl_risk</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>2. Smoke/Smokeless products: ${calc_q_smoke}</t>
+          <t>**Risk Category:** ${risk_category}</t>
         </is>
       </c>
     </row>
@@ -2739,12 +2723,12 @@
       </c>
       <c r="B135" s="13" t="inlineStr">
         <is>
-          <t>calc_q_smoke</t>
+          <t>calc_risk</t>
         </is>
       </c>
       <c r="F135" s="13" t="inlineStr">
         <is>
-          <t>jr:choice-name(${smoke_frequency}, '${smoke_frequency}')</t>
+          <t>${risk_category}</t>
         </is>
       </c>
     </row>
@@ -2756,281 +2740,276 @@
       </c>
       <c r="B136" s="13" t="inlineStr">
         <is>
-          <t>grp_q_smoke</t>
+          <t>grp_risk</t>
         </is>
       </c>
     </row>
     <row r="137" ht="15" customHeight="1" s="11">
       <c r="A137" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B137" s="13" t="inlineStr">
         <is>
-          <t>grp_q_alcohol</t>
-        </is>
-      </c>
-      <c r="E137" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>sum_hdr_a</t>
+        </is>
+      </c>
+      <c r="C137" s="13" t="inlineStr">
+        <is>
+          <t>**Part A: Risk Assessment**</t>
         </is>
       </c>
     </row>
     <row r="138" ht="15" customHeight="1" s="11">
       <c r="A138" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B138" s="13" t="inlineStr">
         <is>
-          <t>q_alcohol</t>
-        </is>
-      </c>
-      <c r="C138" s="13" t="inlineStr">
-        <is>
-          <t>3. Alcohol daily: ${calc_q_alcohol}</t>
+          <t>grp_q_age</t>
+        </is>
+      </c>
+      <c r="E138" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="11">
       <c r="A139" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B139" s="13" t="inlineStr">
         <is>
-          <t>calc_q_alcohol</t>
-        </is>
-      </c>
-      <c r="F139" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${alcohol_frequency}, '${alcohol_frequency}')</t>
+          <t>q_age</t>
+        </is>
+      </c>
+      <c r="C139" s="13" t="inlineStr">
+        <is>
+          <t>1. Age: ${calc_q_age}</t>
         </is>
       </c>
     </row>
     <row r="140" ht="15" customHeight="1" s="11">
       <c r="A140" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B140" s="13" t="inlineStr">
         <is>
-          <t>grp_q_alcohol</t>
+          <t>calc_q_age</t>
+        </is>
+      </c>
+      <c r="F140" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${age_range}, '${age_range}')</t>
         </is>
       </c>
     </row>
     <row r="141" ht="15" customHeight="1" s="11">
       <c r="A141" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B141" s="13" t="inlineStr">
         <is>
-          <t>grp_q_waist</t>
-        </is>
-      </c>
-      <c r="E141" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_age</t>
         </is>
       </c>
     </row>
     <row r="142" ht="15" customHeight="1" s="11">
       <c r="A142" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B142" s="13" t="inlineStr">
         <is>
-          <t>q_waist</t>
-        </is>
-      </c>
-      <c r="C142" s="13" t="inlineStr">
-        <is>
-          <t>4. Waist measurement: ${calc_q_waist}</t>
+          <t>grp_q_smoke</t>
+        </is>
+      </c>
+      <c r="E142" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="143" ht="15" customHeight="1" s="11">
       <c r="A143" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B143" s="13" t="inlineStr">
         <is>
-          <t>calc_q_waist</t>
-        </is>
-      </c>
-      <c r="F143" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${waist_size}, '${waist_size}')</t>
+          <t>q_smoke</t>
+        </is>
+      </c>
+      <c r="C143" s="13" t="inlineStr">
+        <is>
+          <t>2. Smoke/Smokeless products: ${calc_q_smoke}</t>
         </is>
       </c>
     </row>
     <row r="144" ht="15" customHeight="1" s="11">
       <c r="A144" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B144" s="13" t="inlineStr">
         <is>
-          <t>grp_q_waist</t>
+          <t>calc_q_smoke</t>
+        </is>
+      </c>
+      <c r="F144" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${smoke_frequency}, '${smoke_frequency}')</t>
         </is>
       </c>
     </row>
     <row r="145" ht="15" customHeight="1" s="11">
       <c r="A145" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B145" s="13" t="inlineStr">
         <is>
-          <t>grp_q_physical</t>
-        </is>
-      </c>
-      <c r="E145" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_smoke</t>
         </is>
       </c>
     </row>
     <row r="146" ht="15" customHeight="1" s="11">
       <c r="A146" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B146" s="13" t="inlineStr">
         <is>
-          <t>q_physical</t>
-        </is>
-      </c>
-      <c r="C146" s="13" t="inlineStr">
-        <is>
-          <t>5. Physical activity (150 min/week): ${calc_q_physical}</t>
+          <t>grp_q_alcohol</t>
+        </is>
+      </c>
+      <c r="E146" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="147" ht="15" customHeight="1" s="11">
       <c r="A147" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B147" s="13" t="inlineStr">
         <is>
-          <t>calc_q_physical</t>
-        </is>
-      </c>
-      <c r="F147" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${physical_activities_frequency}, '${physical_activities_frequency}')</t>
+          <t>q_alcohol</t>
+        </is>
+      </c>
+      <c r="C147" s="13" t="inlineStr">
+        <is>
+          <t>3. Alcohol daily: ${calc_q_alcohol}</t>
         </is>
       </c>
     </row>
     <row r="148" ht="15" customHeight="1" s="11">
       <c r="A148" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B148" s="13" t="inlineStr">
         <is>
-          <t>grp_q_physical</t>
+          <t>calc_q_alcohol</t>
+        </is>
+      </c>
+      <c r="F148" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${alcohol_frequency}, '${alcohol_frequency}')</t>
         </is>
       </c>
     </row>
     <row r="149" ht="15" customHeight="1" s="11">
       <c r="A149" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B149" s="13" t="inlineStr">
         <is>
-          <t>grp_q_family</t>
-        </is>
-      </c>
-      <c r="E149" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_alcohol</t>
         </is>
       </c>
     </row>
     <row r="150" ht="15" customHeight="1" s="11">
       <c r="A150" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B150" s="13" t="inlineStr">
         <is>
-          <t>q_family</t>
-        </is>
-      </c>
-      <c r="C150" s="13" t="inlineStr">
-        <is>
-          <t>6. Family history of BP/Diabetes/Heart disease: ${calc_q_family}</t>
+          <t>grp_q_waist</t>
+        </is>
+      </c>
+      <c r="E150" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="151" ht="15" customHeight="1" s="11">
       <c r="A151" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B151" s="13" t="inlineStr">
         <is>
-          <t>calc_q_family</t>
-        </is>
-      </c>
-      <c r="F151" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${family_medical_history}, '${family_medical_history}')</t>
+          <t>q_waist</t>
+        </is>
+      </c>
+      <c r="C151" s="13" t="inlineStr">
+        <is>
+          <t>4. Waist measurement: ${calc_q_waist}</t>
         </is>
       </c>
     </row>
     <row r="152" ht="15" customHeight="1" s="11">
       <c r="A152" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B152" s="13" t="inlineStr">
         <is>
-          <t>grp_q_family</t>
+          <t>calc_q_waist</t>
+        </is>
+      </c>
+      <c r="F152" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${waist_size}, '${waist_size}')</t>
         </is>
       </c>
     </row>
     <row r="153" ht="15" customHeight="1" s="11">
       <c r="A153" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B153" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_b</t>
-        </is>
-      </c>
-      <c r="C153" s="13" t="inlineStr">
-        <is>
-          <t>**Part B: Early Detection**</t>
-        </is>
-      </c>
-      <c r="H153" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>grp_q_waist</t>
         </is>
       </c>
     </row>
@@ -3042,17 +3021,12 @@
       </c>
       <c r="B154" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_lump</t>
+          <t>grp_q_physical</t>
         </is>
       </c>
       <c r="E154" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
-        </is>
-      </c>
-      <c r="H154" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3064,17 +3038,12 @@
       </c>
       <c r="B155" s="13" t="inlineStr">
         <is>
-          <t>q_breast_lump</t>
+          <t>q_physical</t>
         </is>
       </c>
       <c r="C155" s="13" t="inlineStr">
         <is>
-          <t>7. Lump in the breast: ${calc_q_breast_lump}</t>
-        </is>
-      </c>
-      <c r="H155" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>5. Physical activity (150 min/week): ${calc_q_physical}</t>
         </is>
       </c>
     </row>
@@ -3086,12 +3055,12 @@
       </c>
       <c r="B156" s="13" t="inlineStr">
         <is>
-          <t>calc_q_breast_lump</t>
+          <t>calc_q_physical</t>
         </is>
       </c>
       <c r="F156" s="13" t="inlineStr">
         <is>
-          <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
+          <t>jr:choice-name(${physical_activities_frequency}, '${physical_activities_frequency}')</t>
         </is>
       </c>
     </row>
@@ -3103,12 +3072,7 @@
       </c>
       <c r="B157" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_lump</t>
-        </is>
-      </c>
-      <c r="H157" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>grp_q_physical</t>
         </is>
       </c>
     </row>
@@ -3120,17 +3084,12 @@
       </c>
       <c r="B158" s="13" t="inlineStr">
         <is>
-          <t>grp_q_nipple</t>
+          <t>grp_q_family</t>
         </is>
       </c>
       <c r="E158" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
-        </is>
-      </c>
-      <c r="H158" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3142,17 +3101,12 @@
       </c>
       <c r="B159" s="13" t="inlineStr">
         <is>
-          <t>q_nipple</t>
+          <t>q_family</t>
         </is>
       </c>
       <c r="C159" s="13" t="inlineStr">
         <is>
-          <t>8. Blood stained nipple discharge: ${calc_q_nipple}</t>
-        </is>
-      </c>
-      <c r="H159" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>6. Family history of BP/Diabetes/Heart disease: ${calc_q_family}</t>
         </is>
       </c>
     </row>
@@ -3164,12 +3118,12 @@
       </c>
       <c r="B160" s="13" t="inlineStr">
         <is>
-          <t>calc_q_nipple</t>
+          <t>calc_q_family</t>
         </is>
       </c>
       <c r="F160" s="13" t="inlineStr">
         <is>
-          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
+          <t>jr:choice-name(${family_medical_history}, '${family_medical_history}')</t>
         </is>
       </c>
     </row>
@@ -3181,29 +3135,24 @@
       </c>
       <c r="B161" s="13" t="inlineStr">
         <is>
-          <t>grp_q_nipple</t>
-        </is>
-      </c>
-      <c r="H161" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>grp_q_family</t>
         </is>
       </c>
     </row>
     <row r="162" ht="15" customHeight="1" s="11">
       <c r="A162" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B162" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_shape</t>
-        </is>
-      </c>
-      <c r="E162" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>sum_hdr_b</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="inlineStr">
+        <is>
+          <t>**Part B: Early Detection**</t>
         </is>
       </c>
       <c r="H162" s="13" t="inlineStr">
@@ -3215,17 +3164,17 @@
     <row r="163" ht="15" customHeight="1" s="11">
       <c r="A163" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B163" s="13" t="inlineStr">
         <is>
-          <t>q_breast_shape</t>
-        </is>
-      </c>
-      <c r="C163" s="13" t="inlineStr">
-        <is>
-          <t>9. Change in breast shape/size: ${calc_q_breast_shape}</t>
+          <t>grp_q_breast_lump</t>
+        </is>
+      </c>
+      <c r="E163" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H163" s="13" t="inlineStr">
@@ -3237,51 +3186,51 @@
     <row r="164" ht="15" customHeight="1" s="11">
       <c r="A164" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B164" s="13" t="inlineStr">
         <is>
-          <t>calc_q_breast_shape</t>
-        </is>
-      </c>
-      <c r="F164" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
+          <t>q_breast_lump</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="inlineStr">
+        <is>
+          <t>7. Lump in the breast: ${calc_q_breast_lump}</t>
+        </is>
+      </c>
+      <c r="H164" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="165" ht="15" customHeight="1" s="11">
       <c r="A165" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B165" s="13" t="inlineStr">
         <is>
-          <t>grp_q_breast_shape</t>
-        </is>
-      </c>
-      <c r="H165" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>calc_q_breast_lump</t>
+        </is>
+      </c>
+      <c r="F165" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_lump}, '${breast_lump}')</t>
         </is>
       </c>
     </row>
     <row r="166" ht="15" customHeight="1" s="11">
       <c r="A166" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B166" s="13" t="inlineStr">
         <is>
-          <t>grp_q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="E166" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_breast_lump</t>
         </is>
       </c>
       <c r="H166" s="13" t="inlineStr">
@@ -3293,17 +3242,17 @@
     <row r="167" ht="15" customHeight="1" s="11">
       <c r="A167" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B167" s="13" t="inlineStr">
         <is>
-          <t>q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="C167" s="13" t="inlineStr">
-        <is>
-          <t>10. Bleeding between periods: ${calc_q_bleeding_periods}</t>
+          <t>grp_q_nipple</t>
+        </is>
+      </c>
+      <c r="E167" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H167" s="13" t="inlineStr">
@@ -3315,51 +3264,51 @@
     <row r="168" ht="15" customHeight="1" s="11">
       <c r="A168" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B168" s="13" t="inlineStr">
         <is>
-          <t>calc_q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="F168" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
+          <t>q_nipple</t>
+        </is>
+      </c>
+      <c r="C168" s="13" t="inlineStr">
+        <is>
+          <t>8. Blood stained nipple discharge: ${calc_q_nipple}</t>
+        </is>
+      </c>
+      <c r="H168" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="169" ht="15" customHeight="1" s="11">
       <c r="A169" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B169" s="13" t="inlineStr">
         <is>
-          <t>grp_q_bleeding_periods</t>
-        </is>
-      </c>
-      <c r="H169" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>calc_q_nipple</t>
+        </is>
+      </c>
+      <c r="F169" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${nipple_discharge}, '${nipple_discharge}')</t>
         </is>
       </c>
     </row>
     <row r="170" ht="15" customHeight="1" s="11">
       <c r="A170" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B170" s="13" t="inlineStr">
         <is>
-          <t>grp_q_menopause</t>
-        </is>
-      </c>
-      <c r="E170" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_nipple</t>
         </is>
       </c>
       <c r="H170" s="13" t="inlineStr">
@@ -3371,17 +3320,17 @@
     <row r="171" ht="15" customHeight="1" s="11">
       <c r="A171" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B171" s="13" t="inlineStr">
         <is>
-          <t>q_menopause</t>
-        </is>
-      </c>
-      <c r="C171" s="13" t="inlineStr">
-        <is>
-          <t>11. Bleeding after menopause: ${calc_q_menopause}</t>
+          <t>grp_q_breast_shape</t>
+        </is>
+      </c>
+      <c r="E171" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H171" s="13" t="inlineStr">
@@ -3393,51 +3342,51 @@
     <row r="172" ht="15" customHeight="1" s="11">
       <c r="A172" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B172" s="13" t="inlineStr">
         <is>
-          <t>calc_q_menopause</t>
-        </is>
-      </c>
-      <c r="F172" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
+          <t>q_breast_shape</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="inlineStr">
+        <is>
+          <t>9. Change in breast shape/size: ${calc_q_breast_shape}</t>
+        </is>
+      </c>
+      <c r="H172" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="173" ht="15" customHeight="1" s="11">
       <c r="A173" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B173" s="13" t="inlineStr">
         <is>
-          <t>grp_q_menopause</t>
-        </is>
-      </c>
-      <c r="H173" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>calc_q_breast_shape</t>
+        </is>
+      </c>
+      <c r="F173" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${breast_shape_size_change}, '${breast_shape_size_change}')</t>
         </is>
       </c>
     </row>
     <row r="174" ht="15" customHeight="1" s="11">
       <c r="A174" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B174" s="13" t="inlineStr">
         <is>
-          <t>grp_q_intercourse</t>
-        </is>
-      </c>
-      <c r="E174" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_breast_shape</t>
         </is>
       </c>
       <c r="H174" s="13" t="inlineStr">
@@ -3449,17 +3398,17 @@
     <row r="175" ht="15" customHeight="1" s="11">
       <c r="A175" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B175" s="13" t="inlineStr">
         <is>
-          <t>q_intercourse</t>
-        </is>
-      </c>
-      <c r="C175" s="13" t="inlineStr">
-        <is>
-          <t>12. Bleeding after intercourse: ${calc_q_intercourse}</t>
+          <t>grp_q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="E175" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H175" s="13" t="inlineStr">
@@ -3471,51 +3420,51 @@
     <row r="176" ht="15" customHeight="1" s="11">
       <c r="A176" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B176" s="13" t="inlineStr">
         <is>
-          <t>calc_q_intercourse</t>
-        </is>
-      </c>
-      <c r="F176" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
+          <t>q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="inlineStr">
+        <is>
+          <t>10. Bleeding between periods: ${calc_q_bleeding_periods}</t>
+        </is>
+      </c>
+      <c r="H176" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="177" ht="15" customHeight="1" s="11">
       <c r="A177" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B177" s="13" t="inlineStr">
         <is>
-          <t>grp_q_intercourse</t>
-        </is>
-      </c>
-      <c r="H177" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>calc_q_bleeding_periods</t>
+        </is>
+      </c>
+      <c r="F177" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${bleeding_between_periods}, '${bleeding_between_periods}')</t>
         </is>
       </c>
     </row>
     <row r="178" ht="15" customHeight="1" s="11">
       <c r="A178" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B178" s="13" t="inlineStr">
         <is>
-          <t>grp_q_discharge</t>
-        </is>
-      </c>
-      <c r="E178" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_q_bleeding_periods</t>
         </is>
       </c>
       <c r="H178" s="13" t="inlineStr">
@@ -3527,17 +3476,17 @@
     <row r="179" ht="15" customHeight="1" s="11">
       <c r="A179" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B179" s="13" t="inlineStr">
         <is>
-          <t>q_discharge</t>
-        </is>
-      </c>
-      <c r="C179" s="13" t="inlineStr">
-        <is>
-          <t>13. Foul smelling vaginal discharge: ${calc_q_discharge}</t>
+          <t>grp_q_menopause</t>
+        </is>
+      </c>
+      <c r="E179" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
       <c r="H179" s="13" t="inlineStr">
@@ -3549,51 +3498,56 @@
     <row r="180" ht="15" customHeight="1" s="11">
       <c r="A180" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B180" s="13" t="inlineStr">
         <is>
-          <t>calc_q_discharge</t>
-        </is>
-      </c>
-      <c r="F180" s="13" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
+          <t>q_menopause</t>
+        </is>
+      </c>
+      <c r="C180" s="13" t="inlineStr">
+        <is>
+          <t>11. Bleeding after menopause: ${calc_q_menopause}</t>
+        </is>
+      </c>
+      <c r="H180" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
     <row r="181" ht="15" customHeight="1" s="11">
       <c r="A181" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B181" s="13" t="inlineStr">
         <is>
-          <t>grp_q_discharge</t>
-        </is>
-      </c>
-      <c r="H181" s="13" t="inlineStr">
-        <is>
-          <t>${patient_gender} = 'female'</t>
+          <t>calc_q_menopause</t>
+        </is>
+      </c>
+      <c r="F181" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${post_menopause_bleeding}, '${post_menopause_bleeding}')</t>
         </is>
       </c>
     </row>
     <row r="182" ht="15" customHeight="1" s="11">
       <c r="A182" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B182" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_c</t>
-        </is>
-      </c>
-      <c r="C182" s="13" t="inlineStr">
-        <is>
-          <t>**Part C: Environmental &amp; Occupational Risk Factors**</t>
+          <t>grp_q_menopause</t>
+        </is>
+      </c>
+      <c r="H182" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3605,12 +3559,17 @@
       </c>
       <c r="B183" s="13" t="inlineStr">
         <is>
-          <t>grp_q_fuel</t>
+          <t>grp_q_intercourse</t>
         </is>
       </c>
       <c r="E183" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
+        </is>
+      </c>
+      <c r="H183" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3622,12 +3581,17 @@
       </c>
       <c r="B184" s="13" t="inlineStr">
         <is>
-          <t>q_fuel</t>
+          <t>q_intercourse</t>
         </is>
       </c>
       <c r="C184" s="13" t="inlineStr">
         <is>
-          <t>Fuel used for cooking: ${calc_q_fuel}</t>
+          <t>12. Bleeding after intercourse: ${calc_q_intercourse}</t>
+        </is>
+      </c>
+      <c r="H184" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3639,12 +3603,12 @@
       </c>
       <c r="B185" s="13" t="inlineStr">
         <is>
-          <t>calc_q_fuel</t>
+          <t>calc_q_intercourse</t>
         </is>
       </c>
       <c r="F185" s="13" t="inlineStr">
         <is>
-          <t>concat(if(selected(${fuel_type_for_cooking}, 'firewood'), 'Firewood', ''), if(selected(${fuel_type_for_cooking}, 'firewood') and string-length(${fuel_type_for_cooking}) &gt; 9, ' / ', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue'), 'Crop Residue', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue') and (selected(${fuel_type_for_cooking}, 'cow_dung_cake') or selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake'), 'Cow dung cake', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake') and (selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'coal'), 'Coal', ''), if(selected(${fuel_type_for_cooking}, 'coal') and (selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'kerosene'), 'Kerosene', ''), if(selected(${fuel_type_for_cooking}, 'kerosene') and selected(${fuel_type_for_cooking}, 'lpg'), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'lpg'), 'LPG', ''))</t>
+          <t>jr:choice-name(${post_intercourse_bleeding}, '${post_intercourse_bleeding}')</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3620,12 @@
       </c>
       <c r="B186" s="13" t="inlineStr">
         <is>
-          <t>grp_q_fuel</t>
+          <t>grp_q_intercourse</t>
+        </is>
+      </c>
+      <c r="H186" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3668,12 +3637,17 @@
       </c>
       <c r="B187" s="13" t="inlineStr">
         <is>
-          <t>grp_q_occupation</t>
+          <t>grp_q_discharge</t>
         </is>
       </c>
       <c r="E187" s="13" t="inlineStr">
         <is>
           <t>field-list</t>
+        </is>
+      </c>
+      <c r="H187" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3685,12 +3659,17 @@
       </c>
       <c r="B188" s="13" t="inlineStr">
         <is>
-          <t>q_occupation</t>
+          <t>q_discharge</t>
         </is>
       </c>
       <c r="C188" s="13" t="inlineStr">
         <is>
-          <t>Occupational exposure: ${calc_q_occupation}</t>
+          <t>13. Foul smelling vaginal discharge: ${calc_q_discharge}</t>
+        </is>
+      </c>
+      <c r="H188" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3702,12 +3681,12 @@
       </c>
       <c r="B189" s="13" t="inlineStr">
         <is>
-          <t>calc_q_occupation</t>
+          <t>calc_q_discharge</t>
         </is>
       </c>
       <c r="F189" s="13" t="inlineStr">
         <is>
-          <t>concat(if(selected(${occupational_exposure}, 'crop_residue_burning'), 'Crop residue burning', ''), if(selected(${occupational_exposure}, 'crop_residue_burning') and (selected(${occupational_exposure}, 'working_in_industries') or selected(${occupational_exposure}, 'none')), ' / ', ''), if(selected(${occupational_exposure}, 'working_in_industries'), 'Working in industries', ''), if(selected(${occupational_exposure}, 'working_in_industries') and selected(${occupational_exposure}, 'none'), ' / ', ''), if(selected(${occupational_exposure}, 'none'), 'None of the above', ''))</t>
+          <t>jr:choice-name(${foul_smelling_vaginal_discharge}, '${foul_smelling_vaginal_discharge}')</t>
         </is>
       </c>
     </row>
@@ -3719,7 +3698,12 @@
       </c>
       <c r="B190" s="13" t="inlineStr">
         <is>
-          <t>grp_q_occupation</t>
+          <t>grp_q_discharge</t>
+        </is>
+      </c>
+      <c r="H190" s="13" t="inlineStr">
+        <is>
+          <t>${patient_gender} = 'female'</t>
         </is>
       </c>
     </row>
@@ -3731,12 +3715,12 @@
       </c>
       <c r="B191" s="13" t="inlineStr">
         <is>
-          <t>sum_hdr_d</t>
+          <t>sum_hdr_c</t>
         </is>
       </c>
       <c r="C191" s="13" t="inlineStr">
         <is>
-          <t>**Part D: PHQ-2**</t>
+          <t>**Part C: Environmental &amp; Occupational Risk Factors**</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3732,7 @@
       </c>
       <c r="B192" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq1</t>
+          <t>grp_q_fuel</t>
         </is>
       </c>
       <c r="E192" s="13" t="inlineStr">
@@ -3765,12 +3749,12 @@
       </c>
       <c r="B193" s="13" t="inlineStr">
         <is>
-          <t>q_phq1</t>
+          <t>q_fuel</t>
         </is>
       </c>
       <c r="C193" s="13" t="inlineStr">
         <is>
-          <t>1. Little interest or pleasure in doing things: ${calc_q_phq1}</t>
+          <t>Fuel used for cooking: ${calc_q_fuel}</t>
         </is>
       </c>
     </row>
@@ -3782,12 +3766,12 @@
       </c>
       <c r="B194" s="13" t="inlineStr">
         <is>
-          <t>calc_q_phq1</t>
+          <t>calc_q_fuel</t>
         </is>
       </c>
       <c r="F194" s="13" t="inlineStr">
         <is>
-          <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
+          <t>concat(if(selected(${fuel_type_for_cooking}, 'firewood'), 'Firewood', ''), if(selected(${fuel_type_for_cooking}, 'firewood') and string-length(${fuel_type_for_cooking}) &gt; 9, ' / ', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue'), 'Crop Residue', ''), if(selected(${fuel_type_for_cooking}, 'crop_residue') and (selected(${fuel_type_for_cooking}, 'cow_dung_cake') or selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake'), 'Cow dung cake', ''), if(selected(${fuel_type_for_cooking}, 'cow_dung_cake') and (selected(${fuel_type_for_cooking}, 'coal') or selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'coal'), 'Coal', ''), if(selected(${fuel_type_for_cooking}, 'coal') and (selected(${fuel_type_for_cooking}, 'kerosene') or selected(${fuel_type_for_cooking}, 'lpg')), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'kerosene'), 'Kerosene', ''), if(selected(${fuel_type_for_cooking}, 'kerosene') and selected(${fuel_type_for_cooking}, 'lpg'), ' / ', ''), if(selected(${fuel_type_for_cooking}, 'lpg'), 'LPG', ''))</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3783,7 @@
       </c>
       <c r="B195" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq1</t>
+          <t>grp_q_fuel</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3795,7 @@
       </c>
       <c r="B196" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq2</t>
+          <t>grp_q_occupation</t>
         </is>
       </c>
       <c r="E196" s="13" t="inlineStr">
@@ -3828,12 +3812,12 @@
       </c>
       <c r="B197" s="13" t="inlineStr">
         <is>
-          <t>q_phq2</t>
+          <t>q_occupation</t>
         </is>
       </c>
       <c r="C197" s="13" t="inlineStr">
         <is>
-          <t>2. Feeling down, depressed or hopeless: ${calc_q_phq2}</t>
+          <t>Occupational exposure: ${calc_q_occupation}</t>
         </is>
       </c>
     </row>
@@ -3845,12 +3829,12 @@
       </c>
       <c r="B198" s="13" t="inlineStr">
         <is>
-          <t>calc_q_phq2</t>
+          <t>calc_q_occupation</t>
         </is>
       </c>
       <c r="F198" s="13" t="inlineStr">
         <is>
-          <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
+          <t>concat(if(selected(${occupational_exposure}, 'crop_residue_burning'), 'Crop residue burning', ''), if(selected(${occupational_exposure}, 'crop_residue_burning') and (selected(${occupational_exposure}, 'working_in_industries') or selected(${occupational_exposure}, 'none')), ' / ', ''), if(selected(${occupational_exposure}, 'working_in_industries'), 'Working in industries', ''), if(selected(${occupational_exposure}, 'working_in_industries') and selected(${occupational_exposure}, 'none'), ' / ', ''), if(selected(${occupational_exposure}, 'none'), 'None of the above', ''))</t>
         </is>
       </c>
     </row>
@@ -3862,126 +3846,121 @@
       </c>
       <c r="B199" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq2</t>
+          <t>grp_q_occupation</t>
         </is>
       </c>
     </row>
     <row r="200" ht="15" customHeight="1" s="11">
       <c r="A200" s="13" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B200" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq_tot</t>
-        </is>
-      </c>
-      <c r="E200" s="13" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>sum_hdr_d</t>
+        </is>
+      </c>
+      <c r="C200" s="13" t="inlineStr">
+        <is>
+          <t>**Part D: PHQ-2**</t>
         </is>
       </c>
     </row>
     <row r="201" ht="15" customHeight="1" s="11">
       <c r="A201" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B201" s="13" t="inlineStr">
         <is>
-          <t>q_phq_tot</t>
-        </is>
-      </c>
-      <c r="C201" s="13" t="inlineStr">
-        <is>
-          <t>PHQ-2 Total Score: ${phq2_total}</t>
+          <t>grp_q_phq1</t>
+        </is>
+      </c>
+      <c r="E201" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="202" ht="15" customHeight="1" s="11">
       <c r="A202" s="13" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B202" s="13" t="inlineStr">
         <is>
-          <t>calc_q_phq_tot</t>
-        </is>
-      </c>
-      <c r="F202" s="13" t="inlineStr">
-        <is>
-          <t>${phq2_total}</t>
+          <t>q_phq1</t>
+        </is>
+      </c>
+      <c r="C202" s="13" t="inlineStr">
+        <is>
+          <t>1. Little interest or pleasure in doing things: ${calc_q_phq1}</t>
         </is>
       </c>
     </row>
     <row r="203" ht="15" customHeight="1" s="11">
       <c r="A203" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B203" s="13" t="inlineStr">
         <is>
-          <t>grp_q_phq_tot</t>
+          <t>calc_q_phq1</t>
+        </is>
+      </c>
+      <c r="F203" s="13" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${phq2_q1}, '${phq2_q1}')</t>
         </is>
       </c>
     </row>
     <row r="204" ht="15" customHeight="1" s="11">
       <c r="A204" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B204" s="13" t="inlineStr">
         <is>
-          <t>summary_high_risk</t>
-        </is>
-      </c>
-      <c r="C204" s="13" t="inlineStr">
-        <is>
-          <t>**Score is greater than 4.** This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
-        </is>
-      </c>
-      <c r="H204" s="13" t="inlineStr">
-        <is>
-          <t>${total_score} &gt; 4</t>
+          <t>grp_q_phq1</t>
         </is>
       </c>
     </row>
     <row r="205" ht="15" customHeight="1" s="11">
       <c r="A205" s="13" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B205" s="13" t="inlineStr">
         <is>
-          <t>summary_low_risk</t>
-        </is>
-      </c>
-      <c r="C205" s="13" t="inlineStr">
-        <is>
-          <t>**Score is 4 or below.** This person appears to be at low risk for NCDs at this time.</t>
-        </is>
-      </c>
-      <c r="H205" s="13" t="inlineStr">
-        <is>
-          <t>${total_score} &lt;= 4</t>
+          <t>grp_q_phq2</t>
+        </is>
+      </c>
+      <c r="E205" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="206" ht="15" customHeight="1" s="11">
       <c r="A206" s="13" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B206" s="13" t="inlineStr">
         <is>
-          <t>group_summary</t>
+          <t>q_phq2</t>
+        </is>
+      </c>
+      <c r="C206" s="13" t="inlineStr">
+        <is>
+          <t>2. Feeling down, depressed or hopeless: ${calc_q_phq2}</t>
         </is>
       </c>
     </row>
@@ -3993,27 +3972,304 @@
       </c>
       <c r="B207" s="13" t="inlineStr">
         <is>
-          <t>form_submit_timestamp_iso</t>
+          <t>calc_q_phq2</t>
         </is>
       </c>
       <c r="F207" s="13" t="inlineStr">
         <is>
-          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+          <t>jr:choice-name(${phq2_q2}, '${phq2_q2}')</t>
         </is>
       </c>
     </row>
     <row r="208" ht="15" customHeight="1" s="11">
       <c r="A208" s="13" t="inlineStr">
         <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B208" s="13" t="inlineStr">
+        <is>
+          <t>grp_q_phq2</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="13" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B209" s="13" t="inlineStr">
+        <is>
+          <t>grp_q_phq_tot</t>
+        </is>
+      </c>
+      <c r="E209" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B210" s="13" t="inlineStr">
+        <is>
+          <t>q_phq_tot</t>
+        </is>
+      </c>
+      <c r="C210" s="13" t="inlineStr">
+        <is>
+          <t>PHQ-2 Total Score: ${phq2_total}</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="13" t="inlineStr">
+        <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B208" s="13" t="inlineStr">
+      <c r="B211" s="13" t="inlineStr">
+        <is>
+          <t>calc_q_phq_tot</t>
+        </is>
+      </c>
+      <c r="F211" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total}</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="13" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B212" s="13" t="inlineStr">
+        <is>
+          <t>grp_q_phq_tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B213" s="13" t="inlineStr">
+        <is>
+          <t>summary_high_risk</t>
+        </is>
+      </c>
+      <c r="C213" s="13" t="inlineStr">
+        <is>
+          <t>**Score is greater than 4.** This person may be at risk for NCDs and should be prioritized for the weekly NCD day.</t>
+        </is>
+      </c>
+      <c r="H213" s="13" t="inlineStr">
+        <is>
+          <t>${total_score} &gt; 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B214" s="13" t="inlineStr">
+        <is>
+          <t>summary_low_risk</t>
+        </is>
+      </c>
+      <c r="C214" s="13" t="inlineStr">
+        <is>
+          <t>**Score is 4 or below.** This person appears to be at low risk for NCDs at this time.</t>
+        </is>
+      </c>
+      <c r="H214" s="13" t="inlineStr">
+        <is>
+          <t>${total_score} &lt;= 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="13" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B215" s="13" t="inlineStr">
+        <is>
+          <t>grp_referral</t>
+        </is>
+      </c>
+      <c r="E215" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H215" s="13" t="inlineStr">
+        <is>
+          <t>${total_score} &gt; 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B216" s="13" t="inlineStr">
+        <is>
+          <t>lbl_referral</t>
+        </is>
+      </c>
+      <c r="C216" s="13" t="inlineStr">
+        <is>
+          <t>**CBAC Risk Score Referral:** Health and Wellness Center (HWC)</t>
+        </is>
+      </c>
+      <c r="H216" s="13" t="inlineStr">
+        <is>
+          <t>${total_score} &gt; 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="13" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B217" s="13" t="inlineStr">
+        <is>
+          <t>grp_referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="13" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B218" s="13" t="inlineStr">
+        <is>
+          <t>grp_phq2_referral</t>
+        </is>
+      </c>
+      <c r="E218" s="13" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+      <c r="H218" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total} &gt; 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B219" s="13" t="inlineStr">
+        <is>
+          <t>lbl_phq2_referral</t>
+        </is>
+      </c>
+      <c r="C219" s="13" t="inlineStr">
+        <is>
+          <t>**PHQ-2 Referral:** Health and Wellness Center (HWC)</t>
+        </is>
+      </c>
+      <c r="H219" s="13" t="inlineStr">
+        <is>
+          <t>${phq2_total} &gt; 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B220" s="13" t="inlineStr">
+        <is>
+          <t>calc_phq2_referral</t>
+        </is>
+      </c>
+      <c r="F220" s="13" t="inlineStr">
+        <is>
+          <t>if(${phq2_total} &gt; 3, 'Health and Wellness Center (HWC)', '')</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="13" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B221" s="13" t="inlineStr">
+        <is>
+          <t>grp_phq2_referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="13" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B222" s="13" t="inlineStr">
+        <is>
+          <t>group_summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B223" s="13" t="inlineStr">
+        <is>
+          <t>form_submit_timestamp_iso</t>
+        </is>
+      </c>
+      <c r="F223" s="13" t="inlineStr">
+        <is>
+          <t>format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30')</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="13" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B224" s="13" t="inlineStr">
         <is>
           <t>form_submit_timestamp_display</t>
         </is>
       </c>
-      <c r="F208" s="13" t="inlineStr">
+      <c r="F224" s="13" t="inlineStr">
         <is>
           <t>format-date-time(now(), '%e-%b-%Y %H:%M:%S')</t>
         </is>
@@ -4032,7 +4288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="27.33" customWidth="1" style="13" min="1" max="1"/>
@@ -5315,6 +5571,94 @@
       <c r="C67" s="13" t="inlineStr">
         <is>
           <t>None of the above</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="n"/>
+      <c r="B68" s="13" t="n"/>
+      <c r="C68" s="13" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="13" t="n"/>
+      <c r="B69" s="13" t="n"/>
+      <c r="C69" s="13" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="n"/>
+      <c r="B70" s="13" t="n"/>
+      <c r="C70" s="13" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="n"/>
+      <c r="B71" s="13" t="n"/>
+      <c r="C71" s="13" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>referral_facility</t>
+        </is>
+      </c>
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>hwc</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>Health and Wellness Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>referral_facility</t>
+        </is>
+      </c>
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>phc</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Primary Health Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>referral_facility</t>
+        </is>
+      </c>
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>chc</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>Community Health Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>referral_facility</t>
+        </is>
+      </c>
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>dh</t>
+        </is>
+      </c>
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>District Hospital</t>
         </is>
       </c>
     </row>

</xml_diff>